<commit_message>
Corrigir calculo de area de linhas e metas na Visao Geral
</commit_message>
<xml_diff>
--- a/dados.xlsx
+++ b/dados.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="BASE_PROCESSAMENTOS" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="BACKLOG" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="FALHAS_PLANTIO" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="METAS_GLOBAIS" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BASE_PROCESSAMENTOS" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BACKLOG" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FALHAS_PLANTIO" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="METAS_GLOBAIS" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,9 +19,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -52,9 +51,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -466,7 +466,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>HÁ</t>
+          <t>HA</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
@@ -514,8 +514,7 @@
           <t>B-24 CENTRO RURAL</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" s="1" t="n">
+      <c r="E2" s="2" t="n">
         <v>46205</v>
       </c>
       <c r="F2" t="inlineStr">
@@ -539,11 +538,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -564,7 +558,7 @@
           <t>-22° 02´ 13.3421 -50° 07´ 13.5185 491.84</t>
         </is>
       </c>
-      <c r="E3" s="1" t="n">
+      <c r="E3" s="2" t="n">
         <v>46217</v>
       </c>
       <c r="F3" t="inlineStr">
@@ -604,7 +598,6 @@
       <c r="N3" t="n">
         <v>586.49</v>
       </c>
-      <c r="O3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -620,8 +613,7 @@
           <t>B-23 FAZ NOSSA SENHORA APARECIDA</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" s="1" t="n">
+      <c r="E4" s="2" t="n">
         <v>46199</v>
       </c>
       <c r="F4" t="inlineStr">
@@ -661,7 +653,6 @@
       <c r="N4" t="n">
         <v>854.9300000000001</v>
       </c>
-      <c r="O4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -682,7 +673,7 @@
           <t>-21° 39´ 13.2100 -50° 32´ 04.0182 418.26</t>
         </is>
       </c>
-      <c r="E5" s="1" t="n">
+      <c r="E5" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F5" t="inlineStr">
@@ -711,10 +702,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -735,7 +722,7 @@
           <t>-21° 39´ 13.2100 -50° 32´ 04.0182 418.26</t>
         </is>
       </c>
-      <c r="E6" s="1" t="n">
+      <c r="E6" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F6" t="inlineStr">
@@ -764,10 +751,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -788,7 +771,7 @@
           <t>-21° 34´ 46.1049 -50° 26´ 00.0424 442.78</t>
         </is>
       </c>
-      <c r="E7" s="1" t="n">
+      <c r="E7" s="2" t="n">
         <v>46183</v>
       </c>
       <c r="F7" t="inlineStr">
@@ -817,7 +800,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr">
         <is>
           <t xml:space="preserve">PROPRIAS </t>
@@ -849,7 +831,7 @@
           <t>-22° 02´ 13.3421 -50° 07´ 13.5185 491.84</t>
         </is>
       </c>
-      <c r="E8" s="1" t="n">
+      <c r="E8" s="2" t="n">
         <v>46196</v>
       </c>
       <c r="F8" t="inlineStr">
@@ -878,7 +860,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr">
         <is>
           <t>TERCEIROS</t>
@@ -905,8 +886,7 @@
           <t>B-23 FAZ NOSSA SENHORA APARECIDA</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" s="1" t="n">
+      <c r="E9" s="2" t="n">
         <v>46199</v>
       </c>
       <c r="F9" t="inlineStr">
@@ -935,10 +915,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -959,7 +935,7 @@
           <t>-21° 31´ 28.9807 -50° 18´ 16.5320 492.23</t>
         </is>
       </c>
-      <c r="E10" s="1" t="n">
+      <c r="E10" s="2" t="n">
         <v>46211</v>
       </c>
       <c r="F10" t="inlineStr">
@@ -988,10 +964,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1012,7 +984,7 @@
           <t>-21° 39´ 13.2100 -50° 32´ 04.0182 418.26</t>
         </is>
       </c>
-      <c r="E11" s="1" t="n">
+      <c r="E11" s="2" t="n">
         <v>46189</v>
       </c>
       <c r="F11" t="inlineStr">
@@ -1041,10 +1013,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1060,8 +1028,7 @@
           <t>B-24 CENTRO RURAL</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" s="1" t="n">
+      <c r="E12" s="2" t="n">
         <v>46203</v>
       </c>
       <c r="F12" t="inlineStr">
@@ -1090,10 +1057,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1114,7 +1077,7 @@
           <t>-21° 31´ 28.9807 -50° 18´ 16.5320 492.23</t>
         </is>
       </c>
-      <c r="E13" s="1" t="n">
+      <c r="E13" s="2" t="n">
         <v>46185</v>
       </c>
       <c r="F13" t="inlineStr">
@@ -1143,10 +1106,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1167,7 +1126,7 @@
           <t>-21° 31´ 28.9807 -50° 18´ 16.5320 492.23</t>
         </is>
       </c>
-      <c r="E14" s="1" t="n">
+      <c r="E14" s="2" t="n">
         <v>46211</v>
       </c>
       <c r="F14" t="inlineStr">
@@ -1196,10 +1155,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1210,9 +1165,7 @@
           <t>SÍTIO SÃO FRANCISCO -</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" s="1" t="n">
+      <c r="E15" s="2" t="n">
         <v>46185</v>
       </c>
       <c r="F15" t="inlineStr">
@@ -1241,10 +1194,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
-      <c r="O15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1260,8 +1209,7 @@
           <t>B-24 CENTRO RURAL</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" s="1" t="n">
+      <c r="E16" s="2" t="n">
         <v>46203</v>
       </c>
       <c r="F16" t="inlineStr">
@@ -1290,10 +1238,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr"/>
-      <c r="O16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1314,7 +1258,7 @@
           <t>-21° 31´ 28.9807 -50° 18´ 16.5320 492.23</t>
         </is>
       </c>
-      <c r="E17" s="1" t="n">
+      <c r="E17" s="2" t="n">
         <v>46185</v>
       </c>
       <c r="F17" t="inlineStr">
@@ -1343,10 +1287,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr"/>
-      <c r="O17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1367,7 +1307,7 @@
           <t>-21° 35´ 32.3241 -50° 10´ 09.0062 470.03</t>
         </is>
       </c>
-      <c r="E18" s="1" t="n">
+      <c r="E18" s="2" t="n">
         <v>46219</v>
       </c>
       <c r="F18" t="inlineStr">
@@ -1396,10 +1336,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
-      <c r="N18" t="inlineStr"/>
-      <c r="O18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1420,7 +1356,7 @@
           <t>-21° 31´ 28.9807 -50° 18´ 16.5320 492.23</t>
         </is>
       </c>
-      <c r="E19" s="1" t="n">
+      <c r="E19" s="2" t="n">
         <v>46211</v>
       </c>
       <c r="F19" t="inlineStr">
@@ -1449,10 +1385,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1463,9 +1395,7 @@
           <t>SÍTIO IRMÃOS ANNELLI -</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" s="1" t="n">
+      <c r="E20" s="2" t="n">
         <v>46185</v>
       </c>
       <c r="F20" t="inlineStr">
@@ -1494,10 +1424,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1508,9 +1434,7 @@
           <t>SÍTIO TREZE DE MAIO</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" s="1" t="n">
+      <c r="E21" s="2" t="n">
         <v>46205</v>
       </c>
       <c r="F21" t="inlineStr">
@@ -1518,7 +1442,7 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="G21" s="1" t="n">
+      <c r="G21" s="2" t="n">
         <v>46210</v>
       </c>
       <c r="H21" t="n">
@@ -1537,10 +1461,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
-      <c r="N21" t="inlineStr"/>
-      <c r="O21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1561,7 +1481,7 @@
           <t>-21° 39´ 59.2206 -50° 19´ 50.9494 405.70</t>
         </is>
       </c>
-      <c r="E22" s="1" t="n">
+      <c r="E22" s="2" t="n">
         <v>46216</v>
       </c>
       <c r="F22" t="inlineStr">
@@ -1590,10 +1510,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr"/>
-      <c r="O22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1614,7 +1530,7 @@
           <t>-21° 31´ 28.9807 -50° 18´ 16.5320 492.23</t>
         </is>
       </c>
-      <c r="E23" s="1" t="n">
+      <c r="E23" s="2" t="n">
         <v>46211</v>
       </c>
       <c r="F23" t="inlineStr">
@@ -1643,10 +1559,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr"/>
-      <c r="O23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1667,7 +1579,7 @@
           <t>-21° 35´ 32.3241 -50° 10´ 09.0062 470.03</t>
         </is>
       </c>
-      <c r="E24" s="1" t="n">
+      <c r="E24" s="2" t="n">
         <v>46219</v>
       </c>
       <c r="F24" t="inlineStr">
@@ -1696,10 +1608,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr"/>
-      <c r="O24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1720,7 +1628,7 @@
           <t>-21° 35´ 32.3241 -50° 10´ 09.0062 470.03</t>
         </is>
       </c>
-      <c r="E25" s="1" t="n">
+      <c r="E25" s="2" t="n">
         <v>46219</v>
       </c>
       <c r="F25" t="inlineStr">
@@ -1749,10 +1657,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1773,7 +1677,7 @@
           <t>-21° 48´ 26.1814 -50° 13´ 14.2006 438.00</t>
         </is>
       </c>
-      <c r="E26" s="1" t="n">
+      <c r="E26" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="F26" t="inlineStr">
@@ -1802,10 +1706,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1826,7 +1726,7 @@
           <t>-21° 48´ 26.1814 -50° 13´ 14.2006 438.00</t>
         </is>
       </c>
-      <c r="E27" s="1" t="n">
+      <c r="E27" s="2" t="n">
         <v>46239</v>
       </c>
       <c r="F27" t="inlineStr">
@@ -1855,10 +1755,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
-      <c r="O27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1879,7 +1775,7 @@
           <t>-21° 45´ 32.6517 -50° 06´ 02.9557 456.63</t>
         </is>
       </c>
-      <c r="E28" s="1" t="n">
+      <c r="E28" s="2" t="n">
         <v>46240</v>
       </c>
       <c r="F28" t="inlineStr">
@@ -1895,13 +1791,6 @@
       <c r="H28" t="n">
         <v>94.87</v>
       </c>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
-      <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr"/>
-      <c r="O28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1922,7 +1811,7 @@
           <t>-21° 48´ 26.1814 -50° 13´ 14.2006 438.00</t>
         </is>
       </c>
-      <c r="E29" s="1" t="n">
+      <c r="E29" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="F29" t="inlineStr">
@@ -1951,10 +1840,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L29" t="inlineStr"/>
-      <c r="M29" t="inlineStr"/>
-      <c r="N29" t="inlineStr"/>
-      <c r="O29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1975,7 +1860,7 @@
           <t>-21° 39´ 13.2100 -50° 32´ 04.0182 418.26</t>
         </is>
       </c>
-      <c r="E30" s="1" t="n">
+      <c r="E30" s="2" t="n">
         <v>46237</v>
       </c>
       <c r="F30" t="inlineStr">
@@ -1991,13 +1876,6 @@
       <c r="H30" t="n">
         <v>57.73</v>
       </c>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr"/>
-      <c r="M30" t="inlineStr"/>
-      <c r="N30" t="inlineStr"/>
-      <c r="O30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -2018,7 +1896,7 @@
           <t>-21° 48´ 26.1814 -50° 13´ 14.2006 438.00</t>
         </is>
       </c>
-      <c r="E31" s="1" t="n">
+      <c r="E31" s="2" t="n">
         <v>46240</v>
       </c>
       <c r="F31" t="inlineStr">
@@ -2034,13 +1912,6 @@
       <c r="H31" t="n">
         <v>60.89</v>
       </c>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr"/>
-      <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr"/>
-      <c r="O31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -2061,7 +1932,7 @@
           <t>-21° 39´ 13.2100 -50° 32´ 04.0182 418.26</t>
         </is>
       </c>
-      <c r="E32" s="1" t="n">
+      <c r="E32" s="2" t="n">
         <v>46237</v>
       </c>
       <c r="F32" t="inlineStr">
@@ -2085,11 +1956,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr"/>
-      <c r="M32" t="inlineStr"/>
-      <c r="N32" t="inlineStr"/>
-      <c r="O32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -2110,7 +1976,7 @@
           <t>-22° 02´ 13.3421 -50° 07´ 13.5185 491.84</t>
         </is>
       </c>
-      <c r="E33" s="1" t="n">
+      <c r="E33" s="2" t="n">
         <v>46231</v>
       </c>
       <c r="F33" t="inlineStr">
@@ -2126,13 +1992,6 @@
       <c r="H33" t="n">
         <v>95.5</v>
       </c>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr"/>
-      <c r="M33" t="inlineStr"/>
-      <c r="N33" t="inlineStr"/>
-      <c r="O33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -2153,7 +2012,7 @@
           <t>-21° 31´ 28.9807 -50° 18´ 16.5320 492.23</t>
         </is>
       </c>
-      <c r="E34" s="1" t="n">
+      <c r="E34" s="2" t="n">
         <v>46241</v>
       </c>
       <c r="F34" t="inlineStr">
@@ -2182,10 +2041,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L34" t="inlineStr"/>
-      <c r="M34" t="inlineStr"/>
-      <c r="N34" t="inlineStr"/>
-      <c r="O34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -2206,7 +2061,7 @@
           <t>-21° 31´ 28.9807 -50° 18´ 16.5320 492.23</t>
         </is>
       </c>
-      <c r="E35" s="1" t="n">
+      <c r="E35" s="2" t="n">
         <v>46241</v>
       </c>
       <c r="F35" t="inlineStr">
@@ -2235,10 +2090,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L35" t="inlineStr"/>
-      <c r="M35" t="inlineStr"/>
-      <c r="N35" t="inlineStr"/>
-      <c r="O35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -2259,7 +2110,7 @@
           <t>-21° 35´ 32.3241 -50° 10´ 09.0062 470.03</t>
         </is>
       </c>
-      <c r="E36" s="1" t="n">
+      <c r="E36" s="2" t="n">
         <v>46246</v>
       </c>
       <c r="F36" t="inlineStr">
@@ -2288,10 +2139,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L36" t="inlineStr"/>
-      <c r="M36" t="inlineStr"/>
-      <c r="N36" t="inlineStr"/>
-      <c r="O36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -2312,7 +2159,7 @@
           <t>-21° 29´ 18.1708 -50° 13´ 39.5944 458.12</t>
         </is>
       </c>
-      <c r="E37" s="1" t="n">
+      <c r="E37" s="2" t="n">
         <v>46245</v>
       </c>
       <c r="F37" t="inlineStr">
@@ -2341,10 +2188,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L37" t="inlineStr"/>
-      <c r="M37" t="inlineStr"/>
-      <c r="N37" t="inlineStr"/>
-      <c r="O37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -2355,9 +2198,7 @@
           <t>FAZ LONQUINHO</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr"/>
-      <c r="D38" t="inlineStr"/>
-      <c r="E38" s="1" t="n">
+      <c r="E38" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="F38" t="inlineStr">
@@ -2373,17 +2214,11 @@
       <c r="H38" t="n">
         <v>202.93</v>
       </c>
-      <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr">
         <is>
           <t>FEITO</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
-      <c r="M38" t="inlineStr"/>
-      <c r="N38" t="inlineStr"/>
-      <c r="O38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -2404,7 +2239,7 @@
           <t>-21° 45´ 32.6517 -50° 06´ 02.9557 456.63</t>
         </is>
       </c>
-      <c r="E39" s="1" t="n">
+      <c r="E39" s="2" t="n">
         <v>46248</v>
       </c>
       <c r="F39" t="inlineStr">
@@ -2433,10 +2268,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L39" t="inlineStr"/>
-      <c r="M39" t="inlineStr"/>
-      <c r="N39" t="inlineStr"/>
-      <c r="O39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -2457,7 +2288,7 @@
           <t>-21° 45´ 32.6517 -50° 06´ 02.9557 456.63</t>
         </is>
       </c>
-      <c r="E40" s="1" t="n">
+      <c r="E40" s="2" t="n">
         <v>46248</v>
       </c>
       <c r="F40" t="inlineStr">
@@ -2486,10 +2317,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L40" t="inlineStr"/>
-      <c r="M40" t="inlineStr"/>
-      <c r="N40" t="inlineStr"/>
-      <c r="O40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -2510,7 +2337,7 @@
           <t>-21° 23´ 27.6854 -50° 29´ 11.8918 453.23</t>
         </is>
       </c>
-      <c r="E41" s="1" t="n">
+      <c r="E41" s="2" t="n">
         <v>46254</v>
       </c>
       <c r="F41" t="inlineStr">
@@ -2526,13 +2353,6 @@
       <c r="H41" t="n">
         <v>83.7</v>
       </c>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr"/>
-      <c r="M41" t="inlineStr"/>
-      <c r="N41" t="inlineStr"/>
-      <c r="O41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -2543,9 +2363,7 @@
           <t>SÍTIO SANTO ANTONIO I</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr"/>
-      <c r="D42" t="inlineStr"/>
-      <c r="E42" s="1" t="n">
+      <c r="E42" s="2" t="n">
         <v>46248</v>
       </c>
       <c r="F42" t="inlineStr">
@@ -2569,11 +2387,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr"/>
-      <c r="M42" t="inlineStr"/>
-      <c r="N42" t="inlineStr"/>
-      <c r="O42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -2584,9 +2397,7 @@
           <t>ESTÂNCIA EBENEZER I</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr"/>
-      <c r="D43" t="inlineStr"/>
-      <c r="E43" s="1" t="n">
+      <c r="E43" s="2" t="n">
         <v>46248</v>
       </c>
       <c r="F43" t="inlineStr">
@@ -2602,17 +2413,11 @@
       <c r="H43" t="n">
         <v>13.34</v>
       </c>
-      <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
       <c r="K43" t="inlineStr">
         <is>
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L43" t="inlineStr"/>
-      <c r="M43" t="inlineStr"/>
-      <c r="N43" t="inlineStr"/>
-      <c r="O43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -2633,7 +2438,7 @@
           <t>-21° 23´ 27.6854 -50° 29´ 11.8918 453.23</t>
         </is>
       </c>
-      <c r="E44" s="1" t="n">
+      <c r="E44" s="2" t="n">
         <v>46248</v>
       </c>
       <c r="F44" t="inlineStr">
@@ -2662,10 +2467,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L44" t="inlineStr"/>
-      <c r="M44" t="inlineStr"/>
-      <c r="N44" t="inlineStr"/>
-      <c r="O44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -2686,7 +2487,7 @@
           <t>-21° 35´ 32.3241 -50° 10´ 09.0062 470.03</t>
         </is>
       </c>
-      <c r="E45" s="1" t="n">
+      <c r="E45" s="2" t="n">
         <v>40037</v>
       </c>
       <c r="F45" t="inlineStr">
@@ -2702,17 +2503,11 @@
       <c r="H45" t="n">
         <v>7.28</v>
       </c>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
       <c r="K45" t="inlineStr">
         <is>
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L45" t="inlineStr"/>
-      <c r="M45" t="inlineStr"/>
-      <c r="N45" t="inlineStr"/>
-      <c r="O45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -2723,9 +2518,7 @@
           <t>SITIO SANTA LUZIA</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr"/>
-      <c r="D46" t="inlineStr"/>
-      <c r="E46" s="1" t="n">
+      <c r="E46" s="2" t="n">
         <v>46246</v>
       </c>
       <c r="F46" t="inlineStr">
@@ -2741,13 +2534,6 @@
       <c r="H46" t="n">
         <v>2.84</v>
       </c>
-      <c r="I46" t="inlineStr"/>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr"/>
-      <c r="M46" t="inlineStr"/>
-      <c r="N46" t="inlineStr"/>
-      <c r="O46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -2758,9 +2544,7 @@
           <t>SÍTIO SANTA INÊS</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr"/>
-      <c r="D47" t="inlineStr"/>
-      <c r="E47" s="1" t="n">
+      <c r="E47" s="2" t="n">
         <v>46246</v>
       </c>
       <c r="F47" t="inlineStr">
@@ -2776,13 +2560,6 @@
       <c r="H47" t="n">
         <v>10.97</v>
       </c>
-      <c r="I47" t="inlineStr"/>
-      <c r="J47" t="inlineStr"/>
-      <c r="K47" t="inlineStr"/>
-      <c r="L47" t="inlineStr"/>
-      <c r="M47" t="inlineStr"/>
-      <c r="N47" t="inlineStr"/>
-      <c r="O47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -2793,9 +2570,7 @@
           <t>FAZENDA NOVA ERA</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr"/>
-      <c r="D48" t="inlineStr"/>
-      <c r="E48" s="1" t="n">
+      <c r="E48" s="2" t="n">
         <v>46248</v>
       </c>
       <c r="F48" t="inlineStr">
@@ -2824,10 +2599,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L48" t="inlineStr"/>
-      <c r="M48" t="inlineStr"/>
-      <c r="N48" t="inlineStr"/>
-      <c r="O48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -2848,7 +2619,7 @@
           <t>-21° 45´ 32.6517 -50° 06´ 02.9557 456.63</t>
         </is>
       </c>
-      <c r="E49" s="1" t="n">
+      <c r="E49" s="2" t="n">
         <v>46248</v>
       </c>
       <c r="F49" t="inlineStr">
@@ -2877,10 +2648,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L49" t="inlineStr"/>
-      <c r="M49" t="inlineStr"/>
-      <c r="N49" t="inlineStr"/>
-      <c r="O49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -2891,9 +2658,7 @@
           <t>SÍTIO SANTO ANTÔNIO</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr"/>
-      <c r="D50" t="inlineStr"/>
-      <c r="E50" s="1" t="n">
+      <c r="E50" s="2" t="n">
         <v>46248</v>
       </c>
       <c r="F50" t="inlineStr">
@@ -2922,10 +2687,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L50" t="inlineStr"/>
-      <c r="M50" t="inlineStr"/>
-      <c r="N50" t="inlineStr"/>
-      <c r="O50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -2946,7 +2707,7 @@
           <t>-21° 48´ 26.1814 -50° 13´ 14.2006 438.00</t>
         </is>
       </c>
-      <c r="E51" s="1" t="n">
+      <c r="E51" s="2" t="n">
         <v>46258</v>
       </c>
       <c r="F51" t="inlineStr">
@@ -2975,10 +2736,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L51" t="inlineStr"/>
-      <c r="M51" t="inlineStr"/>
-      <c r="N51" t="inlineStr"/>
-      <c r="O51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -2999,7 +2756,7 @@
           <t>-21° 24´ 42.3464 -50° 12´ 32.2760 396.57</t>
         </is>
       </c>
-      <c r="E52" s="1" t="n">
+      <c r="E52" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="F52" t="inlineStr">
@@ -3028,10 +2785,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L52" t="inlineStr"/>
-      <c r="M52" t="inlineStr"/>
-      <c r="N52" t="inlineStr"/>
-      <c r="O52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -3052,7 +2805,7 @@
           <t>-21° 24´ 42.3464 -50° 12´ 32.2760 396.57</t>
         </is>
       </c>
-      <c r="E53" s="1" t="n">
+      <c r="E53" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="F53" t="inlineStr">
@@ -3081,10 +2834,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L53" t="inlineStr"/>
-      <c r="M53" t="inlineStr"/>
-      <c r="N53" t="inlineStr"/>
-      <c r="O53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -3105,7 +2854,7 @@
           <t>-21° 47´ 12.2305 -50° 35´ 27.8405 436.14</t>
         </is>
       </c>
-      <c r="E54" s="1" t="n">
+      <c r="E54" s="2" t="n">
         <v>46261</v>
       </c>
       <c r="F54" t="inlineStr">
@@ -3113,19 +2862,12 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="G54" s="1" t="n">
+      <c r="G54" s="2" t="n">
         <v>46262</v>
       </c>
       <c r="H54" t="n">
         <v>200.36</v>
       </c>
-      <c r="I54" t="inlineStr"/>
-      <c r="J54" t="inlineStr"/>
-      <c r="K54" t="inlineStr"/>
-      <c r="L54" t="inlineStr"/>
-      <c r="M54" t="inlineStr"/>
-      <c r="N54" t="inlineStr"/>
-      <c r="O54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -3146,7 +2888,7 @@
           <t>-21° 39´ 13.2100 -50° 32´ 04.0182 418.26</t>
         </is>
       </c>
-      <c r="E55" s="1" t="n">
+      <c r="E55" s="2" t="n">
         <v>46261</v>
       </c>
       <c r="F55" t="inlineStr">
@@ -3175,10 +2917,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L55" t="inlineStr"/>
-      <c r="M55" t="inlineStr"/>
-      <c r="N55" t="inlineStr"/>
-      <c r="O55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -3199,7 +2937,7 @@
           <t>-21° 39´ 13.2100 -50° 32´ 04.0182 418.26</t>
         </is>
       </c>
-      <c r="E56" s="1" t="n">
+      <c r="E56" s="2" t="n">
         <v>46261</v>
       </c>
       <c r="F56" t="inlineStr">
@@ -3223,11 +2961,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="K56" t="inlineStr"/>
-      <c r="L56" t="inlineStr"/>
-      <c r="M56" t="inlineStr"/>
-      <c r="N56" t="inlineStr"/>
-      <c r="O56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -3238,9 +2971,7 @@
           <t>ESTÂNCIA BOA SORTE</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr"/>
-      <c r="D57" t="inlineStr"/>
-      <c r="E57" s="1" t="n">
+      <c r="E57" s="2" t="n">
         <v>46248</v>
       </c>
       <c r="F57" t="inlineStr">
@@ -3269,10 +3000,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L57" t="inlineStr"/>
-      <c r="M57" t="inlineStr"/>
-      <c r="N57" t="inlineStr"/>
-      <c r="O57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -3283,9 +3010,7 @@
           <t>SITIO SANTA CLARA I</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr"/>
-      <c r="D58" t="inlineStr"/>
-      <c r="E58" s="1" t="n">
+      <c r="E58" s="2" t="n">
         <v>46246</v>
       </c>
       <c r="F58" t="inlineStr">
@@ -3301,17 +3026,11 @@
       <c r="H58" t="n">
         <v>12.89</v>
       </c>
-      <c r="I58" t="inlineStr"/>
-      <c r="J58" t="inlineStr"/>
       <c r="K58" t="inlineStr">
         <is>
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L58" t="inlineStr"/>
-      <c r="M58" t="inlineStr"/>
-      <c r="N58" t="inlineStr"/>
-      <c r="O58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -3327,7 +3046,6 @@
           <t>B-19 SEDE TIAGO TUNES</t>
         </is>
       </c>
-      <c r="D59" t="inlineStr"/>
       <c r="E59" t="inlineStr">
         <is>
           <t>28/08/2026</t>
@@ -3346,17 +3064,11 @@
       <c r="H59" t="n">
         <v>37.72</v>
       </c>
-      <c r="I59" t="inlineStr"/>
-      <c r="J59" t="inlineStr"/>
       <c r="K59" t="inlineStr">
         <is>
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L59" t="inlineStr"/>
-      <c r="M59" t="inlineStr"/>
-      <c r="N59" t="inlineStr"/>
-      <c r="O59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -3372,7 +3084,6 @@
           <t>B-19 SEDE TIAGO TUNES</t>
         </is>
       </c>
-      <c r="D60" t="inlineStr"/>
       <c r="E60" t="inlineStr">
         <is>
           <t>28/08/2026</t>
@@ -3399,11 +3110,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="K60" t="inlineStr"/>
-      <c r="L60" t="inlineStr"/>
-      <c r="M60" t="inlineStr"/>
-      <c r="N60" t="inlineStr"/>
-      <c r="O60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -3419,7 +3125,6 @@
           <t>B-19 SEDE TIAGO TUNES</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr"/>
       <c r="E61" t="inlineStr">
         <is>
           <t>28/09/2026</t>
@@ -3446,11 +3151,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="K61" t="inlineStr"/>
-      <c r="L61" t="inlineStr"/>
-      <c r="M61" t="inlineStr"/>
-      <c r="N61" t="inlineStr"/>
-      <c r="O61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -3466,7 +3166,6 @@
           <t>B-19 SEDE TIAGO TUNES</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr"/>
       <c r="E62" t="inlineStr">
         <is>
           <t>28/08/2026</t>
@@ -3498,10 +3197,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L62" t="inlineStr"/>
-      <c r="M62" t="inlineStr"/>
-      <c r="N62" t="inlineStr"/>
-      <c r="O62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -3512,8 +3207,6 @@
           <t>SITIO SÃO JOSE</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr"/>
-      <c r="D63" t="inlineStr"/>
       <c r="E63" t="inlineStr">
         <is>
           <t>28/09/2026</t>
@@ -3540,11 +3233,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="K63" t="inlineStr"/>
-      <c r="L63" t="inlineStr"/>
-      <c r="M63" t="inlineStr"/>
-      <c r="N63" t="inlineStr"/>
-      <c r="O63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -3580,14 +3268,6 @@
           <t>09/09/2026</t>
         </is>
       </c>
-      <c r="H64" t="inlineStr"/>
-      <c r="I64" t="inlineStr"/>
-      <c r="J64" t="inlineStr"/>
-      <c r="K64" t="inlineStr"/>
-      <c r="L64" t="inlineStr"/>
-      <c r="M64" t="inlineStr"/>
-      <c r="N64" t="inlineStr"/>
-      <c r="O64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -3639,10 +3319,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L65" t="inlineStr"/>
-      <c r="M65" t="inlineStr"/>
-      <c r="N65" t="inlineStr"/>
-      <c r="O65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -3681,17 +3357,11 @@
       <c r="H66" t="n">
         <v>99.37</v>
       </c>
-      <c r="I66" t="inlineStr"/>
-      <c r="J66" t="inlineStr"/>
       <c r="K66" t="inlineStr">
         <is>
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L66" t="inlineStr"/>
-      <c r="M66" t="inlineStr"/>
-      <c r="N66" t="inlineStr"/>
-      <c r="O66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -3740,11 +3410,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="K67" t="inlineStr"/>
-      <c r="L67" t="inlineStr"/>
-      <c r="M67" t="inlineStr"/>
-      <c r="N67" t="inlineStr"/>
-      <c r="O67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -3793,11 +3458,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="K68" t="inlineStr"/>
-      <c r="L68" t="inlineStr"/>
-      <c r="M68" t="inlineStr"/>
-      <c r="N68" t="inlineStr"/>
-      <c r="O68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -3849,10 +3509,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L69" t="inlineStr"/>
-      <c r="M69" t="inlineStr"/>
-      <c r="N69" t="inlineStr"/>
-      <c r="O69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -3904,10 +3560,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L70" t="inlineStr"/>
-      <c r="M70" t="inlineStr"/>
-      <c r="N70" t="inlineStr"/>
-      <c r="O70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -3918,8 +3570,6 @@
           <t>SÍTIO LIMEIRA</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr"/>
-      <c r="D71" t="inlineStr"/>
       <c r="E71" t="inlineStr">
         <is>
           <t>04/09/2026</t>
@@ -3938,13 +3588,6 @@
       <c r="H71" t="n">
         <v>59.32</v>
       </c>
-      <c r="I71" t="inlineStr"/>
-      <c r="J71" t="inlineStr"/>
-      <c r="K71" t="inlineStr"/>
-      <c r="L71" t="inlineStr"/>
-      <c r="M71" t="inlineStr"/>
-      <c r="N71" t="inlineStr"/>
-      <c r="O71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -3983,13 +3626,6 @@
       <c r="H72" t="n">
         <v>669.6</v>
       </c>
-      <c r="I72" t="inlineStr"/>
-      <c r="J72" t="inlineStr"/>
-      <c r="K72" t="inlineStr"/>
-      <c r="L72" t="inlineStr"/>
-      <c r="M72" t="inlineStr"/>
-      <c r="N72" t="inlineStr"/>
-      <c r="O72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -4028,13 +3664,6 @@
       <c r="H73" t="n">
         <v>42.13</v>
       </c>
-      <c r="I73" t="inlineStr"/>
-      <c r="J73" t="inlineStr"/>
-      <c r="K73" t="inlineStr"/>
-      <c r="L73" t="inlineStr"/>
-      <c r="M73" t="inlineStr"/>
-      <c r="N73" t="inlineStr"/>
-      <c r="O73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -4050,7 +3679,6 @@
           <t>B-23 FAZ NOSSA SENHORA APARECIDA</t>
         </is>
       </c>
-      <c r="D74" t="inlineStr"/>
       <c r="E74" t="inlineStr">
         <is>
           <t>10/09/2026</t>
@@ -4082,10 +3710,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L74" t="inlineStr"/>
-      <c r="M74" t="inlineStr"/>
-      <c r="N74" t="inlineStr"/>
-      <c r="O74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -4101,7 +3725,6 @@
           <t>B-24 CENTRO RURAL</t>
         </is>
       </c>
-      <c r="D75" t="inlineStr"/>
       <c r="E75" t="inlineStr">
         <is>
           <t>11/09/2026</t>
@@ -4128,11 +3751,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="K75" t="inlineStr"/>
-      <c r="L75" t="inlineStr"/>
-      <c r="M75" t="inlineStr"/>
-      <c r="N75" t="inlineStr"/>
-      <c r="O75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -4148,7 +3766,6 @@
           <t>B-24 CENTRO RURAL</t>
         </is>
       </c>
-      <c r="D76" t="inlineStr"/>
       <c r="E76" t="inlineStr">
         <is>
           <t>11/09/2026</t>
@@ -4180,10 +3797,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L76" t="inlineStr"/>
-      <c r="M76" t="inlineStr"/>
-      <c r="N76" t="inlineStr"/>
-      <c r="O76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -4199,7 +3812,6 @@
           <t>B-24 CENTRO RURAL</t>
         </is>
       </c>
-      <c r="D77" t="inlineStr"/>
       <c r="E77" t="inlineStr">
         <is>
           <t>11/09/2026</t>
@@ -4215,14 +3827,6 @@
           <t>15/09/2026</t>
         </is>
       </c>
-      <c r="H77" t="inlineStr"/>
-      <c r="I77" t="inlineStr"/>
-      <c r="J77" t="inlineStr"/>
-      <c r="K77" t="inlineStr"/>
-      <c r="L77" t="inlineStr"/>
-      <c r="M77" t="inlineStr"/>
-      <c r="N77" t="inlineStr"/>
-      <c r="O77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -4238,7 +3842,6 @@
           <t>B-24 CENTRO RURAL</t>
         </is>
       </c>
-      <c r="D78" t="inlineStr"/>
       <c r="E78" t="inlineStr">
         <is>
           <t>11/09/2026</t>
@@ -4265,11 +3868,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="K78" t="inlineStr"/>
-      <c r="L78" t="inlineStr"/>
-      <c r="M78" t="inlineStr"/>
-      <c r="N78" t="inlineStr"/>
-      <c r="O78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -4285,7 +3883,6 @@
           <t>B-24 CENTRO RURAL</t>
         </is>
       </c>
-      <c r="D79" t="inlineStr"/>
       <c r="E79" t="inlineStr">
         <is>
           <t>11/09/2026</t>
@@ -4312,11 +3909,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="K79" t="inlineStr"/>
-      <c r="L79" t="inlineStr"/>
-      <c r="M79" t="inlineStr"/>
-      <c r="N79" t="inlineStr"/>
-      <c r="O79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -4368,10 +3960,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L80" t="inlineStr"/>
-      <c r="M80" t="inlineStr"/>
-      <c r="N80" t="inlineStr"/>
-      <c r="O80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -4410,17 +3998,11 @@
       <c r="H81" t="n">
         <v>84.09</v>
       </c>
-      <c r="I81" t="inlineStr"/>
-      <c r="J81" t="inlineStr"/>
       <c r="K81" t="inlineStr">
         <is>
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L81" t="inlineStr"/>
-      <c r="M81" t="inlineStr"/>
-      <c r="N81" t="inlineStr"/>
-      <c r="O81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -4436,7 +4018,6 @@
           <t>B-24 CENTRO RURAL</t>
         </is>
       </c>
-      <c r="D82" t="inlineStr"/>
       <c r="E82" t="inlineStr">
         <is>
           <t>11/09/2026</t>
@@ -4463,11 +4044,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="K82" t="inlineStr"/>
-      <c r="L82" t="inlineStr"/>
-      <c r="M82" t="inlineStr"/>
-      <c r="N82" t="inlineStr"/>
-      <c r="O82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -4503,14 +4079,6 @@
           <t>17/09/2026</t>
         </is>
       </c>
-      <c r="H83" t="inlineStr"/>
-      <c r="I83" t="inlineStr"/>
-      <c r="J83" t="inlineStr"/>
-      <c r="K83" t="inlineStr"/>
-      <c r="L83" t="inlineStr"/>
-      <c r="M83" t="inlineStr"/>
-      <c r="N83" t="inlineStr"/>
-      <c r="O83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -4562,10 +4130,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L84" t="inlineStr"/>
-      <c r="M84" t="inlineStr"/>
-      <c r="N84" t="inlineStr"/>
-      <c r="O84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -4612,11 +4176,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="K85" t="inlineStr"/>
-      <c r="L85" t="inlineStr"/>
-      <c r="M85" t="inlineStr"/>
-      <c r="N85" t="inlineStr"/>
-      <c r="O85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -4668,10 +4227,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L86" t="inlineStr"/>
-      <c r="M86" t="inlineStr"/>
-      <c r="N86" t="inlineStr"/>
-      <c r="O86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -4723,10 +4278,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L87" t="inlineStr"/>
-      <c r="M87" t="inlineStr"/>
-      <c r="N87" t="inlineStr"/>
-      <c r="O87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -4778,10 +4329,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L88" t="inlineStr"/>
-      <c r="M88" t="inlineStr"/>
-      <c r="N88" t="inlineStr"/>
-      <c r="O88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -4797,7 +4344,6 @@
           <t>B-09 FAZ SANTA ROSA AURELIO</t>
         </is>
       </c>
-      <c r="D89" t="inlineStr"/>
       <c r="E89" t="inlineStr">
         <is>
           <t>18/09/2026</t>
@@ -4816,17 +4362,11 @@
       <c r="H89" t="n">
         <v>552.0599999999999</v>
       </c>
-      <c r="I89" t="inlineStr"/>
-      <c r="J89" t="inlineStr"/>
       <c r="K89" t="inlineStr">
         <is>
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L89" t="inlineStr"/>
-      <c r="M89" t="inlineStr"/>
-      <c r="N89" t="inlineStr"/>
-      <c r="O89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -4842,7 +4382,6 @@
           <t>B-24 CENTRO RURAL</t>
         </is>
       </c>
-      <c r="D90" t="inlineStr"/>
       <c r="E90" t="inlineStr">
         <is>
           <t>11/09/2026</t>
@@ -4853,7 +4392,7 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="G90" s="1" t="n">
+      <c r="G90" s="2" t="n">
         <v>46286</v>
       </c>
       <c r="H90" t="n">
@@ -4867,11 +4406,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="K90" t="inlineStr"/>
-      <c r="L90" t="inlineStr"/>
-      <c r="M90" t="inlineStr"/>
-      <c r="N90" t="inlineStr"/>
-      <c r="O90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -4902,7 +4436,7 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="G91" s="1" t="n">
+      <c r="G91" s="2" t="n">
         <v>46286</v>
       </c>
       <c r="H91" t="n">
@@ -4921,10 +4455,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L91" t="inlineStr"/>
-      <c r="M91" t="inlineStr"/>
-      <c r="N91" t="inlineStr"/>
-      <c r="O91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -4955,7 +4485,7 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="G92" s="1" t="n">
+      <c r="G92" s="2" t="n">
         <v>46286</v>
       </c>
       <c r="H92" t="n">
@@ -4974,10 +4504,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L92" t="inlineStr"/>
-      <c r="M92" t="inlineStr"/>
-      <c r="N92" t="inlineStr"/>
-      <c r="O92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -4993,7 +4519,6 @@
           <t>B-23 FAZ NOSSA SENHORA APARECIDA</t>
         </is>
       </c>
-      <c r="D93" t="inlineStr"/>
       <c r="E93" t="inlineStr">
         <is>
           <t>21/09/2026</t>
@@ -5025,10 +4550,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L93" t="inlineStr"/>
-      <c r="M93" t="inlineStr"/>
-      <c r="N93" t="inlineStr"/>
-      <c r="O93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -5080,10 +4601,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L94" t="inlineStr"/>
-      <c r="M94" t="inlineStr"/>
-      <c r="N94" t="inlineStr"/>
-      <c r="O94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -5099,7 +4616,6 @@
           <t>B-23 FAZ NOSSA SENHORA APARECIDA</t>
         </is>
       </c>
-      <c r="D95" t="inlineStr"/>
       <c r="E95" t="inlineStr">
         <is>
           <t>21/09/2026</t>
@@ -5115,7 +4631,6 @@
           <t>24/07/2026</t>
         </is>
       </c>
-      <c r="H95" t="inlineStr"/>
       <c r="I95" t="n">
         <v>82.73999999999999</v>
       </c>
@@ -5124,11 +4639,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="K95" t="inlineStr"/>
-      <c r="L95" t="inlineStr"/>
-      <c r="M95" t="inlineStr"/>
-      <c r="N95" t="inlineStr"/>
-      <c r="O95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -5144,7 +4654,6 @@
           <t>B-016 FAZ RODA VIVA</t>
         </is>
       </c>
-      <c r="D96" t="inlineStr"/>
       <c r="E96" t="inlineStr">
         <is>
           <t>24/09/2026</t>
@@ -5163,17 +4672,11 @@
       <c r="H96" t="n">
         <v>345.05</v>
       </c>
-      <c r="I96" t="inlineStr"/>
-      <c r="J96" t="inlineStr"/>
       <c r="K96" t="inlineStr">
         <is>
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L96" t="inlineStr"/>
-      <c r="M96" t="inlineStr"/>
-      <c r="N96" t="inlineStr"/>
-      <c r="O96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -5220,11 +4723,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="K97" t="inlineStr"/>
-      <c r="L97" t="inlineStr"/>
-      <c r="M97" t="inlineStr"/>
-      <c r="N97" t="inlineStr"/>
-      <c r="O97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -5271,11 +4769,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="K98" t="inlineStr"/>
-      <c r="L98" t="inlineStr"/>
-      <c r="M98" t="inlineStr"/>
-      <c r="N98" t="inlineStr"/>
-      <c r="O98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -5322,11 +4815,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="K99" t="inlineStr"/>
-      <c r="L99" t="inlineStr"/>
-      <c r="M99" t="inlineStr"/>
-      <c r="N99" t="inlineStr"/>
-      <c r="O99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -5373,11 +4861,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="K100" t="inlineStr"/>
-      <c r="L100" t="inlineStr"/>
-      <c r="M100" t="inlineStr"/>
-      <c r="N100" t="inlineStr"/>
-      <c r="O100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -5393,7 +4876,6 @@
           <t>B-04 HARAS BILAC</t>
         </is>
       </c>
-      <c r="D101" t="inlineStr"/>
       <c r="E101" t="inlineStr">
         <is>
           <t>23/09/2026</t>
@@ -5425,10 +4907,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L101" t="inlineStr"/>
-      <c r="M101" t="inlineStr"/>
-      <c r="N101" t="inlineStr"/>
-      <c r="O101" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -20292,7 +19770,6 @@
       <c r="E391" t="n">
         <v>18.47</v>
       </c>
-      <c r="F391" t="inlineStr"/>
       <c r="G391" t="n">
         <v>0</v>
       </c>
@@ -20326,7 +19803,6 @@
       <c r="E392" t="n">
         <v>10.7</v>
       </c>
-      <c r="F392" t="inlineStr"/>
       <c r="G392" t="n">
         <v>0</v>
       </c>
@@ -20360,7 +19836,6 @@
       <c r="E393" t="n">
         <v>3.89</v>
       </c>
-      <c r="F393" t="inlineStr"/>
       <c r="G393" t="n">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Atualizacao de dados: Wed 10/21/2026 16:51:07.54
</commit_message>
<xml_diff>
--- a/dados.xlsx
+++ b/dados.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BASE_PROCESSAMENTOS" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BACKLOG" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FALHAS_PLANTIO" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="METAS_GLOBAIS" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="BASE_PROCESSAMENTOS" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="BACKLOG" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="FALHAS_PLANTIO" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="METAS_GLOBAIS" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,8 +19,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -51,10 +52,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -466,7 +466,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>HA</t>
+          <t>HÁ</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
@@ -514,7 +514,8 @@
           <t>B-24 CENTRO RURAL</t>
         </is>
       </c>
-      <c r="E2" s="2" t="n">
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" s="1" t="n">
         <v>46205</v>
       </c>
       <c r="F2" t="inlineStr">
@@ -538,6 +539,11 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -558,7 +564,7 @@
           <t>-22° 02´ 13.3421 -50° 07´ 13.5185 491.84</t>
         </is>
       </c>
-      <c r="E3" s="2" t="n">
+      <c r="E3" s="1" t="n">
         <v>46217</v>
       </c>
       <c r="F3" t="inlineStr">
@@ -598,6 +604,7 @@
       <c r="N3" t="n">
         <v>586.49</v>
       </c>
+      <c r="O3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -613,7 +620,8 @@
           <t>B-23 FAZ NOSSA SENHORA APARECIDA</t>
         </is>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="F4" t="inlineStr">
@@ -653,6 +661,7 @@
       <c r="N4" t="n">
         <v>854.9300000000001</v>
       </c>
+      <c r="O4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -673,7 +682,7 @@
           <t>-21° 39´ 13.2100 -50° 32´ 04.0182 418.26</t>
         </is>
       </c>
-      <c r="E5" s="2" t="n">
+      <c r="E5" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F5" t="inlineStr">
@@ -702,6 +711,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -722,7 +735,7 @@
           <t>-21° 39´ 13.2100 -50° 32´ 04.0182 418.26</t>
         </is>
       </c>
-      <c r="E6" s="2" t="n">
+      <c r="E6" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F6" t="inlineStr">
@@ -751,6 +764,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -771,7 +788,7 @@
           <t>-21° 34´ 46.1049 -50° 26´ 00.0424 442.78</t>
         </is>
       </c>
-      <c r="E7" s="2" t="n">
+      <c r="E7" s="1" t="n">
         <v>46183</v>
       </c>
       <c r="F7" t="inlineStr">
@@ -800,6 +817,7 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr">
         <is>
           <t xml:space="preserve">PROPRIAS </t>
@@ -831,7 +849,7 @@
           <t>-22° 02´ 13.3421 -50° 07´ 13.5185 491.84</t>
         </is>
       </c>
-      <c r="E8" s="2" t="n">
+      <c r="E8" s="1" t="n">
         <v>46196</v>
       </c>
       <c r="F8" t="inlineStr">
@@ -860,16 +878,17 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr">
         <is>
           <t>TERCEIROS</t>
         </is>
       </c>
       <c r="N8" t="n">
-        <v>10486.27</v>
+        <v>10425.63</v>
       </c>
       <c r="O8" t="n">
-        <v>2424.77</v>
+        <v>2485.41</v>
       </c>
     </row>
     <row r="9">
@@ -886,7 +905,8 @@
           <t>B-23 FAZ NOSSA SENHORA APARECIDA</t>
         </is>
       </c>
-      <c r="E9" s="2" t="n">
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="F9" t="inlineStr">
@@ -915,6 +935,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -935,7 +959,7 @@
           <t>-21° 31´ 28.9807 -50° 18´ 16.5320 492.23</t>
         </is>
       </c>
-      <c r="E10" s="2" t="n">
+      <c r="E10" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="F10" t="inlineStr">
@@ -964,6 +988,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -984,7 +1012,7 @@
           <t>-21° 39´ 13.2100 -50° 32´ 04.0182 418.26</t>
         </is>
       </c>
-      <c r="E11" s="2" t="n">
+      <c r="E11" s="1" t="n">
         <v>46189</v>
       </c>
       <c r="F11" t="inlineStr">
@@ -1013,6 +1041,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1028,7 +1060,8 @@
           <t>B-24 CENTRO RURAL</t>
         </is>
       </c>
-      <c r="E12" s="2" t="n">
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" s="1" t="n">
         <v>46203</v>
       </c>
       <c r="F12" t="inlineStr">
@@ -1057,6 +1090,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1077,7 +1114,7 @@
           <t>-21° 31´ 28.9807 -50° 18´ 16.5320 492.23</t>
         </is>
       </c>
-      <c r="E13" s="2" t="n">
+      <c r="E13" s="1" t="n">
         <v>46185</v>
       </c>
       <c r="F13" t="inlineStr">
@@ -1106,6 +1143,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1126,7 +1167,7 @@
           <t>-21° 31´ 28.9807 -50° 18´ 16.5320 492.23</t>
         </is>
       </c>
-      <c r="E14" s="2" t="n">
+      <c r="E14" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="F14" t="inlineStr">
@@ -1155,6 +1196,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1165,7 +1210,9 @@
           <t>SÍTIO SÃO FRANCISCO -</t>
         </is>
       </c>
-      <c r="E15" s="2" t="n">
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" s="1" t="n">
         <v>46185</v>
       </c>
       <c r="F15" t="inlineStr">
@@ -1194,6 +1241,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1209,7 +1260,8 @@
           <t>B-24 CENTRO RURAL</t>
         </is>
       </c>
-      <c r="E16" s="2" t="n">
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" s="1" t="n">
         <v>46203</v>
       </c>
       <c r="F16" t="inlineStr">
@@ -1238,6 +1290,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1258,7 +1314,7 @@
           <t>-21° 31´ 28.9807 -50° 18´ 16.5320 492.23</t>
         </is>
       </c>
-      <c r="E17" s="2" t="n">
+      <c r="E17" s="1" t="n">
         <v>46185</v>
       </c>
       <c r="F17" t="inlineStr">
@@ -1287,6 +1343,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1307,7 +1367,7 @@
           <t>-21° 35´ 32.3241 -50° 10´ 09.0062 470.03</t>
         </is>
       </c>
-      <c r="E18" s="2" t="n">
+      <c r="E18" s="1" t="n">
         <v>46219</v>
       </c>
       <c r="F18" t="inlineStr">
@@ -1336,6 +1396,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1356,7 +1420,7 @@
           <t>-21° 31´ 28.9807 -50° 18´ 16.5320 492.23</t>
         </is>
       </c>
-      <c r="E19" s="2" t="n">
+      <c r="E19" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="F19" t="inlineStr">
@@ -1385,6 +1449,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1395,7 +1463,9 @@
           <t>SÍTIO IRMÃOS ANNELLI -</t>
         </is>
       </c>
-      <c r="E20" s="2" t="n">
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" s="1" t="n">
         <v>46185</v>
       </c>
       <c r="F20" t="inlineStr">
@@ -1424,6 +1494,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1434,7 +1508,9 @@
           <t>SÍTIO TREZE DE MAIO</t>
         </is>
       </c>
-      <c r="E21" s="2" t="n">
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" s="1" t="n">
         <v>46205</v>
       </c>
       <c r="F21" t="inlineStr">
@@ -1442,7 +1518,7 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="G21" s="2" t="n">
+      <c r="G21" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="H21" t="n">
@@ -1461,6 +1537,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1481,7 +1561,7 @@
           <t>-21° 39´ 59.2206 -50° 19´ 50.9494 405.70</t>
         </is>
       </c>
-      <c r="E22" s="2" t="n">
+      <c r="E22" s="1" t="n">
         <v>46216</v>
       </c>
       <c r="F22" t="inlineStr">
@@ -1510,6 +1590,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1530,7 +1614,7 @@
           <t>-21° 31´ 28.9807 -50° 18´ 16.5320 492.23</t>
         </is>
       </c>
-      <c r="E23" s="2" t="n">
+      <c r="E23" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="F23" t="inlineStr">
@@ -1559,6 +1643,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1579,7 +1667,7 @@
           <t>-21° 35´ 32.3241 -50° 10´ 09.0062 470.03</t>
         </is>
       </c>
-      <c r="E24" s="2" t="n">
+      <c r="E24" s="1" t="n">
         <v>46219</v>
       </c>
       <c r="F24" t="inlineStr">
@@ -1608,6 +1696,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1628,7 +1720,7 @@
           <t>-21° 35´ 32.3241 -50° 10´ 09.0062 470.03</t>
         </is>
       </c>
-      <c r="E25" s="2" t="n">
+      <c r="E25" s="1" t="n">
         <v>46219</v>
       </c>
       <c r="F25" t="inlineStr">
@@ -1657,6 +1749,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1677,7 +1773,7 @@
           <t>-21° 48´ 26.1814 -50° 13´ 14.2006 438.00</t>
         </is>
       </c>
-      <c r="E26" s="2" t="n">
+      <c r="E26" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="F26" t="inlineStr">
@@ -1706,6 +1802,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1726,7 +1826,7 @@
           <t>-21° 48´ 26.1814 -50° 13´ 14.2006 438.00</t>
         </is>
       </c>
-      <c r="E27" s="2" t="n">
+      <c r="E27" s="1" t="n">
         <v>46239</v>
       </c>
       <c r="F27" t="inlineStr">
@@ -1755,6 +1855,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1775,7 +1879,7 @@
           <t>-21° 45´ 32.6517 -50° 06´ 02.9557 456.63</t>
         </is>
       </c>
-      <c r="E28" s="2" t="n">
+      <c r="E28" s="1" t="n">
         <v>46240</v>
       </c>
       <c r="F28" t="inlineStr">
@@ -1791,6 +1895,13 @@
       <c r="H28" t="n">
         <v>94.87</v>
       </c>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1811,7 +1922,7 @@
           <t>-21° 48´ 26.1814 -50° 13´ 14.2006 438.00</t>
         </is>
       </c>
-      <c r="E29" s="2" t="n">
+      <c r="E29" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="F29" t="inlineStr">
@@ -1840,6 +1951,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr"/>
+      <c r="N29" t="inlineStr"/>
+      <c r="O29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1860,7 +1975,7 @@
           <t>-21° 39´ 13.2100 -50° 32´ 04.0182 418.26</t>
         </is>
       </c>
-      <c r="E30" s="2" t="n">
+      <c r="E30" s="1" t="n">
         <v>46237</v>
       </c>
       <c r="F30" t="inlineStr">
@@ -1876,6 +1991,13 @@
       <c r="H30" t="n">
         <v>57.73</v>
       </c>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" t="inlineStr"/>
+      <c r="O30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1896,7 +2018,7 @@
           <t>-21° 48´ 26.1814 -50° 13´ 14.2006 438.00</t>
         </is>
       </c>
-      <c r="E31" s="2" t="n">
+      <c r="E31" s="1" t="n">
         <v>46240</v>
       </c>
       <c r="F31" t="inlineStr">
@@ -1912,6 +2034,21 @@
       <c r="H31" t="n">
         <v>60.89</v>
       </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>60,64</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>FEITO</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr"/>
+      <c r="N31" t="inlineStr"/>
+      <c r="O31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1932,7 +2069,7 @@
           <t>-21° 39´ 13.2100 -50° 32´ 04.0182 418.26</t>
         </is>
       </c>
-      <c r="E32" s="2" t="n">
+      <c r="E32" s="1" t="n">
         <v>46237</v>
       </c>
       <c r="F32" t="inlineStr">
@@ -1956,6 +2093,11 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr"/>
+      <c r="N32" t="inlineStr"/>
+      <c r="O32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1976,7 +2118,7 @@
           <t>-22° 02´ 13.3421 -50° 07´ 13.5185 491.84</t>
         </is>
       </c>
-      <c r="E33" s="2" t="n">
+      <c r="E33" s="1" t="n">
         <v>46231</v>
       </c>
       <c r="F33" t="inlineStr">
@@ -1992,6 +2134,13 @@
       <c r="H33" t="n">
         <v>95.5</v>
       </c>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr"/>
+      <c r="N33" t="inlineStr"/>
+      <c r="O33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -2012,7 +2161,7 @@
           <t>-21° 31´ 28.9807 -50° 18´ 16.5320 492.23</t>
         </is>
       </c>
-      <c r="E34" s="2" t="n">
+      <c r="E34" s="1" t="n">
         <v>46241</v>
       </c>
       <c r="F34" t="inlineStr">
@@ -2041,6 +2190,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr"/>
+      <c r="N34" t="inlineStr"/>
+      <c r="O34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -2061,7 +2214,7 @@
           <t>-21° 31´ 28.9807 -50° 18´ 16.5320 492.23</t>
         </is>
       </c>
-      <c r="E35" s="2" t="n">
+      <c r="E35" s="1" t="n">
         <v>46241</v>
       </c>
       <c r="F35" t="inlineStr">
@@ -2090,6 +2243,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="inlineStr"/>
+      <c r="N35" t="inlineStr"/>
+      <c r="O35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -2110,7 +2267,7 @@
           <t>-21° 35´ 32.3241 -50° 10´ 09.0062 470.03</t>
         </is>
       </c>
-      <c r="E36" s="2" t="n">
+      <c r="E36" s="1" t="n">
         <v>46246</v>
       </c>
       <c r="F36" t="inlineStr">
@@ -2139,6 +2296,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="inlineStr"/>
+      <c r="N36" t="inlineStr"/>
+      <c r="O36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -2159,7 +2320,7 @@
           <t>-21° 29´ 18.1708 -50° 13´ 39.5944 458.12</t>
         </is>
       </c>
-      <c r="E37" s="2" t="n">
+      <c r="E37" s="1" t="n">
         <v>46245</v>
       </c>
       <c r="F37" t="inlineStr">
@@ -2188,6 +2349,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr"/>
+      <c r="N37" t="inlineStr"/>
+      <c r="O37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -2198,7 +2363,9 @@
           <t>FAZ LONQUINHO</t>
         </is>
       </c>
-      <c r="E38" s="2" t="n">
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" s="1" t="n">
         <v>46247</v>
       </c>
       <c r="F38" t="inlineStr">
@@ -2214,11 +2381,17 @@
       <c r="H38" t="n">
         <v>202.93</v>
       </c>
+      <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr">
         <is>
           <t>FEITO</t>
         </is>
       </c>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr"/>
+      <c r="N38" t="inlineStr"/>
+      <c r="O38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -2239,7 +2412,7 @@
           <t>-21° 45´ 32.6517 -50° 06´ 02.9557 456.63</t>
         </is>
       </c>
-      <c r="E39" s="2" t="n">
+      <c r="E39" s="1" t="n">
         <v>46248</v>
       </c>
       <c r="F39" t="inlineStr">
@@ -2268,6 +2441,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr"/>
+      <c r="N39" t="inlineStr"/>
+      <c r="O39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -2288,7 +2465,7 @@
           <t>-21° 45´ 32.6517 -50° 06´ 02.9557 456.63</t>
         </is>
       </c>
-      <c r="E40" s="2" t="n">
+      <c r="E40" s="1" t="n">
         <v>46248</v>
       </c>
       <c r="F40" t="inlineStr">
@@ -2317,6 +2494,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr"/>
+      <c r="N40" t="inlineStr"/>
+      <c r="O40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -2337,7 +2518,7 @@
           <t>-21° 23´ 27.6854 -50° 29´ 11.8918 453.23</t>
         </is>
       </c>
-      <c r="E41" s="2" t="n">
+      <c r="E41" s="1" t="n">
         <v>46254</v>
       </c>
       <c r="F41" t="inlineStr">
@@ -2353,6 +2534,13 @@
       <c r="H41" t="n">
         <v>83.7</v>
       </c>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr"/>
+      <c r="N41" t="inlineStr"/>
+      <c r="O41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -2363,7 +2551,9 @@
           <t>SÍTIO SANTO ANTONIO I</t>
         </is>
       </c>
-      <c r="E42" s="2" t="n">
+      <c r="C42" t="inlineStr"/>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" s="1" t="n">
         <v>46248</v>
       </c>
       <c r="F42" t="inlineStr">
@@ -2387,6 +2577,11 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr"/>
+      <c r="N42" t="inlineStr"/>
+      <c r="O42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -2397,7 +2592,9 @@
           <t>ESTÂNCIA EBENEZER I</t>
         </is>
       </c>
-      <c r="E43" s="2" t="n">
+      <c r="C43" t="inlineStr"/>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" s="1" t="n">
         <v>46248</v>
       </c>
       <c r="F43" t="inlineStr">
@@ -2413,11 +2610,17 @@
       <c r="H43" t="n">
         <v>13.34</v>
       </c>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr"/>
       <c r="K43" t="inlineStr">
         <is>
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr"/>
+      <c r="N43" t="inlineStr"/>
+      <c r="O43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -2438,7 +2641,7 @@
           <t>-21° 23´ 27.6854 -50° 29´ 11.8918 453.23</t>
         </is>
       </c>
-      <c r="E44" s="2" t="n">
+      <c r="E44" s="1" t="n">
         <v>46248</v>
       </c>
       <c r="F44" t="inlineStr">
@@ -2467,6 +2670,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr"/>
+      <c r="N44" t="inlineStr"/>
+      <c r="O44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -2487,7 +2694,7 @@
           <t>-21° 35´ 32.3241 -50° 10´ 09.0062 470.03</t>
         </is>
       </c>
-      <c r="E45" s="2" t="n">
+      <c r="E45" s="1" t="n">
         <v>40037</v>
       </c>
       <c r="F45" t="inlineStr">
@@ -2503,11 +2710,17 @@
       <c r="H45" t="n">
         <v>7.28</v>
       </c>
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="inlineStr"/>
       <c r="K45" t="inlineStr">
         <is>
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L45" t="inlineStr"/>
+      <c r="M45" t="inlineStr"/>
+      <c r="N45" t="inlineStr"/>
+      <c r="O45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -2518,7 +2731,9 @@
           <t>SITIO SANTA LUZIA</t>
         </is>
       </c>
-      <c r="E46" s="2" t="n">
+      <c r="C46" t="inlineStr"/>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" s="1" t="n">
         <v>46246</v>
       </c>
       <c r="F46" t="inlineStr">
@@ -2534,6 +2749,13 @@
       <c r="H46" t="n">
         <v>2.84</v>
       </c>
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr"/>
+      <c r="N46" t="inlineStr"/>
+      <c r="O46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -2544,7 +2766,9 @@
           <t>SÍTIO SANTA INÊS</t>
         </is>
       </c>
-      <c r="E47" s="2" t="n">
+      <c r="C47" t="inlineStr"/>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" s="1" t="n">
         <v>46246</v>
       </c>
       <c r="F47" t="inlineStr">
@@ -2560,6 +2784,13 @@
       <c r="H47" t="n">
         <v>10.97</v>
       </c>
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr"/>
+      <c r="N47" t="inlineStr"/>
+      <c r="O47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -2570,7 +2801,9 @@
           <t>FAZENDA NOVA ERA</t>
         </is>
       </c>
-      <c r="E48" s="2" t="n">
+      <c r="C48" t="inlineStr"/>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" s="1" t="n">
         <v>46248</v>
       </c>
       <c r="F48" t="inlineStr">
@@ -2599,6 +2832,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr"/>
+      <c r="N48" t="inlineStr"/>
+      <c r="O48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -2619,7 +2856,7 @@
           <t>-21° 45´ 32.6517 -50° 06´ 02.9557 456.63</t>
         </is>
       </c>
-      <c r="E49" s="2" t="n">
+      <c r="E49" s="1" t="n">
         <v>46248</v>
       </c>
       <c r="F49" t="inlineStr">
@@ -2648,6 +2885,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr"/>
+      <c r="N49" t="inlineStr"/>
+      <c r="O49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -2658,7 +2899,9 @@
           <t>SÍTIO SANTO ANTÔNIO</t>
         </is>
       </c>
-      <c r="E50" s="2" t="n">
+      <c r="C50" t="inlineStr"/>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" s="1" t="n">
         <v>46248</v>
       </c>
       <c r="F50" t="inlineStr">
@@ -2687,6 +2930,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr"/>
+      <c r="N50" t="inlineStr"/>
+      <c r="O50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -2707,7 +2954,7 @@
           <t>-21° 48´ 26.1814 -50° 13´ 14.2006 438.00</t>
         </is>
       </c>
-      <c r="E51" s="2" t="n">
+      <c r="E51" s="1" t="n">
         <v>46258</v>
       </c>
       <c r="F51" t="inlineStr">
@@ -2736,6 +2983,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr"/>
+      <c r="N51" t="inlineStr"/>
+      <c r="O51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -2756,7 +3007,7 @@
           <t>-21° 24´ 42.3464 -50° 12´ 32.2760 396.57</t>
         </is>
       </c>
-      <c r="E52" s="2" t="n">
+      <c r="E52" s="1" t="n">
         <v>46259</v>
       </c>
       <c r="F52" t="inlineStr">
@@ -2785,6 +3036,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L52" t="inlineStr"/>
+      <c r="M52" t="inlineStr"/>
+      <c r="N52" t="inlineStr"/>
+      <c r="O52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -2805,7 +3060,7 @@
           <t>-21° 24´ 42.3464 -50° 12´ 32.2760 396.57</t>
         </is>
       </c>
-      <c r="E53" s="2" t="n">
+      <c r="E53" s="1" t="n">
         <v>46259</v>
       </c>
       <c r="F53" t="inlineStr">
@@ -2834,6 +3089,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L53" t="inlineStr"/>
+      <c r="M53" t="inlineStr"/>
+      <c r="N53" t="inlineStr"/>
+      <c r="O53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -2854,7 +3113,7 @@
           <t>-21° 47´ 12.2305 -50° 35´ 27.8405 436.14</t>
         </is>
       </c>
-      <c r="E54" s="2" t="n">
+      <c r="E54" s="1" t="n">
         <v>46261</v>
       </c>
       <c r="F54" t="inlineStr">
@@ -2862,12 +3121,19 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="G54" s="2" t="n">
+      <c r="G54" s="1" t="n">
         <v>46262</v>
       </c>
       <c r="H54" t="n">
         <v>200.36</v>
       </c>
+      <c r="I54" t="inlineStr"/>
+      <c r="J54" t="inlineStr"/>
+      <c r="K54" t="inlineStr"/>
+      <c r="L54" t="inlineStr"/>
+      <c r="M54" t="inlineStr"/>
+      <c r="N54" t="inlineStr"/>
+      <c r="O54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -2888,7 +3154,7 @@
           <t>-21° 39´ 13.2100 -50° 32´ 04.0182 418.26</t>
         </is>
       </c>
-      <c r="E55" s="2" t="n">
+      <c r="E55" s="1" t="n">
         <v>46261</v>
       </c>
       <c r="F55" t="inlineStr">
@@ -2917,6 +3183,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L55" t="inlineStr"/>
+      <c r="M55" t="inlineStr"/>
+      <c r="N55" t="inlineStr"/>
+      <c r="O55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -2937,7 +3207,7 @@
           <t>-21° 39´ 13.2100 -50° 32´ 04.0182 418.26</t>
         </is>
       </c>
-      <c r="E56" s="2" t="n">
+      <c r="E56" s="1" t="n">
         <v>46261</v>
       </c>
       <c r="F56" t="inlineStr">
@@ -2961,6 +3231,11 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="K56" t="inlineStr"/>
+      <c r="L56" t="inlineStr"/>
+      <c r="M56" t="inlineStr"/>
+      <c r="N56" t="inlineStr"/>
+      <c r="O56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -2971,7 +3246,9 @@
           <t>ESTÂNCIA BOA SORTE</t>
         </is>
       </c>
-      <c r="E57" s="2" t="n">
+      <c r="C57" t="inlineStr"/>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" s="1" t="n">
         <v>46248</v>
       </c>
       <c r="F57" t="inlineStr">
@@ -3000,6 +3277,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L57" t="inlineStr"/>
+      <c r="M57" t="inlineStr"/>
+      <c r="N57" t="inlineStr"/>
+      <c r="O57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -3010,7 +3291,9 @@
           <t>SITIO SANTA CLARA I</t>
         </is>
       </c>
-      <c r="E58" s="2" t="n">
+      <c r="C58" t="inlineStr"/>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" s="1" t="n">
         <v>46246</v>
       </c>
       <c r="F58" t="inlineStr">
@@ -3026,11 +3309,17 @@
       <c r="H58" t="n">
         <v>12.89</v>
       </c>
+      <c r="I58" t="inlineStr"/>
+      <c r="J58" t="inlineStr"/>
       <c r="K58" t="inlineStr">
         <is>
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L58" t="inlineStr"/>
+      <c r="M58" t="inlineStr"/>
+      <c r="N58" t="inlineStr"/>
+      <c r="O58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -3046,6 +3335,7 @@
           <t>B-19 SEDE TIAGO TUNES</t>
         </is>
       </c>
+      <c r="D59" t="inlineStr"/>
       <c r="E59" t="inlineStr">
         <is>
           <t>28/08/2026</t>
@@ -3064,11 +3354,17 @@
       <c r="H59" t="n">
         <v>37.72</v>
       </c>
+      <c r="I59" t="inlineStr"/>
+      <c r="J59" t="inlineStr"/>
       <c r="K59" t="inlineStr">
         <is>
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L59" t="inlineStr"/>
+      <c r="M59" t="inlineStr"/>
+      <c r="N59" t="inlineStr"/>
+      <c r="O59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -3084,6 +3380,7 @@
           <t>B-19 SEDE TIAGO TUNES</t>
         </is>
       </c>
+      <c r="D60" t="inlineStr"/>
       <c r="E60" t="inlineStr">
         <is>
           <t>28/08/2026</t>
@@ -3110,6 +3407,11 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="K60" t="inlineStr"/>
+      <c r="L60" t="inlineStr"/>
+      <c r="M60" t="inlineStr"/>
+      <c r="N60" t="inlineStr"/>
+      <c r="O60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -3125,6 +3427,7 @@
           <t>B-19 SEDE TIAGO TUNES</t>
         </is>
       </c>
+      <c r="D61" t="inlineStr"/>
       <c r="E61" t="inlineStr">
         <is>
           <t>28/09/2026</t>
@@ -3151,6 +3454,11 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="K61" t="inlineStr"/>
+      <c r="L61" t="inlineStr"/>
+      <c r="M61" t="inlineStr"/>
+      <c r="N61" t="inlineStr"/>
+      <c r="O61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -3166,6 +3474,7 @@
           <t>B-19 SEDE TIAGO TUNES</t>
         </is>
       </c>
+      <c r="D62" t="inlineStr"/>
       <c r="E62" t="inlineStr">
         <is>
           <t>28/08/2026</t>
@@ -3197,6 +3506,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L62" t="inlineStr"/>
+      <c r="M62" t="inlineStr"/>
+      <c r="N62" t="inlineStr"/>
+      <c r="O62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -3207,6 +3520,8 @@
           <t>SITIO SÃO JOSE</t>
         </is>
       </c>
+      <c r="C63" t="inlineStr"/>
+      <c r="D63" t="inlineStr"/>
       <c r="E63" t="inlineStr">
         <is>
           <t>28/09/2026</t>
@@ -3233,6 +3548,11 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="K63" t="inlineStr"/>
+      <c r="L63" t="inlineStr"/>
+      <c r="M63" t="inlineStr"/>
+      <c r="N63" t="inlineStr"/>
+      <c r="O63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -3268,6 +3588,14 @@
           <t>09/09/2026</t>
         </is>
       </c>
+      <c r="H64" t="inlineStr"/>
+      <c r="I64" t="inlineStr"/>
+      <c r="J64" t="inlineStr"/>
+      <c r="K64" t="inlineStr"/>
+      <c r="L64" t="inlineStr"/>
+      <c r="M64" t="inlineStr"/>
+      <c r="N64" t="inlineStr"/>
+      <c r="O64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -3319,6 +3647,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L65" t="inlineStr"/>
+      <c r="M65" t="inlineStr"/>
+      <c r="N65" t="inlineStr"/>
+      <c r="O65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -3357,11 +3689,17 @@
       <c r="H66" t="n">
         <v>99.37</v>
       </c>
+      <c r="I66" t="inlineStr"/>
+      <c r="J66" t="inlineStr"/>
       <c r="K66" t="inlineStr">
         <is>
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L66" t="inlineStr"/>
+      <c r="M66" t="inlineStr"/>
+      <c r="N66" t="inlineStr"/>
+      <c r="O66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -3410,6 +3748,11 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="K67" t="inlineStr"/>
+      <c r="L67" t="inlineStr"/>
+      <c r="M67" t="inlineStr"/>
+      <c r="N67" t="inlineStr"/>
+      <c r="O67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -3458,6 +3801,11 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="K68" t="inlineStr"/>
+      <c r="L68" t="inlineStr"/>
+      <c r="M68" t="inlineStr"/>
+      <c r="N68" t="inlineStr"/>
+      <c r="O68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -3509,6 +3857,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L69" t="inlineStr"/>
+      <c r="M69" t="inlineStr"/>
+      <c r="N69" t="inlineStr"/>
+      <c r="O69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -3560,6 +3912,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L70" t="inlineStr"/>
+      <c r="M70" t="inlineStr"/>
+      <c r="N70" t="inlineStr"/>
+      <c r="O70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -3570,6 +3926,8 @@
           <t>SÍTIO LIMEIRA</t>
         </is>
       </c>
+      <c r="C71" t="inlineStr"/>
+      <c r="D71" t="inlineStr"/>
       <c r="E71" t="inlineStr">
         <is>
           <t>04/09/2026</t>
@@ -3588,6 +3946,13 @@
       <c r="H71" t="n">
         <v>59.32</v>
       </c>
+      <c r="I71" t="inlineStr"/>
+      <c r="J71" t="inlineStr"/>
+      <c r="K71" t="inlineStr"/>
+      <c r="L71" t="inlineStr"/>
+      <c r="M71" t="inlineStr"/>
+      <c r="N71" t="inlineStr"/>
+      <c r="O71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -3626,6 +3991,13 @@
       <c r="H72" t="n">
         <v>669.6</v>
       </c>
+      <c r="I72" t="inlineStr"/>
+      <c r="J72" t="inlineStr"/>
+      <c r="K72" t="inlineStr"/>
+      <c r="L72" t="inlineStr"/>
+      <c r="M72" t="inlineStr"/>
+      <c r="N72" t="inlineStr"/>
+      <c r="O72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -3664,6 +4036,13 @@
       <c r="H73" t="n">
         <v>42.13</v>
       </c>
+      <c r="I73" t="inlineStr"/>
+      <c r="J73" t="inlineStr"/>
+      <c r="K73" t="inlineStr"/>
+      <c r="L73" t="inlineStr"/>
+      <c r="M73" t="inlineStr"/>
+      <c r="N73" t="inlineStr"/>
+      <c r="O73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -3679,6 +4058,7 @@
           <t>B-23 FAZ NOSSA SENHORA APARECIDA</t>
         </is>
       </c>
+      <c r="D74" t="inlineStr"/>
       <c r="E74" t="inlineStr">
         <is>
           <t>10/09/2026</t>
@@ -3710,6 +4090,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L74" t="inlineStr"/>
+      <c r="M74" t="inlineStr"/>
+      <c r="N74" t="inlineStr"/>
+      <c r="O74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -3725,6 +4109,7 @@
           <t>B-24 CENTRO RURAL</t>
         </is>
       </c>
+      <c r="D75" t="inlineStr"/>
       <c r="E75" t="inlineStr">
         <is>
           <t>11/09/2026</t>
@@ -3751,6 +4136,11 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="K75" t="inlineStr"/>
+      <c r="L75" t="inlineStr"/>
+      <c r="M75" t="inlineStr"/>
+      <c r="N75" t="inlineStr"/>
+      <c r="O75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -3766,6 +4156,7 @@
           <t>B-24 CENTRO RURAL</t>
         </is>
       </c>
+      <c r="D76" t="inlineStr"/>
       <c r="E76" t="inlineStr">
         <is>
           <t>11/09/2026</t>
@@ -3797,6 +4188,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L76" t="inlineStr"/>
+      <c r="M76" t="inlineStr"/>
+      <c r="N76" t="inlineStr"/>
+      <c r="O76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -3812,6 +4207,7 @@
           <t>B-24 CENTRO RURAL</t>
         </is>
       </c>
+      <c r="D77" t="inlineStr"/>
       <c r="E77" t="inlineStr">
         <is>
           <t>11/09/2026</t>
@@ -3827,6 +4223,14 @@
           <t>15/09/2026</t>
         </is>
       </c>
+      <c r="H77" t="inlineStr"/>
+      <c r="I77" t="inlineStr"/>
+      <c r="J77" t="inlineStr"/>
+      <c r="K77" t="inlineStr"/>
+      <c r="L77" t="inlineStr"/>
+      <c r="M77" t="inlineStr"/>
+      <c r="N77" t="inlineStr"/>
+      <c r="O77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -3842,6 +4246,7 @@
           <t>B-24 CENTRO RURAL</t>
         </is>
       </c>
+      <c r="D78" t="inlineStr"/>
       <c r="E78" t="inlineStr">
         <is>
           <t>11/09/2026</t>
@@ -3868,6 +4273,11 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="K78" t="inlineStr"/>
+      <c r="L78" t="inlineStr"/>
+      <c r="M78" t="inlineStr"/>
+      <c r="N78" t="inlineStr"/>
+      <c r="O78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -3883,6 +4293,7 @@
           <t>B-24 CENTRO RURAL</t>
         </is>
       </c>
+      <c r="D79" t="inlineStr"/>
       <c r="E79" t="inlineStr">
         <is>
           <t>11/09/2026</t>
@@ -3909,6 +4320,11 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="K79" t="inlineStr"/>
+      <c r="L79" t="inlineStr"/>
+      <c r="M79" t="inlineStr"/>
+      <c r="N79" t="inlineStr"/>
+      <c r="O79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -3960,6 +4376,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L80" t="inlineStr"/>
+      <c r="M80" t="inlineStr"/>
+      <c r="N80" t="inlineStr"/>
+      <c r="O80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -3998,11 +4418,17 @@
       <c r="H81" t="n">
         <v>84.09</v>
       </c>
+      <c r="I81" t="inlineStr"/>
+      <c r="J81" t="inlineStr"/>
       <c r="K81" t="inlineStr">
         <is>
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L81" t="inlineStr"/>
+      <c r="M81" t="inlineStr"/>
+      <c r="N81" t="inlineStr"/>
+      <c r="O81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -4018,6 +4444,7 @@
           <t>B-24 CENTRO RURAL</t>
         </is>
       </c>
+      <c r="D82" t="inlineStr"/>
       <c r="E82" t="inlineStr">
         <is>
           <t>11/09/2026</t>
@@ -4044,6 +4471,11 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="K82" t="inlineStr"/>
+      <c r="L82" t="inlineStr"/>
+      <c r="M82" t="inlineStr"/>
+      <c r="N82" t="inlineStr"/>
+      <c r="O82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -4079,6 +4511,14 @@
           <t>17/09/2026</t>
         </is>
       </c>
+      <c r="H83" t="inlineStr"/>
+      <c r="I83" t="inlineStr"/>
+      <c r="J83" t="inlineStr"/>
+      <c r="K83" t="inlineStr"/>
+      <c r="L83" t="inlineStr"/>
+      <c r="M83" t="inlineStr"/>
+      <c r="N83" t="inlineStr"/>
+      <c r="O83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -4130,6 +4570,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L84" t="inlineStr"/>
+      <c r="M84" t="inlineStr"/>
+      <c r="N84" t="inlineStr"/>
+      <c r="O84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -4176,6 +4620,11 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="K85" t="inlineStr"/>
+      <c r="L85" t="inlineStr"/>
+      <c r="M85" t="inlineStr"/>
+      <c r="N85" t="inlineStr"/>
+      <c r="O85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -4227,6 +4676,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L86" t="inlineStr"/>
+      <c r="M86" t="inlineStr"/>
+      <c r="N86" t="inlineStr"/>
+      <c r="O86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -4278,6 +4731,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L87" t="inlineStr"/>
+      <c r="M87" t="inlineStr"/>
+      <c r="N87" t="inlineStr"/>
+      <c r="O87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -4329,6 +4786,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L88" t="inlineStr"/>
+      <c r="M88" t="inlineStr"/>
+      <c r="N88" t="inlineStr"/>
+      <c r="O88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -4344,6 +4805,7 @@
           <t>B-09 FAZ SANTA ROSA AURELIO</t>
         </is>
       </c>
+      <c r="D89" t="inlineStr"/>
       <c r="E89" t="inlineStr">
         <is>
           <t>18/09/2026</t>
@@ -4362,11 +4824,17 @@
       <c r="H89" t="n">
         <v>552.0599999999999</v>
       </c>
+      <c r="I89" t="inlineStr"/>
+      <c r="J89" t="inlineStr"/>
       <c r="K89" t="inlineStr">
         <is>
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L89" t="inlineStr"/>
+      <c r="M89" t="inlineStr"/>
+      <c r="N89" t="inlineStr"/>
+      <c r="O89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -4382,6 +4850,7 @@
           <t>B-24 CENTRO RURAL</t>
         </is>
       </c>
+      <c r="D90" t="inlineStr"/>
       <c r="E90" t="inlineStr">
         <is>
           <t>11/09/2026</t>
@@ -4392,7 +4861,7 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="G90" s="2" t="n">
+      <c r="G90" s="1" t="n">
         <v>46286</v>
       </c>
       <c r="H90" t="n">
@@ -4406,6 +4875,11 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="K90" t="inlineStr"/>
+      <c r="L90" t="inlineStr"/>
+      <c r="M90" t="inlineStr"/>
+      <c r="N90" t="inlineStr"/>
+      <c r="O90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -4436,7 +4910,7 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="G91" s="2" t="n">
+      <c r="G91" s="1" t="n">
         <v>46286</v>
       </c>
       <c r="H91" t="n">
@@ -4455,6 +4929,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L91" t="inlineStr"/>
+      <c r="M91" t="inlineStr"/>
+      <c r="N91" t="inlineStr"/>
+      <c r="O91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -4485,7 +4963,7 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="G92" s="2" t="n">
+      <c r="G92" s="1" t="n">
         <v>46286</v>
       </c>
       <c r="H92" t="n">
@@ -4504,6 +4982,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L92" t="inlineStr"/>
+      <c r="M92" t="inlineStr"/>
+      <c r="N92" t="inlineStr"/>
+      <c r="O92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -4519,6 +5001,7 @@
           <t>B-23 FAZ NOSSA SENHORA APARECIDA</t>
         </is>
       </c>
+      <c r="D93" t="inlineStr"/>
       <c r="E93" t="inlineStr">
         <is>
           <t>21/09/2026</t>
@@ -4550,6 +5033,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L93" t="inlineStr"/>
+      <c r="M93" t="inlineStr"/>
+      <c r="N93" t="inlineStr"/>
+      <c r="O93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -4601,6 +5088,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L94" t="inlineStr"/>
+      <c r="M94" t="inlineStr"/>
+      <c r="N94" t="inlineStr"/>
+      <c r="O94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -4616,6 +5107,7 @@
           <t>B-23 FAZ NOSSA SENHORA APARECIDA</t>
         </is>
       </c>
+      <c r="D95" t="inlineStr"/>
       <c r="E95" t="inlineStr">
         <is>
           <t>21/09/2026</t>
@@ -4631,6 +5123,7 @@
           <t>24/07/2026</t>
         </is>
       </c>
+      <c r="H95" t="inlineStr"/>
       <c r="I95" t="n">
         <v>82.73999999999999</v>
       </c>
@@ -4639,6 +5132,11 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="K95" t="inlineStr"/>
+      <c r="L95" t="inlineStr"/>
+      <c r="M95" t="inlineStr"/>
+      <c r="N95" t="inlineStr"/>
+      <c r="O95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -4654,6 +5152,7 @@
           <t>B-016 FAZ RODA VIVA</t>
         </is>
       </c>
+      <c r="D96" t="inlineStr"/>
       <c r="E96" t="inlineStr">
         <is>
           <t>24/09/2026</t>
@@ -4672,11 +5171,17 @@
       <c r="H96" t="n">
         <v>345.05</v>
       </c>
+      <c r="I96" t="inlineStr"/>
+      <c r="J96" t="inlineStr"/>
       <c r="K96" t="inlineStr">
         <is>
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L96" t="inlineStr"/>
+      <c r="M96" t="inlineStr"/>
+      <c r="N96" t="inlineStr"/>
+      <c r="O96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -4723,6 +5228,11 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="K97" t="inlineStr"/>
+      <c r="L97" t="inlineStr"/>
+      <c r="M97" t="inlineStr"/>
+      <c r="N97" t="inlineStr"/>
+      <c r="O97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -4769,6 +5279,11 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="K98" t="inlineStr"/>
+      <c r="L98" t="inlineStr"/>
+      <c r="M98" t="inlineStr"/>
+      <c r="N98" t="inlineStr"/>
+      <c r="O98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -4815,6 +5330,11 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="K99" t="inlineStr"/>
+      <c r="L99" t="inlineStr"/>
+      <c r="M99" t="inlineStr"/>
+      <c r="N99" t="inlineStr"/>
+      <c r="O99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -4861,6 +5381,11 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="K100" t="inlineStr"/>
+      <c r="L100" t="inlineStr"/>
+      <c r="M100" t="inlineStr"/>
+      <c r="N100" t="inlineStr"/>
+      <c r="O100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -4876,6 +5401,7 @@
           <t>B-04 HARAS BILAC</t>
         </is>
       </c>
+      <c r="D101" t="inlineStr"/>
       <c r="E101" t="inlineStr">
         <is>
           <t>23/09/2026</t>
@@ -4907,6 +5433,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L101" t="inlineStr"/>
+      <c r="M101" t="inlineStr"/>
+      <c r="N101" t="inlineStr"/>
+      <c r="O101" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -19770,6 +20300,7 @@
       <c r="E391" t="n">
         <v>18.47</v>
       </c>
+      <c r="F391" t="inlineStr"/>
       <c r="G391" t="n">
         <v>0</v>
       </c>
@@ -19803,6 +20334,7 @@
       <c r="E392" t="n">
         <v>10.7</v>
       </c>
+      <c r="F392" t="inlineStr"/>
       <c r="G392" t="n">
         <v>0</v>
       </c>
@@ -19836,6 +20368,7 @@
       <c r="E393" t="n">
         <v>3.89</v>
       </c>
+      <c r="F393" t="inlineStr"/>
       <c r="G393" t="n">
         <v>0</v>
       </c>
@@ -19932,7 +20465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H84"/>
+  <dimension ref="A1:H85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22088,12 +22621,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>308098</t>
+          <t>308096</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>SÍTIO SANTA MARCELINA - 301274 - SÍTIO LIMEIRA</t>
+          <t>SÍTIO TAKATA</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -22102,16 +22635,16 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>45.53</v>
+        <v>46.86</v>
       </c>
       <c r="E64" t="n">
-        <v>585824.86</v>
+        <v>776146.4500000001</v>
       </c>
       <c r="F64" t="n">
-        <v>1500</v>
+        <v>1653.8</v>
       </c>
       <c r="G64" t="n">
-        <v>0.26</v>
+        <v>0.21</v>
       </c>
       <c r="H64" t="inlineStr">
         <is>
@@ -22122,12 +22655,12 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>308112</t>
+          <t>308098</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>SÍTIO UNIÃO</t>
+          <t>SÍTIO SANTA MARCELINA - 301274 - SÍTIO LIMEIRA</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -22136,16 +22669,16 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>27.59</v>
+        <v>45.53</v>
       </c>
       <c r="E65" t="n">
-        <v>367038.91</v>
+        <v>585824.86</v>
       </c>
       <c r="F65" t="n">
-        <v>1515</v>
+        <v>1500</v>
       </c>
       <c r="G65" t="n">
-        <v>0.41</v>
+        <v>0.26</v>
       </c>
       <c r="H65" t="inlineStr">
         <is>
@@ -22156,12 +22689,12 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>308120</t>
+          <t>308112</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>ESTÂNCIA PRIMAVERA</t>
+          <t>SÍTIO UNIÃO</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -22170,16 +22703,16 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>10.06</v>
+        <v>27.59</v>
       </c>
       <c r="E66" t="n">
-        <v>135639.5</v>
+        <v>367038.91</v>
       </c>
       <c r="F66" t="n">
-        <v>508.4000000000001</v>
+        <v>1515</v>
       </c>
       <c r="G66" t="n">
-        <v>0.37</v>
+        <v>0.41</v>
       </c>
       <c r="H66" t="inlineStr">
         <is>
@@ -22190,12 +22723,12 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>308123</t>
+          <t>308120</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>SÍTIO SANTO ANTÔNIO</t>
+          <t>ESTÂNCIA PRIMAVERA</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -22204,16 +22737,16 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>33.25</v>
+        <v>10.06</v>
       </c>
       <c r="E67" t="n">
-        <v>448944.35</v>
+        <v>135639.5</v>
       </c>
       <c r="F67" t="n">
-        <v>5004.799999999999</v>
+        <v>508.4000000000001</v>
       </c>
       <c r="G67" t="n">
-        <v>1.11</v>
+        <v>0.37</v>
       </c>
       <c r="H67" t="inlineStr">
         <is>
@@ -22224,12 +22757,12 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>308152</t>
+          <t>308123</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>FAZENDA SÃO JOÃO DA BARRA</t>
+          <t>SÍTIO SANTO ANTÔNIO</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -22238,16 +22771,16 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>190.43</v>
+        <v>33.25</v>
       </c>
       <c r="E68" t="n">
-        <v>2511618.14</v>
+        <v>448944.35</v>
       </c>
       <c r="F68" t="n">
-        <v>72840.20000000001</v>
+        <v>5004.799999999999</v>
       </c>
       <c r="G68" t="n">
-        <v>2.9</v>
+        <v>1.11</v>
       </c>
       <c r="H68" t="inlineStr">
         <is>
@@ -22258,12 +22791,12 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>308186</t>
+          <t>308152</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>FAZENDA SANTA RITA</t>
+          <t>FAZENDA SÃO JOÃO DA BARRA</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -22272,16 +22805,16 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>98.25</v>
+        <v>190.43</v>
       </c>
       <c r="E69" t="n">
-        <v>1287741.67</v>
+        <v>2511618.14</v>
       </c>
       <c r="F69" t="n">
-        <v>13637.4</v>
+        <v>72840.20000000001</v>
       </c>
       <c r="G69" t="n">
-        <v>1.06</v>
+        <v>2.9</v>
       </c>
       <c r="H69" t="inlineStr">
         <is>
@@ -22292,12 +22825,12 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>308193</t>
+          <t>308186</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>SITIO IRMÃOS FERNANDES</t>
+          <t>FAZENDA SANTA RITA</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -22306,16 +22839,16 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>19.14</v>
+        <v>98.25</v>
       </c>
       <c r="E70" t="n">
-        <v>236647.12</v>
+        <v>1287741.67</v>
       </c>
       <c r="F70" t="n">
-        <v>9806</v>
+        <v>13637.4</v>
       </c>
       <c r="G70" t="n">
-        <v>4.14</v>
+        <v>1.06</v>
       </c>
       <c r="H70" t="inlineStr">
         <is>
@@ -22326,12 +22859,12 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>308214</t>
+          <t>308193</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>ESTANCIA DYMONT</t>
+          <t>SITIO IRMÃOS FERNANDES</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -22340,16 +22873,16 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>14.33</v>
+        <v>19.14</v>
       </c>
       <c r="E71" t="n">
-        <v>201117.62</v>
+        <v>236647.12</v>
       </c>
       <c r="F71" t="n">
-        <v>150.4</v>
+        <v>9806</v>
       </c>
       <c r="G71" t="n">
-        <v>0.07000000000000001</v>
+        <v>4.14</v>
       </c>
       <c r="H71" t="inlineStr">
         <is>
@@ -22360,12 +22893,12 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>308225</t>
+          <t>308214</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>SITIO BOM JESUS</t>
+          <t>ESTANCIA DYMONT</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -22374,16 +22907,16 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>42.9</v>
+        <v>14.33</v>
       </c>
       <c r="E72" t="n">
-        <v>567803.14</v>
+        <v>201117.62</v>
       </c>
       <c r="F72" t="n">
-        <v>2287.4</v>
+        <v>150.4</v>
       </c>
       <c r="G72" t="n">
-        <v>0.4</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="H72" t="inlineStr">
         <is>
@@ -22394,12 +22927,12 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>308226</t>
+          <t>308225</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>SITIO CAPITAO HONORIO</t>
+          <t>SITIO BOM JESUS</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -22408,16 +22941,16 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>43.04</v>
+        <v>42.9</v>
       </c>
       <c r="E73" t="n">
-        <v>593292.2899999999</v>
+        <v>567803.14</v>
       </c>
       <c r="F73" t="n">
-        <v>2039.4</v>
+        <v>2287.4</v>
       </c>
       <c r="G73" t="n">
-        <v>0.34</v>
+        <v>0.4</v>
       </c>
       <c r="H73" t="inlineStr">
         <is>
@@ -22428,12 +22961,12 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>308231</t>
+          <t>308226</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>SITIO SÃO FRANCISCO - 30310- SITIO SANTA HELENA</t>
+          <t>SITIO CAPITAO HONORIO</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -22442,16 +22975,16 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>15.89</v>
+        <v>43.04</v>
       </c>
       <c r="E74" t="n">
-        <v>221144.51</v>
+        <v>593292.2899999999</v>
       </c>
       <c r="F74" t="n">
-        <v>633.4000000000001</v>
+        <v>2039.4</v>
       </c>
       <c r="G74" t="n">
-        <v>0.29</v>
+        <v>0.34</v>
       </c>
       <c r="H74" t="inlineStr">
         <is>
@@ -22462,12 +22995,12 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>308233</t>
+          <t>308231</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>SITIO SÃO JOSÉ PEROLA</t>
+          <t>SITIO SÃO FRANCISCO - 30310- SITIO SANTA HELENA</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -22476,16 +23009,16 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>12.48</v>
+        <v>15.89</v>
       </c>
       <c r="E75" t="n">
-        <v>166148.27</v>
+        <v>221144.51</v>
       </c>
       <c r="F75" t="n">
-        <v>531.4</v>
+        <v>633.4000000000001</v>
       </c>
       <c r="G75" t="n">
-        <v>0.32</v>
+        <v>0.29</v>
       </c>
       <c r="H75" t="inlineStr">
         <is>
@@ -22496,12 +23029,12 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>308238</t>
+          <t>308233</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>FAZ VALE DO SOL</t>
+          <t>SITIO SÃO JOSÉ PEROLA</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -22510,16 +23043,16 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>54.12</v>
+        <v>12.48</v>
       </c>
       <c r="E76" t="n">
-        <v>699691.55</v>
+        <v>166148.27</v>
       </c>
       <c r="F76" t="n">
-        <v>6555.2</v>
+        <v>531.4</v>
       </c>
       <c r="G76" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.32</v>
       </c>
       <c r="H76" t="inlineStr">
         <is>
@@ -22530,12 +23063,12 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>308239</t>
+          <t>308238</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>SITIO METODIO III</t>
+          <t>FAZ VALE DO SOL</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -22544,16 +23077,16 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>168.43</v>
+        <v>54.12</v>
       </c>
       <c r="E77" t="n">
-        <v>0</v>
+        <v>699691.55</v>
       </c>
       <c r="F77" t="n">
-        <v>0</v>
+        <v>6555.2</v>
       </c>
       <c r="G77" t="n">
-        <v>0</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="H77" t="inlineStr">
         <is>
@@ -22564,12 +23097,12 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>308247</t>
+          <t>308239</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>SITIO BOA VISTA</t>
+          <t>SITIO METODIO III</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -22578,16 +23111,16 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>51.26</v>
+        <v>168.43</v>
       </c>
       <c r="E78" t="n">
-        <v>669737.62</v>
+        <v>0</v>
       </c>
       <c r="F78" t="n">
-        <v>2331</v>
+        <v>0</v>
       </c>
       <c r="G78" t="n">
-        <v>0.35</v>
+        <v>0</v>
       </c>
       <c r="H78" t="inlineStr">
         <is>
@@ -22598,12 +23131,12 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>308248</t>
+          <t>308247</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>SITIO 3DJ</t>
+          <t>SITIO BOA VISTA</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -22612,16 +23145,16 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>18.01</v>
+        <v>51.26</v>
       </c>
       <c r="E79" t="n">
-        <v>215580.29</v>
+        <v>669737.62</v>
       </c>
       <c r="F79" t="n">
-        <v>4613.4</v>
+        <v>2331</v>
       </c>
       <c r="G79" t="n">
-        <v>2.14</v>
+        <v>0.35</v>
       </c>
       <c r="H79" t="inlineStr">
         <is>
@@ -22632,12 +23165,12 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>308261</t>
+          <t>308248</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>FAZ RIO FEIO</t>
+          <t>SITIO 3DJ</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -22646,16 +23179,16 @@
         </is>
       </c>
       <c r="D80" t="n">
-        <v>41.97</v>
+        <v>18.01</v>
       </c>
       <c r="E80" t="n">
-        <v>555218.6199999999</v>
+        <v>215580.29</v>
       </c>
       <c r="F80" t="n">
-        <v>27273.4</v>
+        <v>4613.4</v>
       </c>
       <c r="G80" t="n">
-        <v>4.91</v>
+        <v>2.14</v>
       </c>
       <c r="H80" t="inlineStr">
         <is>
@@ -22666,12 +23199,12 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>308268</t>
+          <t>308261</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>SITIO SÃO JOSE</t>
+          <t>FAZ RIO FEIO</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -22680,16 +23213,16 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>30.22</v>
+        <v>41.97</v>
       </c>
       <c r="E81" t="n">
-        <v>401557.88</v>
+        <v>555218.6199999999</v>
       </c>
       <c r="F81" t="n">
-        <v>1984.8</v>
+        <v>27273.4</v>
       </c>
       <c r="G81" t="n">
-        <v>0.49</v>
+        <v>4.91</v>
       </c>
       <c r="H81" t="inlineStr">
         <is>
@@ -22700,12 +23233,12 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>308269</t>
+          <t>308268</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>FAZENDA SANTA CECILIA</t>
+          <t>SITIO SÃO JOSE</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -22714,16 +23247,16 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>55.4</v>
+        <v>30.22</v>
       </c>
       <c r="E82" t="n">
-        <v>735048.67</v>
+        <v>401557.88</v>
       </c>
       <c r="F82" t="n">
-        <v>2871.400000000001</v>
+        <v>1984.8</v>
       </c>
       <c r="G82" t="n">
-        <v>0.39</v>
+        <v>0.49</v>
       </c>
       <c r="H82" t="inlineStr">
         <is>
@@ -22734,12 +23267,12 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>comparativo_kml_vs_banco_falhas</t>
+          <t>308269</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>FAZENDA SANTA CECILIA</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -22748,16 +23281,16 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>0</v>
+        <v>55.4</v>
       </c>
       <c r="E83" t="n">
-        <v>0</v>
+        <v>735048.67</v>
       </c>
       <c r="F83" t="n">
-        <v>0</v>
+        <v>2871.400000000001</v>
       </c>
       <c r="G83" t="n">
-        <v>0</v>
+        <v>0.39</v>
       </c>
       <c r="H83" t="inlineStr">
         <is>
@@ -22768,7 +23301,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>valores_coluna_C_linha_2</t>
+          <t>comparativo_kml_vs_banco_falhas</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -22794,6 +23327,40 @@
         <v>0</v>
       </c>
       <c r="H84" t="inlineStr">
+        <is>
+          <t>Aceitável</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>valores_coluna_C_linha_2</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Terceiro</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>0</v>
+      </c>
+      <c r="E85" t="n">
+        <v>0</v>
+      </c>
+      <c r="F85" t="n">
+        <v>0</v>
+      </c>
+      <c r="G85" t="n">
+        <v>0</v>
+      </c>
+      <c r="H85" t="inlineStr">
         <is>
           <t>Aceitável</t>
         </is>

</xml_diff>

<commit_message>
Atualizacao de dados: Thu 10/22/2026  7:03:50.94
</commit_message>
<xml_diff>
--- a/dados.xlsx
+++ b/dados.xlsx
@@ -5524,7 +5524,7 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -5562,7 +5562,7 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -5600,7 +5600,7 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -5638,7 +5638,7 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -5676,7 +5676,7 @@
         </is>
       </c>
       <c r="G6" t="n">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -5714,7 +5714,7 @@
         </is>
       </c>
       <c r="G7" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -5752,7 +5752,7 @@
         </is>
       </c>
       <c r="G8" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -5790,7 +5790,7 @@
         </is>
       </c>
       <c r="G9" t="n">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -5828,7 +5828,7 @@
         </is>
       </c>
       <c r="G10" t="n">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -5866,7 +5866,7 @@
         </is>
       </c>
       <c r="G11" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -5904,7 +5904,7 @@
         </is>
       </c>
       <c r="G12" t="n">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -5942,7 +5942,7 @@
         </is>
       </c>
       <c r="G13" t="n">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -5980,7 +5980,7 @@
         </is>
       </c>
       <c r="G14" t="n">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
@@ -6018,7 +6018,7 @@
         </is>
       </c>
       <c r="G15" t="n">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -6056,7 +6056,7 @@
         </is>
       </c>
       <c r="G16" t="n">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -6094,7 +6094,7 @@
         </is>
       </c>
       <c r="G17" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
@@ -6132,7 +6132,7 @@
         </is>
       </c>
       <c r="G18" t="n">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
@@ -6170,7 +6170,7 @@
         </is>
       </c>
       <c r="G19" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -6208,7 +6208,7 @@
         </is>
       </c>
       <c r="G20" t="n">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -6246,7 +6246,7 @@
         </is>
       </c>
       <c r="G21" t="n">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
@@ -6284,7 +6284,7 @@
         </is>
       </c>
       <c r="G22" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
@@ -6322,7 +6322,7 @@
         </is>
       </c>
       <c r="G23" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
@@ -6360,7 +6360,7 @@
         </is>
       </c>
       <c r="G24" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
@@ -6398,7 +6398,7 @@
         </is>
       </c>
       <c r="G25" t="n">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
@@ -6436,7 +6436,7 @@
         </is>
       </c>
       <c r="G26" t="n">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
@@ -6474,7 +6474,7 @@
         </is>
       </c>
       <c r="G27" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
@@ -6512,7 +6512,7 @@
         </is>
       </c>
       <c r="G28" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
@@ -6550,7 +6550,7 @@
         </is>
       </c>
       <c r="G29" t="n">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="H29" t="inlineStr">
         <is>
@@ -6588,7 +6588,7 @@
         </is>
       </c>
       <c r="G30" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
@@ -6626,7 +6626,7 @@
         </is>
       </c>
       <c r="G31" t="n">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
@@ -6664,7 +6664,7 @@
         </is>
       </c>
       <c r="G32" t="n">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="H32" t="inlineStr">
         <is>
@@ -6702,7 +6702,7 @@
         </is>
       </c>
       <c r="G33" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="H33" t="inlineStr">
         <is>
@@ -6740,7 +6740,7 @@
         </is>
       </c>
       <c r="G34" t="n">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>
@@ -6778,7 +6778,7 @@
         </is>
       </c>
       <c r="G35" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
@@ -6816,7 +6816,7 @@
         </is>
       </c>
       <c r="G36" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
@@ -6854,7 +6854,7 @@
         </is>
       </c>
       <c r="G37" t="n">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
@@ -6892,7 +6892,7 @@
         </is>
       </c>
       <c r="G38" t="n">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H38" t="inlineStr">
         <is>
@@ -6930,7 +6930,7 @@
         </is>
       </c>
       <c r="G39" t="n">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
@@ -6968,7 +6968,7 @@
         </is>
       </c>
       <c r="G40" t="n">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
@@ -7006,7 +7006,7 @@
         </is>
       </c>
       <c r="G41" t="n">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
@@ -7044,7 +7044,7 @@
         </is>
       </c>
       <c r="G42" t="n">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
@@ -7082,7 +7082,7 @@
         </is>
       </c>
       <c r="G43" t="n">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
@@ -7120,7 +7120,7 @@
         </is>
       </c>
       <c r="G44" t="n">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="H44" t="inlineStr">
         <is>
@@ -7158,7 +7158,7 @@
         </is>
       </c>
       <c r="G45" t="n">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>
@@ -7196,7 +7196,7 @@
         </is>
       </c>
       <c r="G46" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H46" t="inlineStr">
         <is>
@@ -7234,7 +7234,7 @@
         </is>
       </c>
       <c r="G47" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="H47" t="inlineStr">
         <is>
@@ -7272,7 +7272,7 @@
         </is>
       </c>
       <c r="G48" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H48" t="inlineStr">
         <is>
@@ -7310,7 +7310,7 @@
         </is>
       </c>
       <c r="G49" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H49" t="inlineStr">
         <is>
@@ -7348,7 +7348,7 @@
         </is>
       </c>
       <c r="G50" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H50" t="inlineStr">
         <is>
@@ -7386,7 +7386,7 @@
         </is>
       </c>
       <c r="G51" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="H51" t="inlineStr">
         <is>
@@ -7424,7 +7424,7 @@
         </is>
       </c>
       <c r="G52" t="n">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H52" t="inlineStr">
         <is>
@@ -7462,7 +7462,7 @@
         </is>
       </c>
       <c r="G53" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="H53" t="inlineStr">
         <is>
@@ -7500,7 +7500,7 @@
         </is>
       </c>
       <c r="G54" t="n">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="H54" t="inlineStr">
         <is>
@@ -7538,7 +7538,7 @@
         </is>
       </c>
       <c r="G55" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H55" t="inlineStr">
         <is>
@@ -7576,7 +7576,7 @@
         </is>
       </c>
       <c r="G56" t="n">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="H56" t="inlineStr">
         <is>
@@ -7614,7 +7614,7 @@
         </is>
       </c>
       <c r="G57" t="n">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H57" t="inlineStr">
         <is>
@@ -7652,7 +7652,7 @@
         </is>
       </c>
       <c r="G58" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H58" t="inlineStr">
         <is>
@@ -7690,7 +7690,7 @@
         </is>
       </c>
       <c r="G59" t="n">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="H59" t="inlineStr">
         <is>
@@ -7728,7 +7728,7 @@
         </is>
       </c>
       <c r="G60" t="n">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H60" t="inlineStr">
         <is>
@@ -7766,7 +7766,7 @@
         </is>
       </c>
       <c r="G61" t="n">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H61" t="inlineStr">
         <is>
@@ -7804,7 +7804,7 @@
         </is>
       </c>
       <c r="G62" t="n">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="H62" t="inlineStr">
         <is>
@@ -7842,7 +7842,7 @@
         </is>
       </c>
       <c r="G63" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="H63" t="inlineStr">
         <is>
@@ -7880,7 +7880,7 @@
         </is>
       </c>
       <c r="G64" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H64" t="inlineStr">
         <is>
@@ -7918,7 +7918,7 @@
         </is>
       </c>
       <c r="G65" t="n">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H65" t="inlineStr">
         <is>
@@ -7956,7 +7956,7 @@
         </is>
       </c>
       <c r="G66" t="n">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="H66" t="inlineStr">
         <is>
@@ -7994,7 +7994,7 @@
         </is>
       </c>
       <c r="G67" t="n">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H67" t="inlineStr">
         <is>
@@ -8032,7 +8032,7 @@
         </is>
       </c>
       <c r="G68" t="n">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="H68" t="inlineStr">
         <is>
@@ -8070,7 +8070,7 @@
         </is>
       </c>
       <c r="G69" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H69" t="inlineStr">
         <is>
@@ -8108,7 +8108,7 @@
         </is>
       </c>
       <c r="G70" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H70" t="inlineStr">
         <is>
@@ -8146,7 +8146,7 @@
         </is>
       </c>
       <c r="G71" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H71" t="inlineStr">
         <is>
@@ -8184,7 +8184,7 @@
         </is>
       </c>
       <c r="G72" t="n">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H72" t="inlineStr">
         <is>
@@ -8222,7 +8222,7 @@
         </is>
       </c>
       <c r="G73" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="H73" t="inlineStr">
         <is>
@@ -8260,7 +8260,7 @@
         </is>
       </c>
       <c r="G74" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="H74" t="inlineStr">
         <is>
@@ -8298,7 +8298,7 @@
         </is>
       </c>
       <c r="G75" t="n">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="H75" t="inlineStr">
         <is>
@@ -8336,7 +8336,7 @@
         </is>
       </c>
       <c r="G76" t="n">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="H76" t="inlineStr">
         <is>
@@ -8374,7 +8374,7 @@
         </is>
       </c>
       <c r="G77" t="n">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="H77" t="inlineStr">
         <is>
@@ -8412,7 +8412,7 @@
         </is>
       </c>
       <c r="G78" t="n">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="H78" t="inlineStr">
         <is>
@@ -8450,7 +8450,7 @@
         </is>
       </c>
       <c r="G79" t="n">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H79" t="inlineStr">
         <is>
@@ -8488,7 +8488,7 @@
         </is>
       </c>
       <c r="G80" t="n">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H80" t="inlineStr">
         <is>
@@ -8526,7 +8526,7 @@
         </is>
       </c>
       <c r="G81" t="n">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="H81" t="inlineStr">
         <is>
@@ -8564,7 +8564,7 @@
         </is>
       </c>
       <c r="G82" t="n">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="H82" t="inlineStr">
         <is>
@@ -8602,7 +8602,7 @@
         </is>
       </c>
       <c r="G83" t="n">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="H83" t="inlineStr">
         <is>
@@ -8640,7 +8640,7 @@
         </is>
       </c>
       <c r="G84" t="n">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="H84" t="inlineStr">
         <is>
@@ -8678,7 +8678,7 @@
         </is>
       </c>
       <c r="G85" t="n">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H85" t="inlineStr">
         <is>
@@ -8716,7 +8716,7 @@
         </is>
       </c>
       <c r="G86" t="n">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="H86" t="inlineStr">
         <is>
@@ -8754,7 +8754,7 @@
         </is>
       </c>
       <c r="G87" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="H87" t="inlineStr">
         <is>
@@ -8792,7 +8792,7 @@
         </is>
       </c>
       <c r="G88" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H88" t="inlineStr">
         <is>
@@ -8830,7 +8830,7 @@
         </is>
       </c>
       <c r="G89" t="n">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="H89" t="inlineStr">
         <is>
@@ -8868,7 +8868,7 @@
         </is>
       </c>
       <c r="G90" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H90" t="inlineStr">
         <is>
@@ -8906,7 +8906,7 @@
         </is>
       </c>
       <c r="G91" t="n">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="H91" t="inlineStr">
         <is>
@@ -8944,7 +8944,7 @@
         </is>
       </c>
       <c r="G92" t="n">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="H92" t="inlineStr">
         <is>
@@ -8982,7 +8982,7 @@
         </is>
       </c>
       <c r="G93" t="n">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H93" t="inlineStr">
         <is>
@@ -9020,7 +9020,7 @@
         </is>
       </c>
       <c r="G94" t="n">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="H94" t="inlineStr">
         <is>
@@ -9058,7 +9058,7 @@
         </is>
       </c>
       <c r="G95" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H95" t="inlineStr">
         <is>
@@ -9096,7 +9096,7 @@
         </is>
       </c>
       <c r="G96" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="H96" t="inlineStr">
         <is>
@@ -9134,7 +9134,7 @@
         </is>
       </c>
       <c r="G97" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H97" t="inlineStr">
         <is>
@@ -9172,7 +9172,7 @@
         </is>
       </c>
       <c r="G98" t="n">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="H98" t="inlineStr">
         <is>
@@ -9210,7 +9210,7 @@
         </is>
       </c>
       <c r="G99" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="H99" t="inlineStr">
         <is>
@@ -9248,7 +9248,7 @@
         </is>
       </c>
       <c r="G100" t="n">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="H100" t="inlineStr">
         <is>
@@ -9286,7 +9286,7 @@
         </is>
       </c>
       <c r="G101" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="H101" t="inlineStr">
         <is>
@@ -9324,7 +9324,7 @@
         </is>
       </c>
       <c r="G102" t="n">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H102" t="inlineStr">
         <is>
@@ -9362,7 +9362,7 @@
         </is>
       </c>
       <c r="G103" t="n">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H103" t="inlineStr">
         <is>
@@ -9400,7 +9400,7 @@
         </is>
       </c>
       <c r="G104" t="n">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="H104" t="inlineStr">
         <is>
@@ -9438,7 +9438,7 @@
         </is>
       </c>
       <c r="G105" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H105" t="inlineStr">
         <is>
@@ -9476,7 +9476,7 @@
         </is>
       </c>
       <c r="G106" t="n">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="H106" t="inlineStr">
         <is>
@@ -9514,7 +9514,7 @@
         </is>
       </c>
       <c r="G107" t="n">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H107" t="inlineStr">
         <is>
@@ -9552,7 +9552,7 @@
         </is>
       </c>
       <c r="G108" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H108" t="inlineStr">
         <is>
@@ -9590,7 +9590,7 @@
         </is>
       </c>
       <c r="G109" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H109" t="inlineStr">
         <is>
@@ -9628,7 +9628,7 @@
         </is>
       </c>
       <c r="G110" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H110" t="inlineStr">
         <is>
@@ -9666,7 +9666,7 @@
         </is>
       </c>
       <c r="G111" t="n">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="H111" t="inlineStr">
         <is>
@@ -9704,7 +9704,7 @@
         </is>
       </c>
       <c r="G112" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="H112" t="inlineStr">
         <is>
@@ -9742,7 +9742,7 @@
         </is>
       </c>
       <c r="G113" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H113" t="inlineStr">
         <is>
@@ -9780,7 +9780,7 @@
         </is>
       </c>
       <c r="G114" t="n">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="H114" t="inlineStr">
         <is>
@@ -9818,7 +9818,7 @@
         </is>
       </c>
       <c r="G115" t="n">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H115" t="inlineStr">
         <is>
@@ -9856,7 +9856,7 @@
         </is>
       </c>
       <c r="G116" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="H116" t="inlineStr">
         <is>
@@ -9894,7 +9894,7 @@
         </is>
       </c>
       <c r="G117" t="n">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H117" t="inlineStr">
         <is>
@@ -9932,7 +9932,7 @@
         </is>
       </c>
       <c r="G118" t="n">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="H118" t="inlineStr">
         <is>
@@ -9970,7 +9970,7 @@
         </is>
       </c>
       <c r="G119" t="n">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="H119" t="inlineStr">
         <is>
@@ -10008,7 +10008,7 @@
         </is>
       </c>
       <c r="G120" t="n">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="H120" t="inlineStr">
         <is>
@@ -10046,7 +10046,7 @@
         </is>
       </c>
       <c r="G121" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H121" t="inlineStr">
         <is>
@@ -10084,7 +10084,7 @@
         </is>
       </c>
       <c r="G122" t="n">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="H122" t="inlineStr">
         <is>
@@ -10122,7 +10122,7 @@
         </is>
       </c>
       <c r="G123" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="H123" t="inlineStr">
         <is>
@@ -10160,7 +10160,7 @@
         </is>
       </c>
       <c r="G124" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H124" t="inlineStr">
         <is>
@@ -10198,7 +10198,7 @@
         </is>
       </c>
       <c r="G125" t="n">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H125" t="inlineStr">
         <is>
@@ -10236,7 +10236,7 @@
         </is>
       </c>
       <c r="G126" t="n">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H126" t="inlineStr">
         <is>
@@ -10274,7 +10274,7 @@
         </is>
       </c>
       <c r="G127" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="H127" t="inlineStr">
         <is>
@@ -10312,7 +10312,7 @@
         </is>
       </c>
       <c r="G128" t="n">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="H128" t="inlineStr">
         <is>
@@ -10350,7 +10350,7 @@
         </is>
       </c>
       <c r="G129" t="n">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H129" t="inlineStr">
         <is>
@@ -10388,7 +10388,7 @@
         </is>
       </c>
       <c r="G130" t="n">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="H130" t="inlineStr">
         <is>
@@ -10426,7 +10426,7 @@
         </is>
       </c>
       <c r="G131" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H131" t="inlineStr">
         <is>
@@ -10464,7 +10464,7 @@
         </is>
       </c>
       <c r="G132" t="n">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H132" t="inlineStr">
         <is>
@@ -10502,7 +10502,7 @@
         </is>
       </c>
       <c r="G133" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="H133" t="inlineStr">
         <is>
@@ -10540,7 +10540,7 @@
         </is>
       </c>
       <c r="G134" t="n">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="H134" t="inlineStr">
         <is>
@@ -10578,7 +10578,7 @@
         </is>
       </c>
       <c r="G135" t="n">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H135" t="inlineStr">
         <is>
@@ -10616,7 +10616,7 @@
         </is>
       </c>
       <c r="G136" t="n">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H136" t="inlineStr">
         <is>
@@ -10654,7 +10654,7 @@
         </is>
       </c>
       <c r="G137" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H137" t="inlineStr">
         <is>
@@ -10692,7 +10692,7 @@
         </is>
       </c>
       <c r="G138" t="n">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H138" t="inlineStr">
         <is>
@@ -10730,7 +10730,7 @@
         </is>
       </c>
       <c r="G139" t="n">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H139" t="inlineStr">
         <is>
@@ -10768,7 +10768,7 @@
         </is>
       </c>
       <c r="G140" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="H140" t="inlineStr">
         <is>
@@ -10806,7 +10806,7 @@
         </is>
       </c>
       <c r="G141" t="n">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="H141" t="inlineStr">
         <is>
@@ -10844,7 +10844,7 @@
         </is>
       </c>
       <c r="G142" t="n">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H142" t="inlineStr">
         <is>
@@ -10882,7 +10882,7 @@
         </is>
       </c>
       <c r="G143" t="n">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H143" t="inlineStr">
         <is>
@@ -10920,7 +10920,7 @@
         </is>
       </c>
       <c r="G144" t="n">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H144" t="inlineStr">
         <is>
@@ -10958,7 +10958,7 @@
         </is>
       </c>
       <c r="G145" t="n">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="H145" t="inlineStr">
         <is>
@@ -10996,7 +10996,7 @@
         </is>
       </c>
       <c r="G146" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H146" t="inlineStr">
         <is>
@@ -11034,7 +11034,7 @@
         </is>
       </c>
       <c r="G147" t="n">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="H147" t="inlineStr">
         <is>
@@ -11072,7 +11072,7 @@
         </is>
       </c>
       <c r="G148" t="n">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="H148" t="inlineStr">
         <is>
@@ -11110,7 +11110,7 @@
         </is>
       </c>
       <c r="G149" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H149" t="inlineStr">
         <is>
@@ -11148,7 +11148,7 @@
         </is>
       </c>
       <c r="G150" t="n">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="H150" t="inlineStr">
         <is>
@@ -11186,7 +11186,7 @@
         </is>
       </c>
       <c r="G151" t="n">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="H151" t="inlineStr">
         <is>
@@ -11224,7 +11224,7 @@
         </is>
       </c>
       <c r="G152" t="n">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H152" t="inlineStr">
         <is>
@@ -11262,7 +11262,7 @@
         </is>
       </c>
       <c r="G153" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="H153" t="inlineStr">
         <is>
@@ -11300,7 +11300,7 @@
         </is>
       </c>
       <c r="G154" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H154" t="inlineStr">
         <is>
@@ -11338,7 +11338,7 @@
         </is>
       </c>
       <c r="G155" t="n">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="H155" t="inlineStr">
         <is>
@@ -11376,7 +11376,7 @@
         </is>
       </c>
       <c r="G156" t="n">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H156" t="inlineStr">
         <is>
@@ -11414,7 +11414,7 @@
         </is>
       </c>
       <c r="G157" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="H157" t="inlineStr">
         <is>
@@ -11452,7 +11452,7 @@
         </is>
       </c>
       <c r="G158" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="H158" t="inlineStr">
         <is>
@@ -11490,7 +11490,7 @@
         </is>
       </c>
       <c r="G159" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="H159" t="inlineStr">
         <is>
@@ -11528,7 +11528,7 @@
         </is>
       </c>
       <c r="G160" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H160" t="inlineStr">
         <is>
@@ -11566,7 +11566,7 @@
         </is>
       </c>
       <c r="G161" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="H161" t="inlineStr">
         <is>
@@ -11604,7 +11604,7 @@
         </is>
       </c>
       <c r="G162" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="H162" t="inlineStr">
         <is>
@@ -11642,7 +11642,7 @@
         </is>
       </c>
       <c r="G163" t="n">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="H163" t="inlineStr">
         <is>
@@ -11680,7 +11680,7 @@
         </is>
       </c>
       <c r="G164" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="H164" t="inlineStr">
         <is>
@@ -11718,7 +11718,7 @@
         </is>
       </c>
       <c r="G165" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H165" t="inlineStr">
         <is>
@@ -11756,7 +11756,7 @@
         </is>
       </c>
       <c r="G166" t="n">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="H166" t="inlineStr">
         <is>
@@ -11794,7 +11794,7 @@
         </is>
       </c>
       <c r="G167" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="H167" t="inlineStr">
         <is>
@@ -11832,7 +11832,7 @@
         </is>
       </c>
       <c r="G168" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H168" t="inlineStr">
         <is>
@@ -11870,7 +11870,7 @@
         </is>
       </c>
       <c r="G169" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="H169" t="inlineStr">
         <is>
@@ -11908,7 +11908,7 @@
         </is>
       </c>
       <c r="G170" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H170" t="inlineStr">
         <is>
@@ -11946,7 +11946,7 @@
         </is>
       </c>
       <c r="G171" t="n">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="H171" t="inlineStr">
         <is>
@@ -11984,7 +11984,7 @@
         </is>
       </c>
       <c r="G172" t="n">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H172" t="inlineStr">
         <is>
@@ -12022,7 +12022,7 @@
         </is>
       </c>
       <c r="G173" t="n">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="H173" t="inlineStr">
         <is>
@@ -12060,7 +12060,7 @@
         </is>
       </c>
       <c r="G174" t="n">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="H174" t="inlineStr">
         <is>
@@ -12098,7 +12098,7 @@
         </is>
       </c>
       <c r="G175" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="H175" t="inlineStr">
         <is>
@@ -12136,7 +12136,7 @@
         </is>
       </c>
       <c r="G176" t="n">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H176" t="inlineStr">
         <is>
@@ -12174,7 +12174,7 @@
         </is>
       </c>
       <c r="G177" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="H177" t="inlineStr">
         <is>
@@ -12212,7 +12212,7 @@
         </is>
       </c>
       <c r="G178" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H178" t="inlineStr">
         <is>
@@ -12250,7 +12250,7 @@
         </is>
       </c>
       <c r="G179" t="n">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="H179" t="inlineStr">
         <is>
@@ -12288,7 +12288,7 @@
         </is>
       </c>
       <c r="G180" t="n">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="H180" t="inlineStr">
         <is>
@@ -12326,7 +12326,7 @@
         </is>
       </c>
       <c r="G181" t="n">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="H181" t="inlineStr">
         <is>
@@ -12364,7 +12364,7 @@
         </is>
       </c>
       <c r="G182" t="n">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="H182" t="inlineStr">
         <is>
@@ -12402,7 +12402,7 @@
         </is>
       </c>
       <c r="G183" t="n">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="H183" t="inlineStr">
         <is>
@@ -12440,7 +12440,7 @@
         </is>
       </c>
       <c r="G184" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="H184" t="inlineStr">
         <is>
@@ -12478,7 +12478,7 @@
         </is>
       </c>
       <c r="G185" t="n">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="H185" t="inlineStr">
         <is>
@@ -12516,7 +12516,7 @@
         </is>
       </c>
       <c r="G186" t="n">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="H186" t="inlineStr">
         <is>
@@ -12554,7 +12554,7 @@
         </is>
       </c>
       <c r="G187" t="n">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H187" t="inlineStr">
         <is>
@@ -12592,7 +12592,7 @@
         </is>
       </c>
       <c r="G188" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H188" t="inlineStr">
         <is>
@@ -12630,7 +12630,7 @@
         </is>
       </c>
       <c r="G189" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H189" t="inlineStr">
         <is>
@@ -12668,7 +12668,7 @@
         </is>
       </c>
       <c r="G190" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="H190" t="inlineStr">
         <is>
@@ -12706,7 +12706,7 @@
         </is>
       </c>
       <c r="G191" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="H191" t="inlineStr">
         <is>
@@ -12744,7 +12744,7 @@
         </is>
       </c>
       <c r="G192" t="n">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H192" t="inlineStr">
         <is>
@@ -12782,7 +12782,7 @@
         </is>
       </c>
       <c r="G193" t="n">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="H193" t="inlineStr">
         <is>
@@ -12820,7 +12820,7 @@
         </is>
       </c>
       <c r="G194" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H194" t="inlineStr">
         <is>
@@ -12858,7 +12858,7 @@
         </is>
       </c>
       <c r="G195" t="n">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="H195" t="inlineStr">
         <is>
@@ -12896,7 +12896,7 @@
         </is>
       </c>
       <c r="G196" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H196" t="inlineStr">
         <is>
@@ -12934,7 +12934,7 @@
         </is>
       </c>
       <c r="G197" t="n">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="H197" t="inlineStr">
         <is>
@@ -12972,7 +12972,7 @@
         </is>
       </c>
       <c r="G198" t="n">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H198" t="inlineStr">
         <is>
@@ -13010,7 +13010,7 @@
         </is>
       </c>
       <c r="G199" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="H199" t="inlineStr">
         <is>
@@ -13048,7 +13048,7 @@
         </is>
       </c>
       <c r="G200" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H200" t="inlineStr">
         <is>
@@ -13086,7 +13086,7 @@
         </is>
       </c>
       <c r="G201" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="H201" t="inlineStr">
         <is>
@@ -13124,7 +13124,7 @@
         </is>
       </c>
       <c r="G202" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H202" t="inlineStr">
         <is>
@@ -13162,7 +13162,7 @@
         </is>
       </c>
       <c r="G203" t="n">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="H203" t="inlineStr">
         <is>
@@ -13200,7 +13200,7 @@
         </is>
       </c>
       <c r="G204" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H204" t="inlineStr">
         <is>
@@ -13238,7 +13238,7 @@
         </is>
       </c>
       <c r="G205" t="n">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="H205" t="inlineStr">
         <is>
@@ -13276,7 +13276,7 @@
         </is>
       </c>
       <c r="G206" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H206" t="inlineStr">
         <is>
@@ -13314,7 +13314,7 @@
         </is>
       </c>
       <c r="G207" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="H207" t="inlineStr">
         <is>
@@ -13352,7 +13352,7 @@
         </is>
       </c>
       <c r="G208" t="n">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="H208" t="inlineStr">
         <is>
@@ -13390,7 +13390,7 @@
         </is>
       </c>
       <c r="G209" t="n">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H209" t="inlineStr">
         <is>
@@ -13428,7 +13428,7 @@
         </is>
       </c>
       <c r="G210" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H210" t="inlineStr">
         <is>
@@ -13466,7 +13466,7 @@
         </is>
       </c>
       <c r="G211" t="n">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="H211" t="inlineStr">
         <is>
@@ -13504,7 +13504,7 @@
         </is>
       </c>
       <c r="G212" t="n">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="H212" t="inlineStr">
         <is>
@@ -13542,7 +13542,7 @@
         </is>
       </c>
       <c r="G213" t="n">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="H213" t="inlineStr">
         <is>
@@ -13580,7 +13580,7 @@
         </is>
       </c>
       <c r="G214" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H214" t="inlineStr">
         <is>
@@ -13618,7 +13618,7 @@
         </is>
       </c>
       <c r="G215" t="n">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H215" t="inlineStr">
         <is>
@@ -13656,7 +13656,7 @@
         </is>
       </c>
       <c r="G216" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H216" t="inlineStr">
         <is>
@@ -13694,7 +13694,7 @@
         </is>
       </c>
       <c r="G217" t="n">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="H217" t="inlineStr">
         <is>
@@ -13732,7 +13732,7 @@
         </is>
       </c>
       <c r="G218" t="n">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H218" t="inlineStr">
         <is>
@@ -13770,7 +13770,7 @@
         </is>
       </c>
       <c r="G219" t="n">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="H219" t="inlineStr">
         <is>
@@ -13808,7 +13808,7 @@
         </is>
       </c>
       <c r="G220" t="n">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="H220" t="inlineStr">
         <is>
@@ -13846,7 +13846,7 @@
         </is>
       </c>
       <c r="G221" t="n">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="H221" t="inlineStr">
         <is>
@@ -13884,7 +13884,7 @@
         </is>
       </c>
       <c r="G222" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H222" t="inlineStr">
         <is>
@@ -13922,7 +13922,7 @@
         </is>
       </c>
       <c r="G223" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="H223" t="inlineStr">
         <is>
@@ -13960,7 +13960,7 @@
         </is>
       </c>
       <c r="G224" t="n">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="H224" t="inlineStr">
         <is>
@@ -13998,7 +13998,7 @@
         </is>
       </c>
       <c r="G225" t="n">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="H225" t="inlineStr">
         <is>
@@ -14036,7 +14036,7 @@
         </is>
       </c>
       <c r="G226" t="n">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H226" t="inlineStr">
         <is>
@@ -14074,7 +14074,7 @@
         </is>
       </c>
       <c r="G227" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="H227" t="inlineStr">
         <is>
@@ -14112,7 +14112,7 @@
         </is>
       </c>
       <c r="G228" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="H228" t="inlineStr">
         <is>
@@ -14150,7 +14150,7 @@
         </is>
       </c>
       <c r="G229" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H229" t="inlineStr">
         <is>
@@ -14188,7 +14188,7 @@
         </is>
       </c>
       <c r="G230" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H230" t="inlineStr">
         <is>
@@ -14226,7 +14226,7 @@
         </is>
       </c>
       <c r="G231" t="n">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="H231" t="inlineStr">
         <is>
@@ -14264,7 +14264,7 @@
         </is>
       </c>
       <c r="G232" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H232" t="inlineStr">
         <is>
@@ -14302,7 +14302,7 @@
         </is>
       </c>
       <c r="G233" t="n">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="H233" t="inlineStr">
         <is>
@@ -14340,7 +14340,7 @@
         </is>
       </c>
       <c r="G234" t="n">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="H234" t="inlineStr">
         <is>
@@ -14378,7 +14378,7 @@
         </is>
       </c>
       <c r="G235" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H235" t="inlineStr">
         <is>
@@ -14416,7 +14416,7 @@
         </is>
       </c>
       <c r="G236" t="n">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H236" t="inlineStr">
         <is>
@@ -14454,7 +14454,7 @@
         </is>
       </c>
       <c r="G237" t="n">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="H237" t="inlineStr">
         <is>
@@ -14492,7 +14492,7 @@
         </is>
       </c>
       <c r="G238" t="n">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="H238" t="inlineStr">
         <is>
@@ -14530,7 +14530,7 @@
         </is>
       </c>
       <c r="G239" t="n">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="H239" t="inlineStr">
         <is>
@@ -14568,7 +14568,7 @@
         </is>
       </c>
       <c r="G240" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="H240" t="inlineStr">
         <is>
@@ -14606,7 +14606,7 @@
         </is>
       </c>
       <c r="G241" t="n">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H241" t="inlineStr">
         <is>
@@ -14644,7 +14644,7 @@
         </is>
       </c>
       <c r="G242" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="H242" t="inlineStr">
         <is>
@@ -14682,7 +14682,7 @@
         </is>
       </c>
       <c r="G243" t="n">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H243" t="inlineStr">
         <is>
@@ -14720,7 +14720,7 @@
         </is>
       </c>
       <c r="G244" t="n">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="H244" t="inlineStr">
         <is>
@@ -14758,7 +14758,7 @@
         </is>
       </c>
       <c r="G245" t="n">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="H245" t="inlineStr">
         <is>
@@ -14796,7 +14796,7 @@
         </is>
       </c>
       <c r="G246" t="n">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="H246" t="inlineStr">
         <is>
@@ -14834,7 +14834,7 @@
         </is>
       </c>
       <c r="G247" t="n">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="H247" t="inlineStr">
         <is>
@@ -14872,7 +14872,7 @@
         </is>
       </c>
       <c r="G248" t="n">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="H248" t="inlineStr">
         <is>
@@ -14910,7 +14910,7 @@
         </is>
       </c>
       <c r="G249" t="n">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="H249" t="inlineStr">
         <is>
@@ -14948,7 +14948,7 @@
         </is>
       </c>
       <c r="G250" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H250" t="inlineStr">
         <is>
@@ -14986,7 +14986,7 @@
         </is>
       </c>
       <c r="G251" t="n">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="H251" t="inlineStr">
         <is>
@@ -15024,7 +15024,7 @@
         </is>
       </c>
       <c r="G252" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="H252" t="inlineStr">
         <is>
@@ -15062,7 +15062,7 @@
         </is>
       </c>
       <c r="G253" t="n">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="H253" t="inlineStr">
         <is>
@@ -15100,7 +15100,7 @@
         </is>
       </c>
       <c r="G254" t="n">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H254" t="inlineStr">
         <is>
@@ -15138,7 +15138,7 @@
         </is>
       </c>
       <c r="G255" t="n">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="H255" t="inlineStr">
         <is>
@@ -15176,7 +15176,7 @@
         </is>
       </c>
       <c r="G256" t="n">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H256" t="inlineStr">
         <is>
@@ -15214,7 +15214,7 @@
         </is>
       </c>
       <c r="G257" t="n">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="H257" t="inlineStr">
         <is>
@@ -15252,7 +15252,7 @@
         </is>
       </c>
       <c r="G258" t="n">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="H258" t="inlineStr">
         <is>
@@ -15290,7 +15290,7 @@
         </is>
       </c>
       <c r="G259" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H259" t="inlineStr">
         <is>
@@ -15328,7 +15328,7 @@
         </is>
       </c>
       <c r="G260" t="n">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="H260" t="inlineStr">
         <is>
@@ -15366,7 +15366,7 @@
         </is>
       </c>
       <c r="G261" t="n">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="H261" t="inlineStr">
         <is>
@@ -15404,7 +15404,7 @@
         </is>
       </c>
       <c r="G262" t="n">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="H262" t="inlineStr">
         <is>
@@ -15442,7 +15442,7 @@
         </is>
       </c>
       <c r="G263" t="n">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H263" t="inlineStr">
         <is>
@@ -15480,7 +15480,7 @@
         </is>
       </c>
       <c r="G264" t="n">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="H264" t="inlineStr">
         <is>
@@ -15518,7 +15518,7 @@
         </is>
       </c>
       <c r="G265" t="n">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="H265" t="inlineStr">
         <is>
@@ -15556,7 +15556,7 @@
         </is>
       </c>
       <c r="G266" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="H266" t="inlineStr">
         <is>
@@ -15594,7 +15594,7 @@
         </is>
       </c>
       <c r="G267" t="n">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="H267" t="inlineStr">
         <is>
@@ -15632,7 +15632,7 @@
         </is>
       </c>
       <c r="G268" t="n">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H268" t="inlineStr">
         <is>
@@ -15670,7 +15670,7 @@
         </is>
       </c>
       <c r="G269" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="H269" t="inlineStr">
         <is>
@@ -15708,7 +15708,7 @@
         </is>
       </c>
       <c r="G270" t="n">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H270" t="inlineStr">
         <is>
@@ -15746,7 +15746,7 @@
         </is>
       </c>
       <c r="G271" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H271" t="inlineStr">
         <is>
@@ -15784,7 +15784,7 @@
         </is>
       </c>
       <c r="G272" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="H272" t="inlineStr">
         <is>
@@ -15822,7 +15822,7 @@
         </is>
       </c>
       <c r="G273" t="n">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="H273" t="inlineStr">
         <is>
@@ -15860,7 +15860,7 @@
         </is>
       </c>
       <c r="G274" t="n">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="H274" t="inlineStr">
         <is>
@@ -15898,7 +15898,7 @@
         </is>
       </c>
       <c r="G275" t="n">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H275" t="inlineStr">
         <is>
@@ -15936,7 +15936,7 @@
         </is>
       </c>
       <c r="G276" t="n">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="H276" t="inlineStr">
         <is>
@@ -15974,7 +15974,7 @@
         </is>
       </c>
       <c r="G277" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H277" t="inlineStr">
         <is>
@@ -16012,7 +16012,7 @@
         </is>
       </c>
       <c r="G278" t="n">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="H278" t="inlineStr">
         <is>
@@ -16050,7 +16050,7 @@
         </is>
       </c>
       <c r="G279" t="n">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H279" t="inlineStr">
         <is>
@@ -16088,7 +16088,7 @@
         </is>
       </c>
       <c r="G280" t="n">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="H280" t="inlineStr">
         <is>
@@ -16126,7 +16126,7 @@
         </is>
       </c>
       <c r="G281" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="H281" t="inlineStr">
         <is>
@@ -16164,7 +16164,7 @@
         </is>
       </c>
       <c r="G282" t="n">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="H282" t="inlineStr">
         <is>
@@ -16202,7 +16202,7 @@
         </is>
       </c>
       <c r="G283" t="n">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H283" t="inlineStr">
         <is>
@@ -16240,7 +16240,7 @@
         </is>
       </c>
       <c r="G284" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H284" t="inlineStr">
         <is>
@@ -16278,7 +16278,7 @@
         </is>
       </c>
       <c r="G285" t="n">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H285" t="inlineStr">
         <is>
@@ -16316,7 +16316,7 @@
         </is>
       </c>
       <c r="G286" t="n">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H286" t="inlineStr">
         <is>
@@ -16354,7 +16354,7 @@
         </is>
       </c>
       <c r="G287" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H287" t="inlineStr">
         <is>
@@ -16392,7 +16392,7 @@
         </is>
       </c>
       <c r="G288" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H288" t="inlineStr">
         <is>
@@ -16430,7 +16430,7 @@
         </is>
       </c>
       <c r="G289" t="n">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H289" t="inlineStr">
         <is>
@@ -16468,7 +16468,7 @@
         </is>
       </c>
       <c r="G290" t="n">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H290" t="inlineStr">
         <is>
@@ -16506,7 +16506,7 @@
         </is>
       </c>
       <c r="G291" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="H291" t="inlineStr">
         <is>
@@ -16544,7 +16544,7 @@
         </is>
       </c>
       <c r="G292" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H292" t="inlineStr">
         <is>
@@ -16582,7 +16582,7 @@
         </is>
       </c>
       <c r="G293" t="n">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H293" t="inlineStr">
         <is>
@@ -16620,7 +16620,7 @@
         </is>
       </c>
       <c r="G294" t="n">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H294" t="inlineStr">
         <is>
@@ -16658,7 +16658,7 @@
         </is>
       </c>
       <c r="G295" t="n">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="H295" t="inlineStr">
         <is>
@@ -16696,7 +16696,7 @@
         </is>
       </c>
       <c r="G296" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="H296" t="inlineStr">
         <is>
@@ -16734,7 +16734,7 @@
         </is>
       </c>
       <c r="G297" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H297" t="inlineStr">
         <is>
@@ -16772,7 +16772,7 @@
         </is>
       </c>
       <c r="G298" t="n">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="H298" t="inlineStr">
         <is>
@@ -16810,7 +16810,7 @@
         </is>
       </c>
       <c r="G299" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H299" t="inlineStr">
         <is>
@@ -16848,7 +16848,7 @@
         </is>
       </c>
       <c r="G300" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H300" t="inlineStr">
         <is>
@@ -16886,7 +16886,7 @@
         </is>
       </c>
       <c r="G301" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H301" t="inlineStr">
         <is>
@@ -16924,7 +16924,7 @@
         </is>
       </c>
       <c r="G302" t="n">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="H302" t="inlineStr">
         <is>
@@ -16962,7 +16962,7 @@
         </is>
       </c>
       <c r="G303" t="n">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H303" t="inlineStr">
         <is>
@@ -17000,7 +17000,7 @@
         </is>
       </c>
       <c r="G304" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H304" t="inlineStr">
         <is>
@@ -17038,7 +17038,7 @@
         </is>
       </c>
       <c r="G305" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H305" t="inlineStr">
         <is>
@@ -17076,7 +17076,7 @@
         </is>
       </c>
       <c r="G306" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="H306" t="inlineStr">
         <is>
@@ -17114,7 +17114,7 @@
         </is>
       </c>
       <c r="G307" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H307" t="inlineStr">
         <is>
@@ -17152,7 +17152,7 @@
         </is>
       </c>
       <c r="G308" t="n">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H308" t="inlineStr">
         <is>
@@ -17190,7 +17190,7 @@
         </is>
       </c>
       <c r="G309" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H309" t="inlineStr">
         <is>
@@ -17228,7 +17228,7 @@
         </is>
       </c>
       <c r="G310" t="n">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="H310" t="inlineStr">
         <is>
@@ -17266,7 +17266,7 @@
         </is>
       </c>
       <c r="G311" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="H311" t="inlineStr">
         <is>
@@ -17304,7 +17304,7 @@
         </is>
       </c>
       <c r="G312" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H312" t="inlineStr">
         <is>
@@ -17342,7 +17342,7 @@
         </is>
       </c>
       <c r="G313" t="n">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="H313" t="inlineStr">
         <is>
@@ -17380,7 +17380,7 @@
         </is>
       </c>
       <c r="G314" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H314" t="inlineStr">
         <is>
@@ -17418,7 +17418,7 @@
         </is>
       </c>
       <c r="G315" t="n">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="H315" t="inlineStr">
         <is>
@@ -17456,7 +17456,7 @@
         </is>
       </c>
       <c r="G316" t="n">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="H316" t="inlineStr">
         <is>
@@ -17494,7 +17494,7 @@
         </is>
       </c>
       <c r="G317" t="n">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H317" t="inlineStr">
         <is>
@@ -17532,7 +17532,7 @@
         </is>
       </c>
       <c r="G318" t="n">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H318" t="inlineStr">
         <is>
@@ -17570,7 +17570,7 @@
         </is>
       </c>
       <c r="G319" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="H319" t="inlineStr">
         <is>
@@ -17608,7 +17608,7 @@
         </is>
       </c>
       <c r="G320" t="n">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="H320" t="inlineStr">
         <is>
@@ -17646,7 +17646,7 @@
         </is>
       </c>
       <c r="G321" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H321" t="inlineStr">
         <is>
@@ -17684,7 +17684,7 @@
         </is>
       </c>
       <c r="G322" t="n">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H322" t="inlineStr">
         <is>
@@ -17722,7 +17722,7 @@
         </is>
       </c>
       <c r="G323" t="n">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="H323" t="inlineStr">
         <is>
@@ -17760,7 +17760,7 @@
         </is>
       </c>
       <c r="G324" t="n">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="H324" t="inlineStr">
         <is>
@@ -17798,7 +17798,7 @@
         </is>
       </c>
       <c r="G325" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="H325" t="inlineStr">
         <is>
@@ -17836,7 +17836,7 @@
         </is>
       </c>
       <c r="G326" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="H326" t="inlineStr">
         <is>
@@ -17874,7 +17874,7 @@
         </is>
       </c>
       <c r="G327" t="n">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H327" t="inlineStr">
         <is>
@@ -17912,7 +17912,7 @@
         </is>
       </c>
       <c r="G328" t="n">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="H328" t="inlineStr">
         <is>
@@ -17950,7 +17950,7 @@
         </is>
       </c>
       <c r="G329" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H329" t="inlineStr">
         <is>
@@ -17988,7 +17988,7 @@
         </is>
       </c>
       <c r="G330" t="n">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H330" t="inlineStr">
         <is>
@@ -18026,7 +18026,7 @@
         </is>
       </c>
       <c r="G331" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H331" t="inlineStr">
         <is>
@@ -18064,7 +18064,7 @@
         </is>
       </c>
       <c r="G332" t="n">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H332" t="inlineStr">
         <is>
@@ -18102,7 +18102,7 @@
         </is>
       </c>
       <c r="G333" t="n">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H333" t="inlineStr">
         <is>
@@ -18140,7 +18140,7 @@
         </is>
       </c>
       <c r="G334" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H334" t="inlineStr">
         <is>
@@ -18178,7 +18178,7 @@
         </is>
       </c>
       <c r="G335" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H335" t="inlineStr">
         <is>
@@ -18216,7 +18216,7 @@
         </is>
       </c>
       <c r="G336" t="n">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="H336" t="inlineStr">
         <is>
@@ -18254,7 +18254,7 @@
         </is>
       </c>
       <c r="G337" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="H337" t="inlineStr">
         <is>
@@ -18292,7 +18292,7 @@
         </is>
       </c>
       <c r="G338" t="n">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="H338" t="inlineStr">
         <is>
@@ -18330,7 +18330,7 @@
         </is>
       </c>
       <c r="G339" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H339" t="inlineStr">
         <is>
@@ -18368,7 +18368,7 @@
         </is>
       </c>
       <c r="G340" t="n">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H340" t="inlineStr">
         <is>
@@ -18406,7 +18406,7 @@
         </is>
       </c>
       <c r="G341" t="n">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="H341" t="inlineStr">
         <is>
@@ -18444,7 +18444,7 @@
         </is>
       </c>
       <c r="G342" t="n">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="H342" t="inlineStr">
         <is>
@@ -18482,7 +18482,7 @@
         </is>
       </c>
       <c r="G343" t="n">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="H343" t="inlineStr">
         <is>
@@ -18520,7 +18520,7 @@
         </is>
       </c>
       <c r="G344" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H344" t="inlineStr">
         <is>
@@ -18558,7 +18558,7 @@
         </is>
       </c>
       <c r="G345" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H345" t="inlineStr">
         <is>
@@ -18596,7 +18596,7 @@
         </is>
       </c>
       <c r="G346" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="H346" t="inlineStr">
         <is>
@@ -18634,7 +18634,7 @@
         </is>
       </c>
       <c r="G347" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H347" t="inlineStr">
         <is>
@@ -18672,7 +18672,7 @@
         </is>
       </c>
       <c r="G348" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H348" t="inlineStr">
         <is>
@@ -18710,7 +18710,7 @@
         </is>
       </c>
       <c r="G349" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H349" t="inlineStr">
         <is>
@@ -18748,7 +18748,7 @@
         </is>
       </c>
       <c r="G350" t="n">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="H350" t="inlineStr">
         <is>
@@ -18786,7 +18786,7 @@
         </is>
       </c>
       <c r="G351" t="n">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="H351" t="inlineStr">
         <is>
@@ -18824,7 +18824,7 @@
         </is>
       </c>
       <c r="G352" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H352" t="inlineStr">
         <is>
@@ -18862,7 +18862,7 @@
         </is>
       </c>
       <c r="G353" t="n">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H353" t="inlineStr">
         <is>
@@ -18900,7 +18900,7 @@
         </is>
       </c>
       <c r="G354" t="n">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="H354" t="inlineStr">
         <is>
@@ -18938,7 +18938,7 @@
         </is>
       </c>
       <c r="G355" t="n">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="H355" t="inlineStr">
         <is>
@@ -18976,7 +18976,7 @@
         </is>
       </c>
       <c r="G356" t="n">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H356" t="inlineStr">
         <is>
@@ -19014,7 +19014,7 @@
         </is>
       </c>
       <c r="G357" t="n">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H357" t="inlineStr">
         <is>
@@ -19052,7 +19052,7 @@
         </is>
       </c>
       <c r="G358" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="H358" t="inlineStr">
         <is>
@@ -19090,7 +19090,7 @@
         </is>
       </c>
       <c r="G359" t="n">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H359" t="inlineStr">
         <is>
@@ -19128,7 +19128,7 @@
         </is>
       </c>
       <c r="G360" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="H360" t="inlineStr">
         <is>
@@ -19166,7 +19166,7 @@
         </is>
       </c>
       <c r="G361" t="n">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H361" t="inlineStr">
         <is>
@@ -19204,7 +19204,7 @@
         </is>
       </c>
       <c r="G362" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H362" t="inlineStr">
         <is>
@@ -19242,7 +19242,7 @@
         </is>
       </c>
       <c r="G363" t="n">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H363" t="inlineStr">
         <is>
@@ -19280,7 +19280,7 @@
         </is>
       </c>
       <c r="G364" t="n">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H364" t="inlineStr">
         <is>
@@ -19318,7 +19318,7 @@
         </is>
       </c>
       <c r="G365" t="n">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="H365" t="inlineStr">
         <is>
@@ -19356,7 +19356,7 @@
         </is>
       </c>
       <c r="G366" t="n">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="H366" t="inlineStr">
         <is>
@@ -19394,7 +19394,7 @@
         </is>
       </c>
       <c r="G367" t="n">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="H367" t="inlineStr">
         <is>
@@ -19432,7 +19432,7 @@
         </is>
       </c>
       <c r="G368" t="n">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H368" t="inlineStr">
         <is>
@@ -19470,7 +19470,7 @@
         </is>
       </c>
       <c r="G369" t="n">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="H369" t="inlineStr">
         <is>
@@ -19508,7 +19508,7 @@
         </is>
       </c>
       <c r="G370" t="n">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H370" t="inlineStr">
         <is>
@@ -19546,7 +19546,7 @@
         </is>
       </c>
       <c r="G371" t="n">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="H371" t="inlineStr">
         <is>
@@ -19584,7 +19584,7 @@
         </is>
       </c>
       <c r="G372" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H372" t="inlineStr">
         <is>
@@ -19622,7 +19622,7 @@
         </is>
       </c>
       <c r="G373" t="n">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="H373" t="inlineStr">
         <is>
@@ -19660,7 +19660,7 @@
         </is>
       </c>
       <c r="G374" t="n">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="H374" t="inlineStr">
         <is>
@@ -19698,7 +19698,7 @@
         </is>
       </c>
       <c r="G375" t="n">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H375" t="inlineStr">
         <is>
@@ -19736,7 +19736,7 @@
         </is>
       </c>
       <c r="G376" t="n">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="H376" t="inlineStr">
         <is>
@@ -19774,7 +19774,7 @@
         </is>
       </c>
       <c r="G377" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H377" t="inlineStr">
         <is>
@@ -19812,7 +19812,7 @@
         </is>
       </c>
       <c r="G378" t="n">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H378" t="inlineStr">
         <is>
@@ -19850,7 +19850,7 @@
         </is>
       </c>
       <c r="G379" t="n">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H379" t="inlineStr">
         <is>
@@ -19888,7 +19888,7 @@
         </is>
       </c>
       <c r="G380" t="n">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="H380" t="inlineStr">
         <is>
@@ -19926,7 +19926,7 @@
         </is>
       </c>
       <c r="G381" t="n">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="H381" t="inlineStr">
         <is>
@@ -19964,7 +19964,7 @@
         </is>
       </c>
       <c r="G382" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H382" t="inlineStr">
         <is>
@@ -20002,7 +20002,7 @@
         </is>
       </c>
       <c r="G383" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H383" t="inlineStr">
         <is>
@@ -20040,7 +20040,7 @@
         </is>
       </c>
       <c r="G384" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H384" t="inlineStr">
         <is>
@@ -20078,7 +20078,7 @@
         </is>
       </c>
       <c r="G385" t="n">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="H385" t="inlineStr">
         <is>
@@ -20116,7 +20116,7 @@
         </is>
       </c>
       <c r="G386" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="H386" t="inlineStr">
         <is>
@@ -20154,7 +20154,7 @@
         </is>
       </c>
       <c r="G387" t="n">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="H387" t="inlineStr">
         <is>
@@ -20192,7 +20192,7 @@
         </is>
       </c>
       <c r="G388" t="n">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="H388" t="inlineStr">
         <is>
@@ -20230,7 +20230,7 @@
         </is>
       </c>
       <c r="G389" t="n">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H389" t="inlineStr">
         <is>
@@ -20268,7 +20268,7 @@
         </is>
       </c>
       <c r="G390" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H390" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Atualizacao de dados: Thu 10/22/2026 10:38:49.87
</commit_message>
<xml_diff>
--- a/dados.xlsx
+++ b/dados.xlsx
@@ -885,10 +885,10 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>10425.63</v>
+        <v>10412.7</v>
       </c>
       <c r="O8" t="n">
-        <v>2485.41</v>
+        <v>2498.34</v>
       </c>
     </row>
     <row r="9">
@@ -3309,8 +3309,16 @@
       <c r="H58" t="n">
         <v>12.89</v>
       </c>
-      <c r="I58" t="inlineStr"/>
-      <c r="J58" t="inlineStr"/>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>12,93</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>FEITO</t>
+        </is>
+      </c>
       <c r="K58" t="inlineStr">
         <is>
           <t>FEITO</t>
@@ -20465,7 +20473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H85"/>
+  <dimension ref="A1:H86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21669,12 +21677,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>306470</t>
+          <t>306366</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>SÍTIO SÃO PAULO</t>
+          <t>SITIO SANTA CLARA I</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -21683,16 +21691,16 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>9.99</v>
+        <v>12.93</v>
       </c>
       <c r="E36" t="n">
-        <v>130465.54</v>
+        <v>167706.74</v>
       </c>
       <c r="F36" t="n">
-        <v>1472.8</v>
+        <v>96.59999999999999</v>
       </c>
       <c r="G36" t="n">
-        <v>1.13</v>
+        <v>0.06</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
@@ -21703,12 +21711,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>306642</t>
+          <t>306470</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>SITIO TUPINIQUINS</t>
+          <t>SÍTIO SÃO PAULO</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -21717,16 +21725,16 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>49.28</v>
+        <v>9.99</v>
       </c>
       <c r="E37" t="n">
-        <v>645654.6900000001</v>
+        <v>130465.54</v>
       </c>
       <c r="F37" t="n">
-        <v>14333</v>
+        <v>1472.8</v>
       </c>
       <c r="G37" t="n">
-        <v>2.22</v>
+        <v>1.13</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
@@ -21737,12 +21745,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>306756</t>
+          <t>306642</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>SITIO SANTO ANTONIO</t>
+          <t>SITIO TUPINIQUINS</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -21751,16 +21759,16 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>23.14</v>
+        <v>49.28</v>
       </c>
       <c r="E38" t="n">
-        <v>306478.99</v>
+        <v>645654.6900000001</v>
       </c>
       <c r="F38" t="n">
-        <v>1023.4</v>
+        <v>14333</v>
       </c>
       <c r="G38" t="n">
-        <v>0.33</v>
+        <v>2.22</v>
       </c>
       <c r="H38" t="inlineStr">
         <is>
@@ -21771,12 +21779,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>306757</t>
+          <t>306756</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>SÍTIO SÃO FRANCISCO -</t>
+          <t>SITIO SANTO ANTONIO</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -21785,16 +21793,16 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>29.87</v>
+        <v>23.14</v>
       </c>
       <c r="E39" t="n">
-        <v>395707.74</v>
+        <v>306478.99</v>
       </c>
       <c r="F39" t="n">
-        <v>4598</v>
+        <v>1023.4</v>
       </c>
       <c r="G39" t="n">
-        <v>1.16</v>
+        <v>0.33</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
@@ -21805,12 +21813,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>306771</t>
+          <t>306757</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>SÍTIO NOSSA SENHORA APARECIDA</t>
+          <t>SÍTIO SÃO FRANCISCO -</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -21819,16 +21827,16 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>5.83</v>
+        <v>29.87</v>
       </c>
       <c r="E40" t="n">
-        <v>79926.32000000001</v>
+        <v>395707.74</v>
       </c>
       <c r="F40" t="n">
-        <v>431</v>
+        <v>4598</v>
       </c>
       <c r="G40" t="n">
-        <v>0.54</v>
+        <v>1.16</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
@@ -21839,12 +21847,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>306775</t>
+          <t>306771</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>SÍTIO SÃO MIGUEL -</t>
+          <t>SÍTIO NOSSA SENHORA APARECIDA</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -21853,16 +21861,16 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>22.88</v>
+        <v>5.83</v>
       </c>
       <c r="E41" t="n">
-        <v>311793.69</v>
+        <v>79926.32000000001</v>
       </c>
       <c r="F41" t="n">
-        <v>1598.8</v>
+        <v>431</v>
       </c>
       <c r="G41" t="n">
-        <v>0.51</v>
+        <v>0.54</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
@@ -21873,12 +21881,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>306781</t>
+          <t>306775</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>SÍTIO SÃO MIGUEL -</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -21887,16 +21895,16 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>24.94</v>
+        <v>22.88</v>
       </c>
       <c r="E42" t="n">
-        <v>322183.93</v>
+        <v>311793.69</v>
       </c>
       <c r="F42" t="n">
-        <v>8958.6</v>
+        <v>1598.8</v>
       </c>
       <c r="G42" t="n">
-        <v>2.78</v>
+        <v>0.51</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
@@ -21907,12 +21915,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>306783</t>
+          <t>306781</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>SITIO SÃO JOSÉ</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -21921,16 +21929,16 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>20.31</v>
+        <v>24.94</v>
       </c>
       <c r="E43" t="n">
-        <v>269107.21</v>
+        <v>322183.93</v>
       </c>
       <c r="F43" t="n">
-        <v>321.4</v>
+        <v>8958.6</v>
       </c>
       <c r="G43" t="n">
-        <v>0.12</v>
+        <v>2.78</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
@@ -21941,12 +21949,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>306829</t>
+          <t>306783</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>FAZENDA SÃO JOÃO T 12-1</t>
+          <t>SITIO SÃO JOSÉ</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -21955,16 +21963,16 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>208.12</v>
+        <v>20.31</v>
       </c>
       <c r="E44" t="n">
-        <v>3851022.33</v>
+        <v>269107.21</v>
       </c>
       <c r="F44" t="n">
-        <v>100609.7</v>
+        <v>321.4</v>
       </c>
       <c r="G44" t="n">
-        <v>2.61</v>
+        <v>0.12</v>
       </c>
       <c r="H44" t="inlineStr">
         <is>
@@ -21975,12 +21983,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>306893</t>
+          <t>306829</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>SÍTIO NOSSA SENHORA DAS GRAÇAS 1-09-26</t>
+          <t>FAZENDA SÃO JOÃO T 12-1</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -21989,16 +21997,16 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>9.69</v>
+        <v>208.12</v>
       </c>
       <c r="E45" t="n">
-        <v>128624.2</v>
+        <v>3851022.33</v>
       </c>
       <c r="F45" t="n">
-        <v>264</v>
+        <v>100609.7</v>
       </c>
       <c r="G45" t="n">
-        <v>0.21</v>
+        <v>2.61</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>
@@ -22009,12 +22017,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>306901</t>
+          <t>306893</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>SÍTIO SÃO JOÃO</t>
+          <t>SÍTIO NOSSA SENHORA DAS GRAÇAS 1-09-26</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -22023,16 +22031,16 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>32.53</v>
+        <v>9.69</v>
       </c>
       <c r="E46" t="n">
-        <v>424524.16</v>
+        <v>128624.2</v>
       </c>
       <c r="F46" t="n">
-        <v>661.1999999999999</v>
+        <v>264</v>
       </c>
       <c r="G46" t="n">
-        <v>0.16</v>
+        <v>0.21</v>
       </c>
       <c r="H46" t="inlineStr">
         <is>
@@ -22043,12 +22051,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>306954</t>
+          <t>306901</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>FAZENDA NOVA ERA</t>
+          <t>SÍTIO SÃO JOÃO</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -22057,32 +22065,32 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>44.76</v>
+        <v>32.53</v>
       </c>
       <c r="E47" t="n">
-        <v>586776.22</v>
+        <v>424524.16</v>
       </c>
       <c r="F47" t="n">
-        <v>43109.4</v>
+        <v>661.1999999999999</v>
       </c>
       <c r="G47" t="n">
-        <v>7.35</v>
+        <v>0.16</v>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>Atenção</t>
+          <t>Aceitável</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>307057</t>
+          <t>306954</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>SÍTIO SÃO PEDRO</t>
+          <t>FAZENDA NOVA ERA</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -22091,32 +22099,32 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>20.85</v>
+        <v>44.76</v>
       </c>
       <c r="E48" t="n">
-        <v>276816.45</v>
+        <v>586776.22</v>
       </c>
       <c r="F48" t="n">
-        <v>1518</v>
+        <v>43109.4</v>
       </c>
       <c r="G48" t="n">
-        <v>0.55</v>
+        <v>7.35</v>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>Aceitável</t>
+          <t>Atenção</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>307116</t>
+          <t>307057</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>FAZENDA SÃO BRAZ</t>
+          <t>SÍTIO SÃO PEDRO</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -22125,16 +22133,16 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>59.52</v>
+        <v>20.85</v>
       </c>
       <c r="E49" t="n">
-        <v>789718.1000000001</v>
+        <v>276816.45</v>
       </c>
       <c r="F49" t="n">
-        <v>4555.2</v>
+        <v>1518</v>
       </c>
       <c r="G49" t="n">
-        <v>0.58</v>
+        <v>0.55</v>
       </c>
       <c r="H49" t="inlineStr">
         <is>
@@ -22145,12 +22153,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>307491</t>
+          <t>307116</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>SÍTIO SÃO LONGUINHO</t>
+          <t>FAZENDA SÃO BRAZ</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -22159,32 +22167,32 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>21.69</v>
+        <v>59.52</v>
       </c>
       <c r="E50" t="n">
-        <v>273400.37</v>
+        <v>789718.1000000001</v>
       </c>
       <c r="F50" t="n">
-        <v>33101.8</v>
+        <v>4555.2</v>
       </c>
       <c r="G50" t="n">
-        <v>12.11</v>
+        <v>0.58</v>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>Crítico</t>
+          <t>Aceitável</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>307559</t>
+          <t>307491</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>SITIO LOPES</t>
+          <t>SÍTIO SÃO LONGUINHO</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -22193,32 +22201,32 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>49.34</v>
+        <v>21.69</v>
       </c>
       <c r="E51" t="n">
-        <v>634158.7</v>
+        <v>273400.37</v>
       </c>
       <c r="F51" t="n">
-        <v>1280.2</v>
+        <v>33101.8</v>
       </c>
       <c r="G51" t="n">
-        <v>0.2</v>
+        <v>12.11</v>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>Aceitável</t>
+          <t>Crítico</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>307615</t>
+          <t>307559</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>FAZENDA PAU D'ALHO</t>
+          <t>SITIO LOPES</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -22227,16 +22235,16 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>82.54000000000001</v>
+        <v>49.34</v>
       </c>
       <c r="E52" t="n">
-        <v>1033334.75</v>
+        <v>634158.7</v>
       </c>
       <c r="F52" t="n">
-        <v>37193</v>
+        <v>1280.2</v>
       </c>
       <c r="G52" t="n">
-        <v>3.6</v>
+        <v>0.2</v>
       </c>
       <c r="H52" t="inlineStr">
         <is>
@@ -22247,12 +22255,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>307637</t>
+          <t>307615</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>FAZ SANTO ANTONIO II</t>
+          <t>FAZENDA PAU D'ALHO</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -22261,32 +22269,32 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>202.72</v>
+        <v>82.54000000000001</v>
       </c>
       <c r="E53" t="n">
-        <v>2701760.93</v>
+        <v>1033334.75</v>
       </c>
       <c r="F53" t="n">
-        <v>145949.4</v>
+        <v>37193</v>
       </c>
       <c r="G53" t="n">
-        <v>5.4</v>
+        <v>3.6</v>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>Atenção</t>
+          <t>Aceitável</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>307658</t>
+          <t>307637</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>SÍTIO IRMÃOS ANNELLI -</t>
+          <t>FAZ SANTO ANTONIO II</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -22295,32 +22303,32 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>13.46</v>
+        <v>202.72</v>
       </c>
       <c r="E54" t="n">
-        <v>173572.58</v>
+        <v>2701760.93</v>
       </c>
       <c r="F54" t="n">
-        <v>2156</v>
+        <v>145949.4</v>
       </c>
       <c r="G54" t="n">
-        <v>1.24</v>
+        <v>5.4</v>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>Aceitável</t>
+          <t>Atenção</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>307770</t>
+          <t>307658</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>FAZENDA SANTA ELIZA</t>
+          <t>SÍTIO IRMÃOS ANNELLI -</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -22329,16 +22337,16 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>13.47</v>
+        <v>13.46</v>
       </c>
       <c r="E55" t="n">
-        <v>178895.5</v>
+        <v>173572.58</v>
       </c>
       <c r="F55" t="n">
-        <v>5256</v>
+        <v>2156</v>
       </c>
       <c r="G55" t="n">
-        <v>2.94</v>
+        <v>1.24</v>
       </c>
       <c r="H55" t="inlineStr">
         <is>
@@ -22349,12 +22357,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>307799</t>
+          <t>307770</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>SÍTIO TREZE DE MAIO</t>
+          <t>FAZENDA SANTA ELIZA</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -22363,27 +22371,27 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>46.17</v>
+        <v>13.47</v>
       </c>
       <c r="E56" t="n">
-        <v>376072.8099999999</v>
+        <v>178895.5</v>
       </c>
       <c r="F56" t="n">
-        <v>27264</v>
+        <v>5256</v>
       </c>
       <c r="G56" t="n">
-        <v>7.25</v>
+        <v>2.94</v>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>Atenção</t>
+          <t>Aceitável</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>307802</t>
+          <t>307799</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -22397,32 +22405,32 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>12.21</v>
+        <v>46.17</v>
       </c>
       <c r="E57" t="n">
-        <v>98076.84</v>
+        <v>376072.8099999999</v>
       </c>
       <c r="F57" t="n">
-        <v>1283.8</v>
+        <v>27264</v>
       </c>
       <c r="G57" t="n">
-        <v>1.31</v>
+        <v>7.25</v>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>Aceitável</t>
+          <t>Atenção</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>307837</t>
+          <t>307802</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>SÍTIO VOLTA GRANDE</t>
+          <t>SÍTIO TREZE DE MAIO</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -22431,16 +22439,16 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>34.78</v>
+        <v>12.21</v>
       </c>
       <c r="E58" t="n">
-        <v>476042.0399999999</v>
+        <v>98076.84</v>
       </c>
       <c r="F58" t="n">
-        <v>3186.4</v>
+        <v>1283.8</v>
       </c>
       <c r="G58" t="n">
-        <v>0.67</v>
+        <v>1.31</v>
       </c>
       <c r="H58" t="inlineStr">
         <is>
@@ -22451,12 +22459,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>307886</t>
+          <t>307837</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>SITIO SANTO ANTONIO</t>
+          <t>SÍTIO VOLTA GRANDE</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -22465,16 +22473,16 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>12.46</v>
+        <v>34.78</v>
       </c>
       <c r="E59" t="n">
-        <v>168355.53</v>
+        <v>476042.0399999999</v>
       </c>
       <c r="F59" t="n">
-        <v>4152.2</v>
+        <v>3186.4</v>
       </c>
       <c r="G59" t="n">
-        <v>2.47</v>
+        <v>0.67</v>
       </c>
       <c r="H59" t="inlineStr">
         <is>
@@ -22485,12 +22493,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>307943</t>
+          <t>307886</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>FAZ SILVANIA</t>
+          <t>SITIO SANTO ANTONIO</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -22499,16 +22507,16 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>32.58</v>
+        <v>12.46</v>
       </c>
       <c r="E60" t="n">
-        <v>440087.89</v>
+        <v>168355.53</v>
       </c>
       <c r="F60" t="n">
-        <v>1628.6</v>
+        <v>4152.2</v>
       </c>
       <c r="G60" t="n">
-        <v>0.37</v>
+        <v>2.47</v>
       </c>
       <c r="H60" t="inlineStr">
         <is>
@@ -22519,12 +22527,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>307980</t>
+          <t>307943</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>FAZENDA UNIÃO</t>
+          <t>FAZ SILVANIA</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -22533,16 +22541,16 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>38.01</v>
+        <v>32.58</v>
       </c>
       <c r="E61" t="n">
-        <v>522084.7599999999</v>
+        <v>440087.89</v>
       </c>
       <c r="F61" t="n">
-        <v>2870.599999999999</v>
+        <v>1628.6</v>
       </c>
       <c r="G61" t="n">
-        <v>0.55</v>
+        <v>0.37</v>
       </c>
       <c r="H61" t="inlineStr">
         <is>
@@ -22553,12 +22561,12 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>308080</t>
+          <t>307980</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>FAZENDA BARREIRÃO</t>
+          <t>FAZENDA UNIÃO</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -22567,16 +22575,16 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>215.38</v>
+        <v>38.01</v>
       </c>
       <c r="E62" t="n">
-        <v>2815276.559999999</v>
+        <v>522084.7599999999</v>
       </c>
       <c r="F62" t="n">
-        <v>39949.8</v>
+        <v>2870.599999999999</v>
       </c>
       <c r="G62" t="n">
-        <v>1.42</v>
+        <v>0.55</v>
       </c>
       <c r="H62" t="inlineStr">
         <is>
@@ -22587,12 +22595,12 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>308087</t>
+          <t>308080</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>FAZENDA NOSSA SENHORA APARECIDA</t>
+          <t>FAZENDA BARREIRÃO</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -22601,16 +22609,16 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>84.54000000000001</v>
+        <v>215.38</v>
       </c>
       <c r="E63" t="n">
-        <v>1121963.9</v>
+        <v>2815276.559999999</v>
       </c>
       <c r="F63" t="n">
-        <v>5588.2</v>
+        <v>39949.8</v>
       </c>
       <c r="G63" t="n">
-        <v>0.5</v>
+        <v>1.42</v>
       </c>
       <c r="H63" t="inlineStr">
         <is>
@@ -22621,12 +22629,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>308096</t>
+          <t>308087</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>SÍTIO TAKATA</t>
+          <t>FAZENDA NOSSA SENHORA APARECIDA</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -22635,16 +22643,16 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>46.86</v>
+        <v>84.54000000000001</v>
       </c>
       <c r="E64" t="n">
-        <v>776146.4500000001</v>
+        <v>1121963.9</v>
       </c>
       <c r="F64" t="n">
-        <v>1653.8</v>
+        <v>5588.2</v>
       </c>
       <c r="G64" t="n">
-        <v>0.21</v>
+        <v>0.5</v>
       </c>
       <c r="H64" t="inlineStr">
         <is>
@@ -22655,12 +22663,12 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>308098</t>
+          <t>308096</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>SÍTIO SANTA MARCELINA - 301274 - SÍTIO LIMEIRA</t>
+          <t>SÍTIO TAKATA</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -22669,16 +22677,16 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>45.53</v>
+        <v>46.86</v>
       </c>
       <c r="E65" t="n">
-        <v>585824.86</v>
+        <v>776146.4500000001</v>
       </c>
       <c r="F65" t="n">
-        <v>1500</v>
+        <v>1653.8</v>
       </c>
       <c r="G65" t="n">
-        <v>0.26</v>
+        <v>0.21</v>
       </c>
       <c r="H65" t="inlineStr">
         <is>
@@ -22689,12 +22697,12 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>308112</t>
+          <t>308098</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>SÍTIO UNIÃO</t>
+          <t>SÍTIO SANTA MARCELINA - 301274 - SÍTIO LIMEIRA</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -22703,16 +22711,16 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>27.59</v>
+        <v>45.53</v>
       </c>
       <c r="E66" t="n">
-        <v>367038.91</v>
+        <v>585824.86</v>
       </c>
       <c r="F66" t="n">
-        <v>1515</v>
+        <v>1500</v>
       </c>
       <c r="G66" t="n">
-        <v>0.41</v>
+        <v>0.26</v>
       </c>
       <c r="H66" t="inlineStr">
         <is>
@@ -22723,12 +22731,12 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>308120</t>
+          <t>308112</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>ESTÂNCIA PRIMAVERA</t>
+          <t>SÍTIO UNIÃO</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -22737,16 +22745,16 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>10.06</v>
+        <v>27.59</v>
       </c>
       <c r="E67" t="n">
-        <v>135639.5</v>
+        <v>367038.91</v>
       </c>
       <c r="F67" t="n">
-        <v>508.4000000000001</v>
+        <v>1515</v>
       </c>
       <c r="G67" t="n">
-        <v>0.37</v>
+        <v>0.41</v>
       </c>
       <c r="H67" t="inlineStr">
         <is>
@@ -22757,12 +22765,12 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>308123</t>
+          <t>308120</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>SÍTIO SANTO ANTÔNIO</t>
+          <t>ESTÂNCIA PRIMAVERA</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -22771,16 +22779,16 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>33.25</v>
+        <v>10.06</v>
       </c>
       <c r="E68" t="n">
-        <v>448944.35</v>
+        <v>135639.5</v>
       </c>
       <c r="F68" t="n">
-        <v>5004.799999999999</v>
+        <v>508.4000000000001</v>
       </c>
       <c r="G68" t="n">
-        <v>1.11</v>
+        <v>0.37</v>
       </c>
       <c r="H68" t="inlineStr">
         <is>
@@ -22791,12 +22799,12 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>308152</t>
+          <t>308123</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>FAZENDA SÃO JOÃO DA BARRA</t>
+          <t>SÍTIO SANTO ANTÔNIO</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -22805,16 +22813,16 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>190.43</v>
+        <v>33.25</v>
       </c>
       <c r="E69" t="n">
-        <v>2511618.14</v>
+        <v>448944.35</v>
       </c>
       <c r="F69" t="n">
-        <v>72840.20000000001</v>
+        <v>5004.799999999999</v>
       </c>
       <c r="G69" t="n">
-        <v>2.9</v>
+        <v>1.11</v>
       </c>
       <c r="H69" t="inlineStr">
         <is>
@@ -22825,12 +22833,12 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>308186</t>
+          <t>308152</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>FAZENDA SANTA RITA</t>
+          <t>FAZENDA SÃO JOÃO DA BARRA</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -22839,16 +22847,16 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>98.25</v>
+        <v>190.43</v>
       </c>
       <c r="E70" t="n">
-        <v>1287741.67</v>
+        <v>2511618.14</v>
       </c>
       <c r="F70" t="n">
-        <v>13637.4</v>
+        <v>72840.20000000001</v>
       </c>
       <c r="G70" t="n">
-        <v>1.06</v>
+        <v>2.9</v>
       </c>
       <c r="H70" t="inlineStr">
         <is>
@@ -22859,12 +22867,12 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>308193</t>
+          <t>308186</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>SITIO IRMÃOS FERNANDES</t>
+          <t>FAZENDA SANTA RITA</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -22873,16 +22881,16 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>19.14</v>
+        <v>98.25</v>
       </c>
       <c r="E71" t="n">
-        <v>236647.12</v>
+        <v>1287741.67</v>
       </c>
       <c r="F71" t="n">
-        <v>9806</v>
+        <v>13637.4</v>
       </c>
       <c r="G71" t="n">
-        <v>4.14</v>
+        <v>1.06</v>
       </c>
       <c r="H71" t="inlineStr">
         <is>
@@ -22893,12 +22901,12 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>308214</t>
+          <t>308193</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>ESTANCIA DYMONT</t>
+          <t>SITIO IRMÃOS FERNANDES</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -22907,16 +22915,16 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>14.33</v>
+        <v>19.14</v>
       </c>
       <c r="E72" t="n">
-        <v>201117.62</v>
+        <v>236647.12</v>
       </c>
       <c r="F72" t="n">
-        <v>150.4</v>
+        <v>9806</v>
       </c>
       <c r="G72" t="n">
-        <v>0.07000000000000001</v>
+        <v>4.14</v>
       </c>
       <c r="H72" t="inlineStr">
         <is>
@@ -22927,12 +22935,12 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>308225</t>
+          <t>308214</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>SITIO BOM JESUS</t>
+          <t>ESTANCIA DYMONT</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -22941,16 +22949,16 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>42.9</v>
+        <v>14.33</v>
       </c>
       <c r="E73" t="n">
-        <v>567803.14</v>
+        <v>201117.62</v>
       </c>
       <c r="F73" t="n">
-        <v>2287.4</v>
+        <v>150.4</v>
       </c>
       <c r="G73" t="n">
-        <v>0.4</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="H73" t="inlineStr">
         <is>
@@ -22961,12 +22969,12 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>308226</t>
+          <t>308225</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>SITIO CAPITAO HONORIO</t>
+          <t>SITIO BOM JESUS</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -22975,16 +22983,16 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>43.04</v>
+        <v>42.9</v>
       </c>
       <c r="E74" t="n">
-        <v>593292.2899999999</v>
+        <v>567803.14</v>
       </c>
       <c r="F74" t="n">
-        <v>2039.4</v>
+        <v>2287.4</v>
       </c>
       <c r="G74" t="n">
-        <v>0.34</v>
+        <v>0.4</v>
       </c>
       <c r="H74" t="inlineStr">
         <is>
@@ -22995,12 +23003,12 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>308231</t>
+          <t>308226</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>SITIO SÃO FRANCISCO - 30310- SITIO SANTA HELENA</t>
+          <t>SITIO CAPITAO HONORIO</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -23009,16 +23017,16 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>15.89</v>
+        <v>43.04</v>
       </c>
       <c r="E75" t="n">
-        <v>221144.51</v>
+        <v>593292.2899999999</v>
       </c>
       <c r="F75" t="n">
-        <v>633.4000000000001</v>
+        <v>2039.4</v>
       </c>
       <c r="G75" t="n">
-        <v>0.29</v>
+        <v>0.34</v>
       </c>
       <c r="H75" t="inlineStr">
         <is>
@@ -23029,12 +23037,12 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>308233</t>
+          <t>308231</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>SITIO SÃO JOSÉ PEROLA</t>
+          <t>SITIO SÃO FRANCISCO - 30310- SITIO SANTA HELENA</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -23043,16 +23051,16 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>12.48</v>
+        <v>15.89</v>
       </c>
       <c r="E76" t="n">
-        <v>166148.27</v>
+        <v>221144.51</v>
       </c>
       <c r="F76" t="n">
-        <v>531.4</v>
+        <v>633.4000000000001</v>
       </c>
       <c r="G76" t="n">
-        <v>0.32</v>
+        <v>0.29</v>
       </c>
       <c r="H76" t="inlineStr">
         <is>
@@ -23063,12 +23071,12 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>308238</t>
+          <t>308233</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>FAZ VALE DO SOL</t>
+          <t>SITIO SÃO JOSÉ PEROLA</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -23077,16 +23085,16 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>54.12</v>
+        <v>12.48</v>
       </c>
       <c r="E77" t="n">
-        <v>699691.55</v>
+        <v>166148.27</v>
       </c>
       <c r="F77" t="n">
-        <v>6555.2</v>
+        <v>531.4</v>
       </c>
       <c r="G77" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.32</v>
       </c>
       <c r="H77" t="inlineStr">
         <is>
@@ -23097,12 +23105,12 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>308239</t>
+          <t>308238</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>SITIO METODIO III</t>
+          <t>FAZ VALE DO SOL</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -23111,16 +23119,16 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>168.43</v>
+        <v>54.12</v>
       </c>
       <c r="E78" t="n">
-        <v>0</v>
+        <v>699691.55</v>
       </c>
       <c r="F78" t="n">
-        <v>0</v>
+        <v>6555.2</v>
       </c>
       <c r="G78" t="n">
-        <v>0</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="H78" t="inlineStr">
         <is>
@@ -23131,12 +23139,12 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>308247</t>
+          <t>308239</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>SITIO BOA VISTA</t>
+          <t>SITIO METODIO III</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -23145,16 +23153,16 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>51.26</v>
+        <v>168.43</v>
       </c>
       <c r="E79" t="n">
-        <v>669737.62</v>
+        <v>0</v>
       </c>
       <c r="F79" t="n">
-        <v>2331</v>
+        <v>0</v>
       </c>
       <c r="G79" t="n">
-        <v>0.35</v>
+        <v>0</v>
       </c>
       <c r="H79" t="inlineStr">
         <is>
@@ -23165,12 +23173,12 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>308248</t>
+          <t>308247</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>SITIO 3DJ</t>
+          <t>SITIO BOA VISTA</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -23179,16 +23187,16 @@
         </is>
       </c>
       <c r="D80" t="n">
-        <v>18.01</v>
+        <v>51.26</v>
       </c>
       <c r="E80" t="n">
-        <v>215580.29</v>
+        <v>669737.62</v>
       </c>
       <c r="F80" t="n">
-        <v>4613.4</v>
+        <v>2331</v>
       </c>
       <c r="G80" t="n">
-        <v>2.14</v>
+        <v>0.35</v>
       </c>
       <c r="H80" t="inlineStr">
         <is>
@@ -23199,12 +23207,12 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>308261</t>
+          <t>308248</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>FAZ RIO FEIO</t>
+          <t>SITIO 3DJ</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -23213,16 +23221,16 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>41.97</v>
+        <v>18.01</v>
       </c>
       <c r="E81" t="n">
-        <v>555218.6199999999</v>
+        <v>215580.29</v>
       </c>
       <c r="F81" t="n">
-        <v>27273.4</v>
+        <v>4613.4</v>
       </c>
       <c r="G81" t="n">
-        <v>4.91</v>
+        <v>2.14</v>
       </c>
       <c r="H81" t="inlineStr">
         <is>
@@ -23233,12 +23241,12 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>308268</t>
+          <t>308261</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>SITIO SÃO JOSE</t>
+          <t>FAZ RIO FEIO</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -23247,16 +23255,16 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>30.22</v>
+        <v>41.97</v>
       </c>
       <c r="E82" t="n">
-        <v>401557.88</v>
+        <v>555218.6199999999</v>
       </c>
       <c r="F82" t="n">
-        <v>1984.8</v>
+        <v>27273.4</v>
       </c>
       <c r="G82" t="n">
-        <v>0.49</v>
+        <v>4.91</v>
       </c>
       <c r="H82" t="inlineStr">
         <is>
@@ -23267,12 +23275,12 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>308269</t>
+          <t>308268</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>FAZENDA SANTA CECILIA</t>
+          <t>SITIO SÃO JOSE</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -23281,16 +23289,16 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>55.4</v>
+        <v>30.22</v>
       </c>
       <c r="E83" t="n">
-        <v>735048.67</v>
+        <v>401557.88</v>
       </c>
       <c r="F83" t="n">
-        <v>2871.400000000001</v>
+        <v>1984.8</v>
       </c>
       <c r="G83" t="n">
-        <v>0.39</v>
+        <v>0.49</v>
       </c>
       <c r="H83" t="inlineStr">
         <is>
@@ -23301,12 +23309,12 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>comparativo_kml_vs_banco_falhas</t>
+          <t>308269</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>FAZENDA SANTA CECILIA</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -23315,16 +23323,16 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>0</v>
+        <v>55.4</v>
       </c>
       <c r="E84" t="n">
-        <v>0</v>
+        <v>735048.67</v>
       </c>
       <c r="F84" t="n">
-        <v>0</v>
+        <v>2871.400000000001</v>
       </c>
       <c r="G84" t="n">
-        <v>0</v>
+        <v>0.39</v>
       </c>
       <c r="H84" t="inlineStr">
         <is>
@@ -23335,7 +23343,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>valores_coluna_C_linha_2</t>
+          <t>comparativo_kml_vs_banco_falhas</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -23361,6 +23369,40 @@
         <v>0</v>
       </c>
       <c r="H85" t="inlineStr">
+        <is>
+          <t>Aceitável</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>valores_coluna_C_linha_2</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Terceiro</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>0</v>
+      </c>
+      <c r="E86" t="n">
+        <v>0</v>
+      </c>
+      <c r="F86" t="n">
+        <v>0</v>
+      </c>
+      <c r="G86" t="n">
+        <v>0</v>
+      </c>
+      <c r="H86" t="inlineStr">
         <is>
           <t>Aceitável</t>
         </is>

</xml_diff>

<commit_message>
Atualizacao de dados: Thu 10/22/2026 11:46:16.44
</commit_message>
<xml_diff>
--- a/dados.xlsx
+++ b/dados.xlsx
@@ -11,6 +11,8 @@
     <sheet name="BACKLOG" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="FALHAS_PLANTIO" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="METAS_GLOBAIS" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="ACOMPANHAMENTO" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="CONFIG" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23509,4 +23511,516 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Ano</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Categoria</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Segmento</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Realizado</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Semana</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Mes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Voos realizados</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Própria</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>3374.33</v>
+      </c>
+      <c r="E2" t="n">
+        <v>2288.66</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Voos realizados</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Fornecedores</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>11000</v>
+      </c>
+      <c r="E3" t="n">
+        <v>5206.870000000002</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Voos realizados</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Consolidado</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>14374.33</v>
+      </c>
+      <c r="E4" t="n">
+        <v>7495.530000000002</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Mosaico processado</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Própria</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>3374.33</v>
+      </c>
+      <c r="E5" t="n">
+        <v>2288.66</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Mosaico processado</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Fornecedores</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>11000</v>
+      </c>
+      <c r="E6" t="n">
+        <v>5206.870000000002</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Mosaico processado</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Consolidado</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>14374.33</v>
+      </c>
+      <c r="E7" t="n">
+        <v>7495.530000000002</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Falhas no plantio</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Própria</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>3374.33</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1854.19</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Falhas no plantio</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Fornecedores</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>11000</v>
+      </c>
+      <c r="E9" t="n">
+        <v>7151.915000000001</v>
+      </c>
+      <c r="F9" t="n">
+        <v>108.19</v>
+      </c>
+      <c r="G9" t="n">
+        <v>634.3399999999999</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Falhas no plantio</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Consolidado</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>14374.33</v>
+      </c>
+      <c r="E10" t="n">
+        <v>9006.105000000001</v>
+      </c>
+      <c r="F10" t="n">
+        <v>108.19</v>
+      </c>
+      <c r="G10" t="n">
+        <v>634.3399999999999</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Pós plantio</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Própria</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>3374.33</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1816.39</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" t="n">
+        <v>266.71</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Pós plantio</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Fornecedores</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>11000</v>
+      </c>
+      <c r="E12" t="n">
+        <v>5702.75</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" t="n">
+        <v>125.57</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Pós plantio</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Consolidado</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>14374.33</v>
+      </c>
+      <c r="E13" t="n">
+        <v>7519.14</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" t="n">
+        <v>392.28</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Exportação para piloto</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Própria</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>3374.33</v>
+      </c>
+      <c r="E14" t="n">
+        <v>236.26</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Exportação para piloto</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Fornecedores</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>11000</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1634.285</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Exportação para piloto</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Consolidado</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>14374.33</v>
+      </c>
+      <c r="E16" t="n">
+        <v>1870.545</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>creditos_inforow</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>11121.66</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Atualizacao automatica de dados: 22/10/2026 14:47:43.25
</commit_message>
<xml_diff>
--- a/dados.xlsx
+++ b/dados.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="BASE_PROCESSAMENTOS" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="BACKLOG" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="FALHAS_PLANTIO" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="METAS_GLOBAIS" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="ACOMPANHAMENTO" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="CONFIG" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BASE_PROCESSAMENTOS" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BACKLOG" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FALHAS_PLANTIO" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="METAS_GLOBAIS" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ACOMPANHAMENTO" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONFIG" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,9 +21,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -54,9 +53,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -516,8 +516,7 @@
           <t>B-24 CENTRO RURAL</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" s="1" t="n">
+      <c r="E2" s="2" t="n">
         <v>46205</v>
       </c>
       <c r="F2" t="inlineStr">
@@ -541,11 +540,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -566,7 +560,7 @@
           <t>-22° 02´ 13.3421 -50° 07´ 13.5185 491.84</t>
         </is>
       </c>
-      <c r="E3" s="1" t="n">
+      <c r="E3" s="2" t="n">
         <v>46217</v>
       </c>
       <c r="F3" t="inlineStr">
@@ -606,7 +600,6 @@
       <c r="N3" t="n">
         <v>586.49</v>
       </c>
-      <c r="O3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -622,8 +615,7 @@
           <t>B-23 FAZ NOSSA SENHORA APARECIDA</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" s="1" t="n">
+      <c r="E4" s="2" t="n">
         <v>46199</v>
       </c>
       <c r="F4" t="inlineStr">
@@ -663,7 +655,6 @@
       <c r="N4" t="n">
         <v>854.9300000000001</v>
       </c>
-      <c r="O4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -684,7 +675,7 @@
           <t>-21° 39´ 13.2100 -50° 32´ 04.0182 418.26</t>
         </is>
       </c>
-      <c r="E5" s="1" t="n">
+      <c r="E5" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F5" t="inlineStr">
@@ -713,10 +704,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -737,7 +724,7 @@
           <t>-21° 39´ 13.2100 -50° 32´ 04.0182 418.26</t>
         </is>
       </c>
-      <c r="E6" s="1" t="n">
+      <c r="E6" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F6" t="inlineStr">
@@ -766,10 +753,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -790,7 +773,7 @@
           <t>-21° 34´ 46.1049 -50° 26´ 00.0424 442.78</t>
         </is>
       </c>
-      <c r="E7" s="1" t="n">
+      <c r="E7" s="2" t="n">
         <v>46183</v>
       </c>
       <c r="F7" t="inlineStr">
@@ -819,7 +802,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr">
         <is>
           <t xml:space="preserve">PROPRIAS </t>
@@ -851,7 +833,7 @@
           <t>-22° 02´ 13.3421 -50° 07´ 13.5185 491.84</t>
         </is>
       </c>
-      <c r="E8" s="1" t="n">
+      <c r="E8" s="2" t="n">
         <v>46196</v>
       </c>
       <c r="F8" t="inlineStr">
@@ -880,7 +862,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr">
         <is>
           <t>TERCEIROS</t>
@@ -907,8 +888,7 @@
           <t>B-23 FAZ NOSSA SENHORA APARECIDA</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" s="1" t="n">
+      <c r="E9" s="2" t="n">
         <v>46199</v>
       </c>
       <c r="F9" t="inlineStr">
@@ -937,10 +917,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -961,7 +937,7 @@
           <t>-21° 31´ 28.9807 -50° 18´ 16.5320 492.23</t>
         </is>
       </c>
-      <c r="E10" s="1" t="n">
+      <c r="E10" s="2" t="n">
         <v>46211</v>
       </c>
       <c r="F10" t="inlineStr">
@@ -990,10 +966,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1014,7 +986,7 @@
           <t>-21° 39´ 13.2100 -50° 32´ 04.0182 418.26</t>
         </is>
       </c>
-      <c r="E11" s="1" t="n">
+      <c r="E11" s="2" t="n">
         <v>46189</v>
       </c>
       <c r="F11" t="inlineStr">
@@ -1043,10 +1015,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1062,8 +1030,7 @@
           <t>B-24 CENTRO RURAL</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" s="1" t="n">
+      <c r="E12" s="2" t="n">
         <v>46203</v>
       </c>
       <c r="F12" t="inlineStr">
@@ -1092,10 +1059,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1116,7 +1079,7 @@
           <t>-21° 31´ 28.9807 -50° 18´ 16.5320 492.23</t>
         </is>
       </c>
-      <c r="E13" s="1" t="n">
+      <c r="E13" s="2" t="n">
         <v>46185</v>
       </c>
       <c r="F13" t="inlineStr">
@@ -1145,10 +1108,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1169,7 +1128,7 @@
           <t>-21° 31´ 28.9807 -50° 18´ 16.5320 492.23</t>
         </is>
       </c>
-      <c r="E14" s="1" t="n">
+      <c r="E14" s="2" t="n">
         <v>46211</v>
       </c>
       <c r="F14" t="inlineStr">
@@ -1198,10 +1157,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1212,9 +1167,7 @@
           <t>SÍTIO SÃO FRANCISCO -</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" s="1" t="n">
+      <c r="E15" s="2" t="n">
         <v>46185</v>
       </c>
       <c r="F15" t="inlineStr">
@@ -1243,10 +1196,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
-      <c r="O15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1262,8 +1211,7 @@
           <t>B-24 CENTRO RURAL</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" s="1" t="n">
+      <c r="E16" s="2" t="n">
         <v>46203</v>
       </c>
       <c r="F16" t="inlineStr">
@@ -1292,10 +1240,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr"/>
-      <c r="O16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1316,7 +1260,7 @@
           <t>-21° 31´ 28.9807 -50° 18´ 16.5320 492.23</t>
         </is>
       </c>
-      <c r="E17" s="1" t="n">
+      <c r="E17" s="2" t="n">
         <v>46185</v>
       </c>
       <c r="F17" t="inlineStr">
@@ -1345,10 +1289,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr"/>
-      <c r="O17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1369,7 +1309,7 @@
           <t>-21° 35´ 32.3241 -50° 10´ 09.0062 470.03</t>
         </is>
       </c>
-      <c r="E18" s="1" t="n">
+      <c r="E18" s="2" t="n">
         <v>46219</v>
       </c>
       <c r="F18" t="inlineStr">
@@ -1398,10 +1338,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
-      <c r="N18" t="inlineStr"/>
-      <c r="O18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1422,7 +1358,7 @@
           <t>-21° 31´ 28.9807 -50° 18´ 16.5320 492.23</t>
         </is>
       </c>
-      <c r="E19" s="1" t="n">
+      <c r="E19" s="2" t="n">
         <v>46211</v>
       </c>
       <c r="F19" t="inlineStr">
@@ -1451,10 +1387,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1465,9 +1397,7 @@
           <t>SÍTIO IRMÃOS ANNELLI -</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" s="1" t="n">
+      <c r="E20" s="2" t="n">
         <v>46185</v>
       </c>
       <c r="F20" t="inlineStr">
@@ -1496,10 +1426,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1510,9 +1436,7 @@
           <t>SÍTIO TREZE DE MAIO</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" s="1" t="n">
+      <c r="E21" s="2" t="n">
         <v>46205</v>
       </c>
       <c r="F21" t="inlineStr">
@@ -1520,7 +1444,7 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="G21" s="1" t="n">
+      <c r="G21" s="2" t="n">
         <v>46210</v>
       </c>
       <c r="H21" t="n">
@@ -1539,10 +1463,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
-      <c r="N21" t="inlineStr"/>
-      <c r="O21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1563,7 +1483,7 @@
           <t>-21° 39´ 59.2206 -50° 19´ 50.9494 405.70</t>
         </is>
       </c>
-      <c r="E22" s="1" t="n">
+      <c r="E22" s="2" t="n">
         <v>46216</v>
       </c>
       <c r="F22" t="inlineStr">
@@ -1592,10 +1512,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr"/>
-      <c r="O22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1616,7 +1532,7 @@
           <t>-21° 31´ 28.9807 -50° 18´ 16.5320 492.23</t>
         </is>
       </c>
-      <c r="E23" s="1" t="n">
+      <c r="E23" s="2" t="n">
         <v>46211</v>
       </c>
       <c r="F23" t="inlineStr">
@@ -1645,10 +1561,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr"/>
-      <c r="O23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1669,7 +1581,7 @@
           <t>-21° 35´ 32.3241 -50° 10´ 09.0062 470.03</t>
         </is>
       </c>
-      <c r="E24" s="1" t="n">
+      <c r="E24" s="2" t="n">
         <v>46219</v>
       </c>
       <c r="F24" t="inlineStr">
@@ -1698,10 +1610,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr"/>
-      <c r="O24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1722,7 +1630,7 @@
           <t>-21° 35´ 32.3241 -50° 10´ 09.0062 470.03</t>
         </is>
       </c>
-      <c r="E25" s="1" t="n">
+      <c r="E25" s="2" t="n">
         <v>46219</v>
       </c>
       <c r="F25" t="inlineStr">
@@ -1751,10 +1659,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1775,7 +1679,7 @@
           <t>-21° 48´ 26.1814 -50° 13´ 14.2006 438.00</t>
         </is>
       </c>
-      <c r="E26" s="1" t="n">
+      <c r="E26" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="F26" t="inlineStr">
@@ -1804,10 +1708,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1828,7 +1728,7 @@
           <t>-21° 48´ 26.1814 -50° 13´ 14.2006 438.00</t>
         </is>
       </c>
-      <c r="E27" s="1" t="n">
+      <c r="E27" s="2" t="n">
         <v>46239</v>
       </c>
       <c r="F27" t="inlineStr">
@@ -1857,10 +1757,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
-      <c r="O27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1881,7 +1777,7 @@
           <t>-21° 45´ 32.6517 -50° 06´ 02.9557 456.63</t>
         </is>
       </c>
-      <c r="E28" s="1" t="n">
+      <c r="E28" s="2" t="n">
         <v>46240</v>
       </c>
       <c r="F28" t="inlineStr">
@@ -1897,13 +1793,6 @@
       <c r="H28" t="n">
         <v>94.87</v>
       </c>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
-      <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr"/>
-      <c r="O28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1924,7 +1813,7 @@
           <t>-21° 48´ 26.1814 -50° 13´ 14.2006 438.00</t>
         </is>
       </c>
-      <c r="E29" s="1" t="n">
+      <c r="E29" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="F29" t="inlineStr">
@@ -1953,10 +1842,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L29" t="inlineStr"/>
-      <c r="M29" t="inlineStr"/>
-      <c r="N29" t="inlineStr"/>
-      <c r="O29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1977,7 +1862,7 @@
           <t>-21° 39´ 13.2100 -50° 32´ 04.0182 418.26</t>
         </is>
       </c>
-      <c r="E30" s="1" t="n">
+      <c r="E30" s="2" t="n">
         <v>46237</v>
       </c>
       <c r="F30" t="inlineStr">
@@ -1993,13 +1878,6 @@
       <c r="H30" t="n">
         <v>57.73</v>
       </c>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr"/>
-      <c r="M30" t="inlineStr"/>
-      <c r="N30" t="inlineStr"/>
-      <c r="O30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -2020,7 +1898,7 @@
           <t>-21° 48´ 26.1814 -50° 13´ 14.2006 438.00</t>
         </is>
       </c>
-      <c r="E31" s="1" t="n">
+      <c r="E31" s="2" t="n">
         <v>46240</v>
       </c>
       <c r="F31" t="inlineStr">
@@ -2046,11 +1924,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr"/>
-      <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr"/>
-      <c r="O31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -2071,7 +1944,7 @@
           <t>-21° 39´ 13.2100 -50° 32´ 04.0182 418.26</t>
         </is>
       </c>
-      <c r="E32" s="1" t="n">
+      <c r="E32" s="2" t="n">
         <v>46237</v>
       </c>
       <c r="F32" t="inlineStr">
@@ -2095,11 +1968,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr"/>
-      <c r="M32" t="inlineStr"/>
-      <c r="N32" t="inlineStr"/>
-      <c r="O32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -2120,7 +1988,7 @@
           <t>-22° 02´ 13.3421 -50° 07´ 13.5185 491.84</t>
         </is>
       </c>
-      <c r="E33" s="1" t="n">
+      <c r="E33" s="2" t="n">
         <v>46231</v>
       </c>
       <c r="F33" t="inlineStr">
@@ -2136,13 +2004,6 @@
       <c r="H33" t="n">
         <v>95.5</v>
       </c>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr"/>
-      <c r="M33" t="inlineStr"/>
-      <c r="N33" t="inlineStr"/>
-      <c r="O33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -2163,7 +2024,7 @@
           <t>-21° 31´ 28.9807 -50° 18´ 16.5320 492.23</t>
         </is>
       </c>
-      <c r="E34" s="1" t="n">
+      <c r="E34" s="2" t="n">
         <v>46241</v>
       </c>
       <c r="F34" t="inlineStr">
@@ -2192,10 +2053,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L34" t="inlineStr"/>
-      <c r="M34" t="inlineStr"/>
-      <c r="N34" t="inlineStr"/>
-      <c r="O34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -2216,7 +2073,7 @@
           <t>-21° 31´ 28.9807 -50° 18´ 16.5320 492.23</t>
         </is>
       </c>
-      <c r="E35" s="1" t="n">
+      <c r="E35" s="2" t="n">
         <v>46241</v>
       </c>
       <c r="F35" t="inlineStr">
@@ -2245,10 +2102,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L35" t="inlineStr"/>
-      <c r="M35" t="inlineStr"/>
-      <c r="N35" t="inlineStr"/>
-      <c r="O35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -2269,7 +2122,7 @@
           <t>-21° 35´ 32.3241 -50° 10´ 09.0062 470.03</t>
         </is>
       </c>
-      <c r="E36" s="1" t="n">
+      <c r="E36" s="2" t="n">
         <v>46246</v>
       </c>
       <c r="F36" t="inlineStr">
@@ -2298,10 +2151,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L36" t="inlineStr"/>
-      <c r="M36" t="inlineStr"/>
-      <c r="N36" t="inlineStr"/>
-      <c r="O36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -2322,7 +2171,7 @@
           <t>-21° 29´ 18.1708 -50° 13´ 39.5944 458.12</t>
         </is>
       </c>
-      <c r="E37" s="1" t="n">
+      <c r="E37" s="2" t="n">
         <v>46245</v>
       </c>
       <c r="F37" t="inlineStr">
@@ -2351,10 +2200,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L37" t="inlineStr"/>
-      <c r="M37" t="inlineStr"/>
-      <c r="N37" t="inlineStr"/>
-      <c r="O37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -2365,9 +2210,7 @@
           <t>FAZ LONQUINHO</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr"/>
-      <c r="D38" t="inlineStr"/>
-      <c r="E38" s="1" t="n">
+      <c r="E38" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="F38" t="inlineStr">
@@ -2383,17 +2226,11 @@
       <c r="H38" t="n">
         <v>202.93</v>
       </c>
-      <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr">
         <is>
           <t>FEITO</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
-      <c r="M38" t="inlineStr"/>
-      <c r="N38" t="inlineStr"/>
-      <c r="O38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -2414,7 +2251,7 @@
           <t>-21° 45´ 32.6517 -50° 06´ 02.9557 456.63</t>
         </is>
       </c>
-      <c r="E39" s="1" t="n">
+      <c r="E39" s="2" t="n">
         <v>46248</v>
       </c>
       <c r="F39" t="inlineStr">
@@ -2443,10 +2280,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L39" t="inlineStr"/>
-      <c r="M39" t="inlineStr"/>
-      <c r="N39" t="inlineStr"/>
-      <c r="O39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -2467,7 +2300,7 @@
           <t>-21° 45´ 32.6517 -50° 06´ 02.9557 456.63</t>
         </is>
       </c>
-      <c r="E40" s="1" t="n">
+      <c r="E40" s="2" t="n">
         <v>46248</v>
       </c>
       <c r="F40" t="inlineStr">
@@ -2496,10 +2329,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L40" t="inlineStr"/>
-      <c r="M40" t="inlineStr"/>
-      <c r="N40" t="inlineStr"/>
-      <c r="O40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -2520,7 +2349,7 @@
           <t>-21° 23´ 27.6854 -50° 29´ 11.8918 453.23</t>
         </is>
       </c>
-      <c r="E41" s="1" t="n">
+      <c r="E41" s="2" t="n">
         <v>46254</v>
       </c>
       <c r="F41" t="inlineStr">
@@ -2536,13 +2365,6 @@
       <c r="H41" t="n">
         <v>83.7</v>
       </c>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr"/>
-      <c r="M41" t="inlineStr"/>
-      <c r="N41" t="inlineStr"/>
-      <c r="O41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -2553,9 +2375,7 @@
           <t>SÍTIO SANTO ANTONIO I</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr"/>
-      <c r="D42" t="inlineStr"/>
-      <c r="E42" s="1" t="n">
+      <c r="E42" s="2" t="n">
         <v>46248</v>
       </c>
       <c r="F42" t="inlineStr">
@@ -2579,11 +2399,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr"/>
-      <c r="M42" t="inlineStr"/>
-      <c r="N42" t="inlineStr"/>
-      <c r="O42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -2594,9 +2409,7 @@
           <t>ESTÂNCIA EBENEZER I</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr"/>
-      <c r="D43" t="inlineStr"/>
-      <c r="E43" s="1" t="n">
+      <c r="E43" s="2" t="n">
         <v>46248</v>
       </c>
       <c r="F43" t="inlineStr">
@@ -2612,17 +2425,11 @@
       <c r="H43" t="n">
         <v>13.34</v>
       </c>
-      <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
       <c r="K43" t="inlineStr">
         <is>
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L43" t="inlineStr"/>
-      <c r="M43" t="inlineStr"/>
-      <c r="N43" t="inlineStr"/>
-      <c r="O43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -2643,7 +2450,7 @@
           <t>-21° 23´ 27.6854 -50° 29´ 11.8918 453.23</t>
         </is>
       </c>
-      <c r="E44" s="1" t="n">
+      <c r="E44" s="2" t="n">
         <v>46248</v>
       </c>
       <c r="F44" t="inlineStr">
@@ -2672,10 +2479,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L44" t="inlineStr"/>
-      <c r="M44" t="inlineStr"/>
-      <c r="N44" t="inlineStr"/>
-      <c r="O44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -2696,7 +2499,7 @@
           <t>-21° 35´ 32.3241 -50° 10´ 09.0062 470.03</t>
         </is>
       </c>
-      <c r="E45" s="1" t="n">
+      <c r="E45" s="2" t="n">
         <v>40037</v>
       </c>
       <c r="F45" t="inlineStr">
@@ -2712,17 +2515,11 @@
       <c r="H45" t="n">
         <v>7.28</v>
       </c>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
       <c r="K45" t="inlineStr">
         <is>
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L45" t="inlineStr"/>
-      <c r="M45" t="inlineStr"/>
-      <c r="N45" t="inlineStr"/>
-      <c r="O45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -2733,9 +2530,7 @@
           <t>SITIO SANTA LUZIA</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr"/>
-      <c r="D46" t="inlineStr"/>
-      <c r="E46" s="1" t="n">
+      <c r="E46" s="2" t="n">
         <v>46246</v>
       </c>
       <c r="F46" t="inlineStr">
@@ -2751,13 +2546,6 @@
       <c r="H46" t="n">
         <v>2.84</v>
       </c>
-      <c r="I46" t="inlineStr"/>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr"/>
-      <c r="M46" t="inlineStr"/>
-      <c r="N46" t="inlineStr"/>
-      <c r="O46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -2768,9 +2556,7 @@
           <t>SÍTIO SANTA INÊS</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr"/>
-      <c r="D47" t="inlineStr"/>
-      <c r="E47" s="1" t="n">
+      <c r="E47" s="2" t="n">
         <v>46246</v>
       </c>
       <c r="F47" t="inlineStr">
@@ -2786,13 +2572,6 @@
       <c r="H47" t="n">
         <v>10.97</v>
       </c>
-      <c r="I47" t="inlineStr"/>
-      <c r="J47" t="inlineStr"/>
-      <c r="K47" t="inlineStr"/>
-      <c r="L47" t="inlineStr"/>
-      <c r="M47" t="inlineStr"/>
-      <c r="N47" t="inlineStr"/>
-      <c r="O47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -2803,9 +2582,7 @@
           <t>FAZENDA NOVA ERA</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr"/>
-      <c r="D48" t="inlineStr"/>
-      <c r="E48" s="1" t="n">
+      <c r="E48" s="2" t="n">
         <v>46248</v>
       </c>
       <c r="F48" t="inlineStr">
@@ -2834,10 +2611,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L48" t="inlineStr"/>
-      <c r="M48" t="inlineStr"/>
-      <c r="N48" t="inlineStr"/>
-      <c r="O48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -2858,7 +2631,7 @@
           <t>-21° 45´ 32.6517 -50° 06´ 02.9557 456.63</t>
         </is>
       </c>
-      <c r="E49" s="1" t="n">
+      <c r="E49" s="2" t="n">
         <v>46248</v>
       </c>
       <c r="F49" t="inlineStr">
@@ -2887,10 +2660,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L49" t="inlineStr"/>
-      <c r="M49" t="inlineStr"/>
-      <c r="N49" t="inlineStr"/>
-      <c r="O49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -2901,9 +2670,7 @@
           <t>SÍTIO SANTO ANTÔNIO</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr"/>
-      <c r="D50" t="inlineStr"/>
-      <c r="E50" s="1" t="n">
+      <c r="E50" s="2" t="n">
         <v>46248</v>
       </c>
       <c r="F50" t="inlineStr">
@@ -2932,10 +2699,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L50" t="inlineStr"/>
-      <c r="M50" t="inlineStr"/>
-      <c r="N50" t="inlineStr"/>
-      <c r="O50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -2956,7 +2719,7 @@
           <t>-21° 48´ 26.1814 -50° 13´ 14.2006 438.00</t>
         </is>
       </c>
-      <c r="E51" s="1" t="n">
+      <c r="E51" s="2" t="n">
         <v>46258</v>
       </c>
       <c r="F51" t="inlineStr">
@@ -2985,10 +2748,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L51" t="inlineStr"/>
-      <c r="M51" t="inlineStr"/>
-      <c r="N51" t="inlineStr"/>
-      <c r="O51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -3009,7 +2768,7 @@
           <t>-21° 24´ 42.3464 -50° 12´ 32.2760 396.57</t>
         </is>
       </c>
-      <c r="E52" s="1" t="n">
+      <c r="E52" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="F52" t="inlineStr">
@@ -3038,10 +2797,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L52" t="inlineStr"/>
-      <c r="M52" t="inlineStr"/>
-      <c r="N52" t="inlineStr"/>
-      <c r="O52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -3062,7 +2817,7 @@
           <t>-21° 24´ 42.3464 -50° 12´ 32.2760 396.57</t>
         </is>
       </c>
-      <c r="E53" s="1" t="n">
+      <c r="E53" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="F53" t="inlineStr">
@@ -3091,10 +2846,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L53" t="inlineStr"/>
-      <c r="M53" t="inlineStr"/>
-      <c r="N53" t="inlineStr"/>
-      <c r="O53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -3115,7 +2866,7 @@
           <t>-21° 47´ 12.2305 -50° 35´ 27.8405 436.14</t>
         </is>
       </c>
-      <c r="E54" s="1" t="n">
+      <c r="E54" s="2" t="n">
         <v>46261</v>
       </c>
       <c r="F54" t="inlineStr">
@@ -3123,19 +2874,12 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="G54" s="1" t="n">
+      <c r="G54" s="2" t="n">
         <v>46262</v>
       </c>
       <c r="H54" t="n">
         <v>200.36</v>
       </c>
-      <c r="I54" t="inlineStr"/>
-      <c r="J54" t="inlineStr"/>
-      <c r="K54" t="inlineStr"/>
-      <c r="L54" t="inlineStr"/>
-      <c r="M54" t="inlineStr"/>
-      <c r="N54" t="inlineStr"/>
-      <c r="O54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -3156,7 +2900,7 @@
           <t>-21° 39´ 13.2100 -50° 32´ 04.0182 418.26</t>
         </is>
       </c>
-      <c r="E55" s="1" t="n">
+      <c r="E55" s="2" t="n">
         <v>46261</v>
       </c>
       <c r="F55" t="inlineStr">
@@ -3185,10 +2929,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L55" t="inlineStr"/>
-      <c r="M55" t="inlineStr"/>
-      <c r="N55" t="inlineStr"/>
-      <c r="O55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -3209,7 +2949,7 @@
           <t>-21° 39´ 13.2100 -50° 32´ 04.0182 418.26</t>
         </is>
       </c>
-      <c r="E56" s="1" t="n">
+      <c r="E56" s="2" t="n">
         <v>46261</v>
       </c>
       <c r="F56" t="inlineStr">
@@ -3233,11 +2973,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="K56" t="inlineStr"/>
-      <c r="L56" t="inlineStr"/>
-      <c r="M56" t="inlineStr"/>
-      <c r="N56" t="inlineStr"/>
-      <c r="O56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -3248,9 +2983,7 @@
           <t>ESTÂNCIA BOA SORTE</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr"/>
-      <c r="D57" t="inlineStr"/>
-      <c r="E57" s="1" t="n">
+      <c r="E57" s="2" t="n">
         <v>46248</v>
       </c>
       <c r="F57" t="inlineStr">
@@ -3279,10 +3012,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L57" t="inlineStr"/>
-      <c r="M57" t="inlineStr"/>
-      <c r="N57" t="inlineStr"/>
-      <c r="O57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -3293,9 +3022,7 @@
           <t>SITIO SANTA CLARA I</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr"/>
-      <c r="D58" t="inlineStr"/>
-      <c r="E58" s="1" t="n">
+      <c r="E58" s="2" t="n">
         <v>46246</v>
       </c>
       <c r="F58" t="inlineStr">
@@ -3326,10 +3053,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L58" t="inlineStr"/>
-      <c r="M58" t="inlineStr"/>
-      <c r="N58" t="inlineStr"/>
-      <c r="O58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -3345,7 +3068,6 @@
           <t>B-19 SEDE TIAGO TUNES</t>
         </is>
       </c>
-      <c r="D59" t="inlineStr"/>
       <c r="E59" t="inlineStr">
         <is>
           <t>28/08/2026</t>
@@ -3364,17 +3086,11 @@
       <c r="H59" t="n">
         <v>37.72</v>
       </c>
-      <c r="I59" t="inlineStr"/>
-      <c r="J59" t="inlineStr"/>
       <c r="K59" t="inlineStr">
         <is>
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L59" t="inlineStr"/>
-      <c r="M59" t="inlineStr"/>
-      <c r="N59" t="inlineStr"/>
-      <c r="O59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -3390,7 +3106,6 @@
           <t>B-19 SEDE TIAGO TUNES</t>
         </is>
       </c>
-      <c r="D60" t="inlineStr"/>
       <c r="E60" t="inlineStr">
         <is>
           <t>28/08/2026</t>
@@ -3417,11 +3132,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="K60" t="inlineStr"/>
-      <c r="L60" t="inlineStr"/>
-      <c r="M60" t="inlineStr"/>
-      <c r="N60" t="inlineStr"/>
-      <c r="O60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -3437,7 +3147,6 @@
           <t>B-19 SEDE TIAGO TUNES</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr"/>
       <c r="E61" t="inlineStr">
         <is>
           <t>28/09/2026</t>
@@ -3464,11 +3173,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="K61" t="inlineStr"/>
-      <c r="L61" t="inlineStr"/>
-      <c r="M61" t="inlineStr"/>
-      <c r="N61" t="inlineStr"/>
-      <c r="O61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -3484,7 +3188,6 @@
           <t>B-19 SEDE TIAGO TUNES</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr"/>
       <c r="E62" t="inlineStr">
         <is>
           <t>28/08/2026</t>
@@ -3516,10 +3219,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L62" t="inlineStr"/>
-      <c r="M62" t="inlineStr"/>
-      <c r="N62" t="inlineStr"/>
-      <c r="O62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -3530,8 +3229,6 @@
           <t>SITIO SÃO JOSE</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr"/>
-      <c r="D63" t="inlineStr"/>
       <c r="E63" t="inlineStr">
         <is>
           <t>28/09/2026</t>
@@ -3558,11 +3255,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="K63" t="inlineStr"/>
-      <c r="L63" t="inlineStr"/>
-      <c r="M63" t="inlineStr"/>
-      <c r="N63" t="inlineStr"/>
-      <c r="O63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -3598,14 +3290,6 @@
           <t>09/09/2026</t>
         </is>
       </c>
-      <c r="H64" t="inlineStr"/>
-      <c r="I64" t="inlineStr"/>
-      <c r="J64" t="inlineStr"/>
-      <c r="K64" t="inlineStr"/>
-      <c r="L64" t="inlineStr"/>
-      <c r="M64" t="inlineStr"/>
-      <c r="N64" t="inlineStr"/>
-      <c r="O64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -3657,10 +3341,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L65" t="inlineStr"/>
-      <c r="M65" t="inlineStr"/>
-      <c r="N65" t="inlineStr"/>
-      <c r="O65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -3699,17 +3379,11 @@
       <c r="H66" t="n">
         <v>99.37</v>
       </c>
-      <c r="I66" t="inlineStr"/>
-      <c r="J66" t="inlineStr"/>
       <c r="K66" t="inlineStr">
         <is>
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L66" t="inlineStr"/>
-      <c r="M66" t="inlineStr"/>
-      <c r="N66" t="inlineStr"/>
-      <c r="O66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -3758,11 +3432,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="K67" t="inlineStr"/>
-      <c r="L67" t="inlineStr"/>
-      <c r="M67" t="inlineStr"/>
-      <c r="N67" t="inlineStr"/>
-      <c r="O67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -3811,11 +3480,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="K68" t="inlineStr"/>
-      <c r="L68" t="inlineStr"/>
-      <c r="M68" t="inlineStr"/>
-      <c r="N68" t="inlineStr"/>
-      <c r="O68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -3867,10 +3531,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L69" t="inlineStr"/>
-      <c r="M69" t="inlineStr"/>
-      <c r="N69" t="inlineStr"/>
-      <c r="O69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -3922,10 +3582,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L70" t="inlineStr"/>
-      <c r="M70" t="inlineStr"/>
-      <c r="N70" t="inlineStr"/>
-      <c r="O70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -3936,8 +3592,6 @@
           <t>SÍTIO LIMEIRA</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr"/>
-      <c r="D71" t="inlineStr"/>
       <c r="E71" t="inlineStr">
         <is>
           <t>04/09/2026</t>
@@ -3956,13 +3610,6 @@
       <c r="H71" t="n">
         <v>59.32</v>
       </c>
-      <c r="I71" t="inlineStr"/>
-      <c r="J71" t="inlineStr"/>
-      <c r="K71" t="inlineStr"/>
-      <c r="L71" t="inlineStr"/>
-      <c r="M71" t="inlineStr"/>
-      <c r="N71" t="inlineStr"/>
-      <c r="O71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -4001,13 +3648,6 @@
       <c r="H72" t="n">
         <v>669.6</v>
       </c>
-      <c r="I72" t="inlineStr"/>
-      <c r="J72" t="inlineStr"/>
-      <c r="K72" t="inlineStr"/>
-      <c r="L72" t="inlineStr"/>
-      <c r="M72" t="inlineStr"/>
-      <c r="N72" t="inlineStr"/>
-      <c r="O72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -4046,13 +3686,6 @@
       <c r="H73" t="n">
         <v>42.13</v>
       </c>
-      <c r="I73" t="inlineStr"/>
-      <c r="J73" t="inlineStr"/>
-      <c r="K73" t="inlineStr"/>
-      <c r="L73" t="inlineStr"/>
-      <c r="M73" t="inlineStr"/>
-      <c r="N73" t="inlineStr"/>
-      <c r="O73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -4068,7 +3701,6 @@
           <t>B-23 FAZ NOSSA SENHORA APARECIDA</t>
         </is>
       </c>
-      <c r="D74" t="inlineStr"/>
       <c r="E74" t="inlineStr">
         <is>
           <t>10/09/2026</t>
@@ -4100,10 +3732,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L74" t="inlineStr"/>
-      <c r="M74" t="inlineStr"/>
-      <c r="N74" t="inlineStr"/>
-      <c r="O74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -4119,7 +3747,6 @@
           <t>B-24 CENTRO RURAL</t>
         </is>
       </c>
-      <c r="D75" t="inlineStr"/>
       <c r="E75" t="inlineStr">
         <is>
           <t>11/09/2026</t>
@@ -4146,11 +3773,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="K75" t="inlineStr"/>
-      <c r="L75" t="inlineStr"/>
-      <c r="M75" t="inlineStr"/>
-      <c r="N75" t="inlineStr"/>
-      <c r="O75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -4166,7 +3788,6 @@
           <t>B-24 CENTRO RURAL</t>
         </is>
       </c>
-      <c r="D76" t="inlineStr"/>
       <c r="E76" t="inlineStr">
         <is>
           <t>11/09/2026</t>
@@ -4198,10 +3819,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L76" t="inlineStr"/>
-      <c r="M76" t="inlineStr"/>
-      <c r="N76" t="inlineStr"/>
-      <c r="O76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -4217,7 +3834,6 @@
           <t>B-24 CENTRO RURAL</t>
         </is>
       </c>
-      <c r="D77" t="inlineStr"/>
       <c r="E77" t="inlineStr">
         <is>
           <t>11/09/2026</t>
@@ -4233,14 +3849,6 @@
           <t>15/09/2026</t>
         </is>
       </c>
-      <c r="H77" t="inlineStr"/>
-      <c r="I77" t="inlineStr"/>
-      <c r="J77" t="inlineStr"/>
-      <c r="K77" t="inlineStr"/>
-      <c r="L77" t="inlineStr"/>
-      <c r="M77" t="inlineStr"/>
-      <c r="N77" t="inlineStr"/>
-      <c r="O77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -4256,7 +3864,6 @@
           <t>B-24 CENTRO RURAL</t>
         </is>
       </c>
-      <c r="D78" t="inlineStr"/>
       <c r="E78" t="inlineStr">
         <is>
           <t>11/09/2026</t>
@@ -4283,11 +3890,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="K78" t="inlineStr"/>
-      <c r="L78" t="inlineStr"/>
-      <c r="M78" t="inlineStr"/>
-      <c r="N78" t="inlineStr"/>
-      <c r="O78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -4303,7 +3905,6 @@
           <t>B-24 CENTRO RURAL</t>
         </is>
       </c>
-      <c r="D79" t="inlineStr"/>
       <c r="E79" t="inlineStr">
         <is>
           <t>11/09/2026</t>
@@ -4330,11 +3931,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="K79" t="inlineStr"/>
-      <c r="L79" t="inlineStr"/>
-      <c r="M79" t="inlineStr"/>
-      <c r="N79" t="inlineStr"/>
-      <c r="O79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -4386,10 +3982,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L80" t="inlineStr"/>
-      <c r="M80" t="inlineStr"/>
-      <c r="N80" t="inlineStr"/>
-      <c r="O80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -4428,17 +4020,11 @@
       <c r="H81" t="n">
         <v>84.09</v>
       </c>
-      <c r="I81" t="inlineStr"/>
-      <c r="J81" t="inlineStr"/>
       <c r="K81" t="inlineStr">
         <is>
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L81" t="inlineStr"/>
-      <c r="M81" t="inlineStr"/>
-      <c r="N81" t="inlineStr"/>
-      <c r="O81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -4454,7 +4040,6 @@
           <t>B-24 CENTRO RURAL</t>
         </is>
       </c>
-      <c r="D82" t="inlineStr"/>
       <c r="E82" t="inlineStr">
         <is>
           <t>11/09/2026</t>
@@ -4481,11 +4066,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="K82" t="inlineStr"/>
-      <c r="L82" t="inlineStr"/>
-      <c r="M82" t="inlineStr"/>
-      <c r="N82" t="inlineStr"/>
-      <c r="O82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -4521,14 +4101,6 @@
           <t>17/09/2026</t>
         </is>
       </c>
-      <c r="H83" t="inlineStr"/>
-      <c r="I83" t="inlineStr"/>
-      <c r="J83" t="inlineStr"/>
-      <c r="K83" t="inlineStr"/>
-      <c r="L83" t="inlineStr"/>
-      <c r="M83" t="inlineStr"/>
-      <c r="N83" t="inlineStr"/>
-      <c r="O83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -4580,10 +4152,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L84" t="inlineStr"/>
-      <c r="M84" t="inlineStr"/>
-      <c r="N84" t="inlineStr"/>
-      <c r="O84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -4630,11 +4198,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="K85" t="inlineStr"/>
-      <c r="L85" t="inlineStr"/>
-      <c r="M85" t="inlineStr"/>
-      <c r="N85" t="inlineStr"/>
-      <c r="O85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -4686,10 +4249,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L86" t="inlineStr"/>
-      <c r="M86" t="inlineStr"/>
-      <c r="N86" t="inlineStr"/>
-      <c r="O86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -4741,10 +4300,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L87" t="inlineStr"/>
-      <c r="M87" t="inlineStr"/>
-      <c r="N87" t="inlineStr"/>
-      <c r="O87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -4796,10 +4351,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L88" t="inlineStr"/>
-      <c r="M88" t="inlineStr"/>
-      <c r="N88" t="inlineStr"/>
-      <c r="O88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -4815,7 +4366,6 @@
           <t>B-09 FAZ SANTA ROSA AURELIO</t>
         </is>
       </c>
-      <c r="D89" t="inlineStr"/>
       <c r="E89" t="inlineStr">
         <is>
           <t>18/09/2026</t>
@@ -4834,17 +4384,11 @@
       <c r="H89" t="n">
         <v>552.0599999999999</v>
       </c>
-      <c r="I89" t="inlineStr"/>
-      <c r="J89" t="inlineStr"/>
       <c r="K89" t="inlineStr">
         <is>
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L89" t="inlineStr"/>
-      <c r="M89" t="inlineStr"/>
-      <c r="N89" t="inlineStr"/>
-      <c r="O89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -4860,7 +4404,6 @@
           <t>B-24 CENTRO RURAL</t>
         </is>
       </c>
-      <c r="D90" t="inlineStr"/>
       <c r="E90" t="inlineStr">
         <is>
           <t>11/09/2026</t>
@@ -4871,7 +4414,7 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="G90" s="1" t="n">
+      <c r="G90" s="2" t="n">
         <v>46286</v>
       </c>
       <c r="H90" t="n">
@@ -4885,11 +4428,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="K90" t="inlineStr"/>
-      <c r="L90" t="inlineStr"/>
-      <c r="M90" t="inlineStr"/>
-      <c r="N90" t="inlineStr"/>
-      <c r="O90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -4920,7 +4458,7 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="G91" s="1" t="n">
+      <c r="G91" s="2" t="n">
         <v>46286</v>
       </c>
       <c r="H91" t="n">
@@ -4939,10 +4477,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L91" t="inlineStr"/>
-      <c r="M91" t="inlineStr"/>
-      <c r="N91" t="inlineStr"/>
-      <c r="O91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -4973,7 +4507,7 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="G92" s="1" t="n">
+      <c r="G92" s="2" t="n">
         <v>46286</v>
       </c>
       <c r="H92" t="n">
@@ -4992,10 +4526,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L92" t="inlineStr"/>
-      <c r="M92" t="inlineStr"/>
-      <c r="N92" t="inlineStr"/>
-      <c r="O92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -5011,7 +4541,6 @@
           <t>B-23 FAZ NOSSA SENHORA APARECIDA</t>
         </is>
       </c>
-      <c r="D93" t="inlineStr"/>
       <c r="E93" t="inlineStr">
         <is>
           <t>21/09/2026</t>
@@ -5043,10 +4572,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L93" t="inlineStr"/>
-      <c r="M93" t="inlineStr"/>
-      <c r="N93" t="inlineStr"/>
-      <c r="O93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -5098,10 +4623,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L94" t="inlineStr"/>
-      <c r="M94" t="inlineStr"/>
-      <c r="N94" t="inlineStr"/>
-      <c r="O94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -5117,7 +4638,6 @@
           <t>B-23 FAZ NOSSA SENHORA APARECIDA</t>
         </is>
       </c>
-      <c r="D95" t="inlineStr"/>
       <c r="E95" t="inlineStr">
         <is>
           <t>21/09/2026</t>
@@ -5133,7 +4653,6 @@
           <t>24/07/2026</t>
         </is>
       </c>
-      <c r="H95" t="inlineStr"/>
       <c r="I95" t="n">
         <v>82.73999999999999</v>
       </c>
@@ -5142,11 +4661,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="K95" t="inlineStr"/>
-      <c r="L95" t="inlineStr"/>
-      <c r="M95" t="inlineStr"/>
-      <c r="N95" t="inlineStr"/>
-      <c r="O95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -5162,7 +4676,6 @@
           <t>B-016 FAZ RODA VIVA</t>
         </is>
       </c>
-      <c r="D96" t="inlineStr"/>
       <c r="E96" t="inlineStr">
         <is>
           <t>24/09/2026</t>
@@ -5181,17 +4694,11 @@
       <c r="H96" t="n">
         <v>345.05</v>
       </c>
-      <c r="I96" t="inlineStr"/>
-      <c r="J96" t="inlineStr"/>
       <c r="K96" t="inlineStr">
         <is>
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L96" t="inlineStr"/>
-      <c r="M96" t="inlineStr"/>
-      <c r="N96" t="inlineStr"/>
-      <c r="O96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -5238,11 +4745,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="K97" t="inlineStr"/>
-      <c r="L97" t="inlineStr"/>
-      <c r="M97" t="inlineStr"/>
-      <c r="N97" t="inlineStr"/>
-      <c r="O97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -5289,11 +4791,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="K98" t="inlineStr"/>
-      <c r="L98" t="inlineStr"/>
-      <c r="M98" t="inlineStr"/>
-      <c r="N98" t="inlineStr"/>
-      <c r="O98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -5340,11 +4837,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="K99" t="inlineStr"/>
-      <c r="L99" t="inlineStr"/>
-      <c r="M99" t="inlineStr"/>
-      <c r="N99" t="inlineStr"/>
-      <c r="O99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -5391,11 +4883,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="K100" t="inlineStr"/>
-      <c r="L100" t="inlineStr"/>
-      <c r="M100" t="inlineStr"/>
-      <c r="N100" t="inlineStr"/>
-      <c r="O100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -5411,7 +4898,6 @@
           <t>B-04 HARAS BILAC</t>
         </is>
       </c>
-      <c r="D101" t="inlineStr"/>
       <c r="E101" t="inlineStr">
         <is>
           <t>23/09/2026</t>
@@ -5443,10 +4929,6 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="L101" t="inlineStr"/>
-      <c r="M101" t="inlineStr"/>
-      <c r="N101" t="inlineStr"/>
-      <c r="O101" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -20310,7 +19792,6 @@
       <c r="E391" t="n">
         <v>18.47</v>
       </c>
-      <c r="F391" t="inlineStr"/>
       <c r="G391" t="n">
         <v>0</v>
       </c>
@@ -20344,7 +19825,6 @@
       <c r="E392" t="n">
         <v>10.7</v>
       </c>
-      <c r="F392" t="inlineStr"/>
       <c r="G392" t="n">
         <v>0</v>
       </c>
@@ -20378,7 +19858,6 @@
       <c r="E393" t="n">
         <v>3.89</v>
       </c>
-      <c r="F393" t="inlineStr"/>
       <c r="G393" t="n">
         <v>0</v>
       </c>
@@ -24005,7 +23484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24014,10 +23493,20 @@
           <t>creditos_inforow</t>
         </is>
       </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>senha_acesso</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
         <v>11121.66</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Clealco@Geo2026</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Remocao do modo escuro, melhorias de responsividade mobile e correcao do GPS
</commit_message>
<xml_diff>
--- a/dados.xlsx
+++ b/dados.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BASE_PROCESSAMENTOS" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BACKLOG" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FALHAS_PLANTIO" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="METAS_GLOBAIS" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ACOMPANHAMENTO" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONFIG" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="BASE_PROCESSAMENTOS" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="BACKLOG" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="FALHAS_PLANTIO" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="METAS_GLOBAIS" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="ACOMPANHAMENTO" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="CONFIG" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,8 +21,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -53,10 +54,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -516,7 +516,8 @@
           <t>B-24 CENTRO RURAL</t>
         </is>
       </c>
-      <c r="E2" s="2" t="n">
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" s="1" t="n">
         <v>46205</v>
       </c>
       <c r="F2" t="inlineStr">
@@ -540,6 +541,11 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -560,7 +566,7 @@
           <t>-22° 02´ 13.3421 -50° 07´ 13.5185 491.84</t>
         </is>
       </c>
-      <c r="E3" s="2" t="n">
+      <c r="E3" s="1" t="n">
         <v>46217</v>
       </c>
       <c r="F3" t="inlineStr">
@@ -600,6 +606,7 @@
       <c r="N3" t="n">
         <v>586.49</v>
       </c>
+      <c r="O3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -615,7 +622,8 @@
           <t>B-23 FAZ NOSSA SENHORA APARECIDA</t>
         </is>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="F4" t="inlineStr">
@@ -655,6 +663,7 @@
       <c r="N4" t="n">
         <v>854.9300000000001</v>
       </c>
+      <c r="O4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -675,7 +684,7 @@
           <t>-21° 39´ 13.2100 -50° 32´ 04.0182 418.26</t>
         </is>
       </c>
-      <c r="E5" s="2" t="n">
+      <c r="E5" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F5" t="inlineStr">
@@ -704,6 +713,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -724,7 +737,7 @@
           <t>-21° 39´ 13.2100 -50° 32´ 04.0182 418.26</t>
         </is>
       </c>
-      <c r="E6" s="2" t="n">
+      <c r="E6" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F6" t="inlineStr">
@@ -753,6 +766,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -773,7 +790,7 @@
           <t>-21° 34´ 46.1049 -50° 26´ 00.0424 442.78</t>
         </is>
       </c>
-      <c r="E7" s="2" t="n">
+      <c r="E7" s="1" t="n">
         <v>46183</v>
       </c>
       <c r="F7" t="inlineStr">
@@ -802,6 +819,7 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr">
         <is>
           <t xml:space="preserve">PROPRIAS </t>
@@ -833,7 +851,7 @@
           <t>-22° 02´ 13.3421 -50° 07´ 13.5185 491.84</t>
         </is>
       </c>
-      <c r="E8" s="2" t="n">
+      <c r="E8" s="1" t="n">
         <v>46196</v>
       </c>
       <c r="F8" t="inlineStr">
@@ -862,6 +880,7 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr">
         <is>
           <t>TERCEIROS</t>
@@ -888,7 +907,8 @@
           <t>B-23 FAZ NOSSA SENHORA APARECIDA</t>
         </is>
       </c>
-      <c r="E9" s="2" t="n">
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="F9" t="inlineStr">
@@ -917,6 +937,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -937,7 +961,7 @@
           <t>-21° 31´ 28.9807 -50° 18´ 16.5320 492.23</t>
         </is>
       </c>
-      <c r="E10" s="2" t="n">
+      <c r="E10" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="F10" t="inlineStr">
@@ -966,6 +990,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -986,7 +1014,7 @@
           <t>-21° 39´ 13.2100 -50° 32´ 04.0182 418.26</t>
         </is>
       </c>
-      <c r="E11" s="2" t="n">
+      <c r="E11" s="1" t="n">
         <v>46189</v>
       </c>
       <c r="F11" t="inlineStr">
@@ -1015,6 +1043,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1030,7 +1062,8 @@
           <t>B-24 CENTRO RURAL</t>
         </is>
       </c>
-      <c r="E12" s="2" t="n">
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" s="1" t="n">
         <v>46203</v>
       </c>
       <c r="F12" t="inlineStr">
@@ -1059,6 +1092,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1079,7 +1116,7 @@
           <t>-21° 31´ 28.9807 -50° 18´ 16.5320 492.23</t>
         </is>
       </c>
-      <c r="E13" s="2" t="n">
+      <c r="E13" s="1" t="n">
         <v>46185</v>
       </c>
       <c r="F13" t="inlineStr">
@@ -1108,6 +1145,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1128,7 +1169,7 @@
           <t>-21° 31´ 28.9807 -50° 18´ 16.5320 492.23</t>
         </is>
       </c>
-      <c r="E14" s="2" t="n">
+      <c r="E14" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="F14" t="inlineStr">
@@ -1157,6 +1198,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1167,7 +1212,9 @@
           <t>SÍTIO SÃO FRANCISCO -</t>
         </is>
       </c>
-      <c r="E15" s="2" t="n">
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" s="1" t="n">
         <v>46185</v>
       </c>
       <c r="F15" t="inlineStr">
@@ -1196,6 +1243,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1211,7 +1262,8 @@
           <t>B-24 CENTRO RURAL</t>
         </is>
       </c>
-      <c r="E16" s="2" t="n">
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" s="1" t="n">
         <v>46203</v>
       </c>
       <c r="F16" t="inlineStr">
@@ -1240,6 +1292,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1260,7 +1316,7 @@
           <t>-21° 31´ 28.9807 -50° 18´ 16.5320 492.23</t>
         </is>
       </c>
-      <c r="E17" s="2" t="n">
+      <c r="E17" s="1" t="n">
         <v>46185</v>
       </c>
       <c r="F17" t="inlineStr">
@@ -1289,6 +1345,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1309,7 +1369,7 @@
           <t>-21° 35´ 32.3241 -50° 10´ 09.0062 470.03</t>
         </is>
       </c>
-      <c r="E18" s="2" t="n">
+      <c r="E18" s="1" t="n">
         <v>46219</v>
       </c>
       <c r="F18" t="inlineStr">
@@ -1338,6 +1398,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1358,7 +1422,7 @@
           <t>-21° 31´ 28.9807 -50° 18´ 16.5320 492.23</t>
         </is>
       </c>
-      <c r="E19" s="2" t="n">
+      <c r="E19" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="F19" t="inlineStr">
@@ -1387,6 +1451,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1397,7 +1465,9 @@
           <t>SÍTIO IRMÃOS ANNELLI -</t>
         </is>
       </c>
-      <c r="E20" s="2" t="n">
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" s="1" t="n">
         <v>46185</v>
       </c>
       <c r="F20" t="inlineStr">
@@ -1426,6 +1496,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1436,7 +1510,9 @@
           <t>SÍTIO TREZE DE MAIO</t>
         </is>
       </c>
-      <c r="E21" s="2" t="n">
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" s="1" t="n">
         <v>46205</v>
       </c>
       <c r="F21" t="inlineStr">
@@ -1444,7 +1520,7 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="G21" s="2" t="n">
+      <c r="G21" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="H21" t="n">
@@ -1463,6 +1539,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1483,7 +1563,7 @@
           <t>-21° 39´ 59.2206 -50° 19´ 50.9494 405.70</t>
         </is>
       </c>
-      <c r="E22" s="2" t="n">
+      <c r="E22" s="1" t="n">
         <v>46216</v>
       </c>
       <c r="F22" t="inlineStr">
@@ -1512,6 +1592,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1532,7 +1616,7 @@
           <t>-21° 31´ 28.9807 -50° 18´ 16.5320 492.23</t>
         </is>
       </c>
-      <c r="E23" s="2" t="n">
+      <c r="E23" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="F23" t="inlineStr">
@@ -1561,6 +1645,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1581,7 +1669,7 @@
           <t>-21° 35´ 32.3241 -50° 10´ 09.0062 470.03</t>
         </is>
       </c>
-      <c r="E24" s="2" t="n">
+      <c r="E24" s="1" t="n">
         <v>46219</v>
       </c>
       <c r="F24" t="inlineStr">
@@ -1610,6 +1698,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1630,7 +1722,7 @@
           <t>-21° 35´ 32.3241 -50° 10´ 09.0062 470.03</t>
         </is>
       </c>
-      <c r="E25" s="2" t="n">
+      <c r="E25" s="1" t="n">
         <v>46219</v>
       </c>
       <c r="F25" t="inlineStr">
@@ -1659,6 +1751,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1679,7 +1775,7 @@
           <t>-21° 48´ 26.1814 -50° 13´ 14.2006 438.00</t>
         </is>
       </c>
-      <c r="E26" s="2" t="n">
+      <c r="E26" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="F26" t="inlineStr">
@@ -1708,6 +1804,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1728,7 +1828,7 @@
           <t>-21° 48´ 26.1814 -50° 13´ 14.2006 438.00</t>
         </is>
       </c>
-      <c r="E27" s="2" t="n">
+      <c r="E27" s="1" t="n">
         <v>46239</v>
       </c>
       <c r="F27" t="inlineStr">
@@ -1757,6 +1857,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1777,7 +1881,7 @@
           <t>-21° 45´ 32.6517 -50° 06´ 02.9557 456.63</t>
         </is>
       </c>
-      <c r="E28" s="2" t="n">
+      <c r="E28" s="1" t="n">
         <v>46240</v>
       </c>
       <c r="F28" t="inlineStr">
@@ -1793,6 +1897,13 @@
       <c r="H28" t="n">
         <v>94.87</v>
       </c>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1813,7 +1924,7 @@
           <t>-21° 48´ 26.1814 -50° 13´ 14.2006 438.00</t>
         </is>
       </c>
-      <c r="E29" s="2" t="n">
+      <c r="E29" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="F29" t="inlineStr">
@@ -1842,6 +1953,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr"/>
+      <c r="N29" t="inlineStr"/>
+      <c r="O29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1862,7 +1977,7 @@
           <t>-21° 39´ 13.2100 -50° 32´ 04.0182 418.26</t>
         </is>
       </c>
-      <c r="E30" s="2" t="n">
+      <c r="E30" s="1" t="n">
         <v>46237</v>
       </c>
       <c r="F30" t="inlineStr">
@@ -1878,6 +1993,13 @@
       <c r="H30" t="n">
         <v>57.73</v>
       </c>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" t="inlineStr"/>
+      <c r="O30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1898,7 +2020,7 @@
           <t>-21° 48´ 26.1814 -50° 13´ 14.2006 438.00</t>
         </is>
       </c>
-      <c r="E31" s="2" t="n">
+      <c r="E31" s="1" t="n">
         <v>46240</v>
       </c>
       <c r="F31" t="inlineStr">
@@ -1924,6 +2046,11 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr"/>
+      <c r="N31" t="inlineStr"/>
+      <c r="O31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1944,7 +2071,7 @@
           <t>-21° 39´ 13.2100 -50° 32´ 04.0182 418.26</t>
         </is>
       </c>
-      <c r="E32" s="2" t="n">
+      <c r="E32" s="1" t="n">
         <v>46237</v>
       </c>
       <c r="F32" t="inlineStr">
@@ -1968,6 +2095,11 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr"/>
+      <c r="N32" t="inlineStr"/>
+      <c r="O32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1988,7 +2120,7 @@
           <t>-22° 02´ 13.3421 -50° 07´ 13.5185 491.84</t>
         </is>
       </c>
-      <c r="E33" s="2" t="n">
+      <c r="E33" s="1" t="n">
         <v>46231</v>
       </c>
       <c r="F33" t="inlineStr">
@@ -2004,6 +2136,13 @@
       <c r="H33" t="n">
         <v>95.5</v>
       </c>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr"/>
+      <c r="N33" t="inlineStr"/>
+      <c r="O33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -2024,7 +2163,7 @@
           <t>-21° 31´ 28.9807 -50° 18´ 16.5320 492.23</t>
         </is>
       </c>
-      <c r="E34" s="2" t="n">
+      <c r="E34" s="1" t="n">
         <v>46241</v>
       </c>
       <c r="F34" t="inlineStr">
@@ -2053,6 +2192,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr"/>
+      <c r="N34" t="inlineStr"/>
+      <c r="O34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -2073,7 +2216,7 @@
           <t>-21° 31´ 28.9807 -50° 18´ 16.5320 492.23</t>
         </is>
       </c>
-      <c r="E35" s="2" t="n">
+      <c r="E35" s="1" t="n">
         <v>46241</v>
       </c>
       <c r="F35" t="inlineStr">
@@ -2102,6 +2245,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="inlineStr"/>
+      <c r="N35" t="inlineStr"/>
+      <c r="O35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -2122,7 +2269,7 @@
           <t>-21° 35´ 32.3241 -50° 10´ 09.0062 470.03</t>
         </is>
       </c>
-      <c r="E36" s="2" t="n">
+      <c r="E36" s="1" t="n">
         <v>46246</v>
       </c>
       <c r="F36" t="inlineStr">
@@ -2151,6 +2298,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="inlineStr"/>
+      <c r="N36" t="inlineStr"/>
+      <c r="O36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -2171,7 +2322,7 @@
           <t>-21° 29´ 18.1708 -50° 13´ 39.5944 458.12</t>
         </is>
       </c>
-      <c r="E37" s="2" t="n">
+      <c r="E37" s="1" t="n">
         <v>46245</v>
       </c>
       <c r="F37" t="inlineStr">
@@ -2200,6 +2351,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr"/>
+      <c r="N37" t="inlineStr"/>
+      <c r="O37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -2210,7 +2365,9 @@
           <t>FAZ LONQUINHO</t>
         </is>
       </c>
-      <c r="E38" s="2" t="n">
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" s="1" t="n">
         <v>46247</v>
       </c>
       <c r="F38" t="inlineStr">
@@ -2226,11 +2383,17 @@
       <c r="H38" t="n">
         <v>202.93</v>
       </c>
+      <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr">
         <is>
           <t>FEITO</t>
         </is>
       </c>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr"/>
+      <c r="N38" t="inlineStr"/>
+      <c r="O38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -2251,7 +2414,7 @@
           <t>-21° 45´ 32.6517 -50° 06´ 02.9557 456.63</t>
         </is>
       </c>
-      <c r="E39" s="2" t="n">
+      <c r="E39" s="1" t="n">
         <v>46248</v>
       </c>
       <c r="F39" t="inlineStr">
@@ -2280,6 +2443,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr"/>
+      <c r="N39" t="inlineStr"/>
+      <c r="O39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -2300,7 +2467,7 @@
           <t>-21° 45´ 32.6517 -50° 06´ 02.9557 456.63</t>
         </is>
       </c>
-      <c r="E40" s="2" t="n">
+      <c r="E40" s="1" t="n">
         <v>46248</v>
       </c>
       <c r="F40" t="inlineStr">
@@ -2329,6 +2496,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr"/>
+      <c r="N40" t="inlineStr"/>
+      <c r="O40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -2349,7 +2520,7 @@
           <t>-21° 23´ 27.6854 -50° 29´ 11.8918 453.23</t>
         </is>
       </c>
-      <c r="E41" s="2" t="n">
+      <c r="E41" s="1" t="n">
         <v>46254</v>
       </c>
       <c r="F41" t="inlineStr">
@@ -2365,6 +2536,13 @@
       <c r="H41" t="n">
         <v>83.7</v>
       </c>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr"/>
+      <c r="N41" t="inlineStr"/>
+      <c r="O41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -2375,7 +2553,9 @@
           <t>SÍTIO SANTO ANTONIO I</t>
         </is>
       </c>
-      <c r="E42" s="2" t="n">
+      <c r="C42" t="inlineStr"/>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" s="1" t="n">
         <v>46248</v>
       </c>
       <c r="F42" t="inlineStr">
@@ -2399,6 +2579,11 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr"/>
+      <c r="N42" t="inlineStr"/>
+      <c r="O42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -2409,7 +2594,9 @@
           <t>ESTÂNCIA EBENEZER I</t>
         </is>
       </c>
-      <c r="E43" s="2" t="n">
+      <c r="C43" t="inlineStr"/>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" s="1" t="n">
         <v>46248</v>
       </c>
       <c r="F43" t="inlineStr">
@@ -2425,11 +2612,17 @@
       <c r="H43" t="n">
         <v>13.34</v>
       </c>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr"/>
       <c r="K43" t="inlineStr">
         <is>
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr"/>
+      <c r="N43" t="inlineStr"/>
+      <c r="O43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -2450,7 +2643,7 @@
           <t>-21° 23´ 27.6854 -50° 29´ 11.8918 453.23</t>
         </is>
       </c>
-      <c r="E44" s="2" t="n">
+      <c r="E44" s="1" t="n">
         <v>46248</v>
       </c>
       <c r="F44" t="inlineStr">
@@ -2479,6 +2672,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr"/>
+      <c r="N44" t="inlineStr"/>
+      <c r="O44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -2499,7 +2696,7 @@
           <t>-21° 35´ 32.3241 -50° 10´ 09.0062 470.03</t>
         </is>
       </c>
-      <c r="E45" s="2" t="n">
+      <c r="E45" s="1" t="n">
         <v>40037</v>
       </c>
       <c r="F45" t="inlineStr">
@@ -2515,11 +2712,17 @@
       <c r="H45" t="n">
         <v>7.28</v>
       </c>
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="inlineStr"/>
       <c r="K45" t="inlineStr">
         <is>
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L45" t="inlineStr"/>
+      <c r="M45" t="inlineStr"/>
+      <c r="N45" t="inlineStr"/>
+      <c r="O45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -2530,7 +2733,9 @@
           <t>SITIO SANTA LUZIA</t>
         </is>
       </c>
-      <c r="E46" s="2" t="n">
+      <c r="C46" t="inlineStr"/>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" s="1" t="n">
         <v>46246</v>
       </c>
       <c r="F46" t="inlineStr">
@@ -2546,6 +2751,13 @@
       <c r="H46" t="n">
         <v>2.84</v>
       </c>
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr"/>
+      <c r="N46" t="inlineStr"/>
+      <c r="O46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -2556,7 +2768,9 @@
           <t>SÍTIO SANTA INÊS</t>
         </is>
       </c>
-      <c r="E47" s="2" t="n">
+      <c r="C47" t="inlineStr"/>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" s="1" t="n">
         <v>46246</v>
       </c>
       <c r="F47" t="inlineStr">
@@ -2572,6 +2786,13 @@
       <c r="H47" t="n">
         <v>10.97</v>
       </c>
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr"/>
+      <c r="N47" t="inlineStr"/>
+      <c r="O47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -2582,7 +2803,9 @@
           <t>FAZENDA NOVA ERA</t>
         </is>
       </c>
-      <c r="E48" s="2" t="n">
+      <c r="C48" t="inlineStr"/>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" s="1" t="n">
         <v>46248</v>
       </c>
       <c r="F48" t="inlineStr">
@@ -2611,6 +2834,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr"/>
+      <c r="N48" t="inlineStr"/>
+      <c r="O48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -2631,7 +2858,7 @@
           <t>-21° 45´ 32.6517 -50° 06´ 02.9557 456.63</t>
         </is>
       </c>
-      <c r="E49" s="2" t="n">
+      <c r="E49" s="1" t="n">
         <v>46248</v>
       </c>
       <c r="F49" t="inlineStr">
@@ -2660,6 +2887,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr"/>
+      <c r="N49" t="inlineStr"/>
+      <c r="O49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -2670,7 +2901,9 @@
           <t>SÍTIO SANTO ANTÔNIO</t>
         </is>
       </c>
-      <c r="E50" s="2" t="n">
+      <c r="C50" t="inlineStr"/>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" s="1" t="n">
         <v>46248</v>
       </c>
       <c r="F50" t="inlineStr">
@@ -2699,6 +2932,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr"/>
+      <c r="N50" t="inlineStr"/>
+      <c r="O50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -2719,7 +2956,7 @@
           <t>-21° 48´ 26.1814 -50° 13´ 14.2006 438.00</t>
         </is>
       </c>
-      <c r="E51" s="2" t="n">
+      <c r="E51" s="1" t="n">
         <v>46258</v>
       </c>
       <c r="F51" t="inlineStr">
@@ -2748,6 +2985,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr"/>
+      <c r="N51" t="inlineStr"/>
+      <c r="O51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -2768,7 +3009,7 @@
           <t>-21° 24´ 42.3464 -50° 12´ 32.2760 396.57</t>
         </is>
       </c>
-      <c r="E52" s="2" t="n">
+      <c r="E52" s="1" t="n">
         <v>46259</v>
       </c>
       <c r="F52" t="inlineStr">
@@ -2797,6 +3038,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L52" t="inlineStr"/>
+      <c r="M52" t="inlineStr"/>
+      <c r="N52" t="inlineStr"/>
+      <c r="O52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -2817,7 +3062,7 @@
           <t>-21° 24´ 42.3464 -50° 12´ 32.2760 396.57</t>
         </is>
       </c>
-      <c r="E53" s="2" t="n">
+      <c r="E53" s="1" t="n">
         <v>46259</v>
       </c>
       <c r="F53" t="inlineStr">
@@ -2846,6 +3091,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L53" t="inlineStr"/>
+      <c r="M53" t="inlineStr"/>
+      <c r="N53" t="inlineStr"/>
+      <c r="O53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -2866,7 +3115,7 @@
           <t>-21° 47´ 12.2305 -50° 35´ 27.8405 436.14</t>
         </is>
       </c>
-      <c r="E54" s="2" t="n">
+      <c r="E54" s="1" t="n">
         <v>46261</v>
       </c>
       <c r="F54" t="inlineStr">
@@ -2874,12 +3123,19 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="G54" s="2" t="n">
+      <c r="G54" s="1" t="n">
         <v>46262</v>
       </c>
       <c r="H54" t="n">
         <v>200.36</v>
       </c>
+      <c r="I54" t="inlineStr"/>
+      <c r="J54" t="inlineStr"/>
+      <c r="K54" t="inlineStr"/>
+      <c r="L54" t="inlineStr"/>
+      <c r="M54" t="inlineStr"/>
+      <c r="N54" t="inlineStr"/>
+      <c r="O54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -2900,7 +3156,7 @@
           <t>-21° 39´ 13.2100 -50° 32´ 04.0182 418.26</t>
         </is>
       </c>
-      <c r="E55" s="2" t="n">
+      <c r="E55" s="1" t="n">
         <v>46261</v>
       </c>
       <c r="F55" t="inlineStr">
@@ -2929,6 +3185,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L55" t="inlineStr"/>
+      <c r="M55" t="inlineStr"/>
+      <c r="N55" t="inlineStr"/>
+      <c r="O55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -2949,7 +3209,7 @@
           <t>-21° 39´ 13.2100 -50° 32´ 04.0182 418.26</t>
         </is>
       </c>
-      <c r="E56" s="2" t="n">
+      <c r="E56" s="1" t="n">
         <v>46261</v>
       </c>
       <c r="F56" t="inlineStr">
@@ -2973,6 +3233,11 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="K56" t="inlineStr"/>
+      <c r="L56" t="inlineStr"/>
+      <c r="M56" t="inlineStr"/>
+      <c r="N56" t="inlineStr"/>
+      <c r="O56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -2983,7 +3248,9 @@
           <t>ESTÂNCIA BOA SORTE</t>
         </is>
       </c>
-      <c r="E57" s="2" t="n">
+      <c r="C57" t="inlineStr"/>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" s="1" t="n">
         <v>46248</v>
       </c>
       <c r="F57" t="inlineStr">
@@ -3012,6 +3279,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L57" t="inlineStr"/>
+      <c r="M57" t="inlineStr"/>
+      <c r="N57" t="inlineStr"/>
+      <c r="O57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -3022,7 +3293,9 @@
           <t>SITIO SANTA CLARA I</t>
         </is>
       </c>
-      <c r="E58" s="2" t="n">
+      <c r="C58" t="inlineStr"/>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" s="1" t="n">
         <v>46246</v>
       </c>
       <c r="F58" t="inlineStr">
@@ -3053,6 +3326,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L58" t="inlineStr"/>
+      <c r="M58" t="inlineStr"/>
+      <c r="N58" t="inlineStr"/>
+      <c r="O58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -3068,6 +3345,7 @@
           <t>B-19 SEDE TIAGO TUNES</t>
         </is>
       </c>
+      <c r="D59" t="inlineStr"/>
       <c r="E59" t="inlineStr">
         <is>
           <t>28/08/2026</t>
@@ -3086,11 +3364,17 @@
       <c r="H59" t="n">
         <v>37.72</v>
       </c>
+      <c r="I59" t="inlineStr"/>
+      <c r="J59" t="inlineStr"/>
       <c r="K59" t="inlineStr">
         <is>
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L59" t="inlineStr"/>
+      <c r="M59" t="inlineStr"/>
+      <c r="N59" t="inlineStr"/>
+      <c r="O59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -3106,6 +3390,7 @@
           <t>B-19 SEDE TIAGO TUNES</t>
         </is>
       </c>
+      <c r="D60" t="inlineStr"/>
       <c r="E60" t="inlineStr">
         <is>
           <t>28/08/2026</t>
@@ -3132,6 +3417,11 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="K60" t="inlineStr"/>
+      <c r="L60" t="inlineStr"/>
+      <c r="M60" t="inlineStr"/>
+      <c r="N60" t="inlineStr"/>
+      <c r="O60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -3147,6 +3437,7 @@
           <t>B-19 SEDE TIAGO TUNES</t>
         </is>
       </c>
+      <c r="D61" t="inlineStr"/>
       <c r="E61" t="inlineStr">
         <is>
           <t>28/09/2026</t>
@@ -3173,6 +3464,11 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="K61" t="inlineStr"/>
+      <c r="L61" t="inlineStr"/>
+      <c r="M61" t="inlineStr"/>
+      <c r="N61" t="inlineStr"/>
+      <c r="O61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -3188,6 +3484,7 @@
           <t>B-19 SEDE TIAGO TUNES</t>
         </is>
       </c>
+      <c r="D62" t="inlineStr"/>
       <c r="E62" t="inlineStr">
         <is>
           <t>28/08/2026</t>
@@ -3219,6 +3516,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L62" t="inlineStr"/>
+      <c r="M62" t="inlineStr"/>
+      <c r="N62" t="inlineStr"/>
+      <c r="O62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -3229,6 +3530,8 @@
           <t>SITIO SÃO JOSE</t>
         </is>
       </c>
+      <c r="C63" t="inlineStr"/>
+      <c r="D63" t="inlineStr"/>
       <c r="E63" t="inlineStr">
         <is>
           <t>28/09/2026</t>
@@ -3255,6 +3558,11 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="K63" t="inlineStr"/>
+      <c r="L63" t="inlineStr"/>
+      <c r="M63" t="inlineStr"/>
+      <c r="N63" t="inlineStr"/>
+      <c r="O63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -3290,6 +3598,14 @@
           <t>09/09/2026</t>
         </is>
       </c>
+      <c r="H64" t="inlineStr"/>
+      <c r="I64" t="inlineStr"/>
+      <c r="J64" t="inlineStr"/>
+      <c r="K64" t="inlineStr"/>
+      <c r="L64" t="inlineStr"/>
+      <c r="M64" t="inlineStr"/>
+      <c r="N64" t="inlineStr"/>
+      <c r="O64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -3341,6 +3657,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L65" t="inlineStr"/>
+      <c r="M65" t="inlineStr"/>
+      <c r="N65" t="inlineStr"/>
+      <c r="O65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -3379,11 +3699,17 @@
       <c r="H66" t="n">
         <v>99.37</v>
       </c>
+      <c r="I66" t="inlineStr"/>
+      <c r="J66" t="inlineStr"/>
       <c r="K66" t="inlineStr">
         <is>
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L66" t="inlineStr"/>
+      <c r="M66" t="inlineStr"/>
+      <c r="N66" t="inlineStr"/>
+      <c r="O66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -3432,6 +3758,11 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="K67" t="inlineStr"/>
+      <c r="L67" t="inlineStr"/>
+      <c r="M67" t="inlineStr"/>
+      <c r="N67" t="inlineStr"/>
+      <c r="O67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -3480,6 +3811,11 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="K68" t="inlineStr"/>
+      <c r="L68" t="inlineStr"/>
+      <c r="M68" t="inlineStr"/>
+      <c r="N68" t="inlineStr"/>
+      <c r="O68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -3531,6 +3867,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L69" t="inlineStr"/>
+      <c r="M69" t="inlineStr"/>
+      <c r="N69" t="inlineStr"/>
+      <c r="O69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -3582,6 +3922,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L70" t="inlineStr"/>
+      <c r="M70" t="inlineStr"/>
+      <c r="N70" t="inlineStr"/>
+      <c r="O70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -3592,6 +3936,8 @@
           <t>SÍTIO LIMEIRA</t>
         </is>
       </c>
+      <c r="C71" t="inlineStr"/>
+      <c r="D71" t="inlineStr"/>
       <c r="E71" t="inlineStr">
         <is>
           <t>04/09/2026</t>
@@ -3610,6 +3956,13 @@
       <c r="H71" t="n">
         <v>59.32</v>
       </c>
+      <c r="I71" t="inlineStr"/>
+      <c r="J71" t="inlineStr"/>
+      <c r="K71" t="inlineStr"/>
+      <c r="L71" t="inlineStr"/>
+      <c r="M71" t="inlineStr"/>
+      <c r="N71" t="inlineStr"/>
+      <c r="O71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -3648,6 +4001,13 @@
       <c r="H72" t="n">
         <v>669.6</v>
       </c>
+      <c r="I72" t="inlineStr"/>
+      <c r="J72" t="inlineStr"/>
+      <c r="K72" t="inlineStr"/>
+      <c r="L72" t="inlineStr"/>
+      <c r="M72" t="inlineStr"/>
+      <c r="N72" t="inlineStr"/>
+      <c r="O72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -3686,6 +4046,13 @@
       <c r="H73" t="n">
         <v>42.13</v>
       </c>
+      <c r="I73" t="inlineStr"/>
+      <c r="J73" t="inlineStr"/>
+      <c r="K73" t="inlineStr"/>
+      <c r="L73" t="inlineStr"/>
+      <c r="M73" t="inlineStr"/>
+      <c r="N73" t="inlineStr"/>
+      <c r="O73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -3701,6 +4068,7 @@
           <t>B-23 FAZ NOSSA SENHORA APARECIDA</t>
         </is>
       </c>
+      <c r="D74" t="inlineStr"/>
       <c r="E74" t="inlineStr">
         <is>
           <t>10/09/2026</t>
@@ -3732,6 +4100,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L74" t="inlineStr"/>
+      <c r="M74" t="inlineStr"/>
+      <c r="N74" t="inlineStr"/>
+      <c r="O74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -3747,6 +4119,7 @@
           <t>B-24 CENTRO RURAL</t>
         </is>
       </c>
+      <c r="D75" t="inlineStr"/>
       <c r="E75" t="inlineStr">
         <is>
           <t>11/09/2026</t>
@@ -3773,6 +4146,11 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="K75" t="inlineStr"/>
+      <c r="L75" t="inlineStr"/>
+      <c r="M75" t="inlineStr"/>
+      <c r="N75" t="inlineStr"/>
+      <c r="O75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -3788,6 +4166,7 @@
           <t>B-24 CENTRO RURAL</t>
         </is>
       </c>
+      <c r="D76" t="inlineStr"/>
       <c r="E76" t="inlineStr">
         <is>
           <t>11/09/2026</t>
@@ -3819,6 +4198,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L76" t="inlineStr"/>
+      <c r="M76" t="inlineStr"/>
+      <c r="N76" t="inlineStr"/>
+      <c r="O76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -3834,6 +4217,7 @@
           <t>B-24 CENTRO RURAL</t>
         </is>
       </c>
+      <c r="D77" t="inlineStr"/>
       <c r="E77" t="inlineStr">
         <is>
           <t>11/09/2026</t>
@@ -3849,6 +4233,14 @@
           <t>15/09/2026</t>
         </is>
       </c>
+      <c r="H77" t="inlineStr"/>
+      <c r="I77" t="inlineStr"/>
+      <c r="J77" t="inlineStr"/>
+      <c r="K77" t="inlineStr"/>
+      <c r="L77" t="inlineStr"/>
+      <c r="M77" t="inlineStr"/>
+      <c r="N77" t="inlineStr"/>
+      <c r="O77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -3864,6 +4256,7 @@
           <t>B-24 CENTRO RURAL</t>
         </is>
       </c>
+      <c r="D78" t="inlineStr"/>
       <c r="E78" t="inlineStr">
         <is>
           <t>11/09/2026</t>
@@ -3890,6 +4283,11 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="K78" t="inlineStr"/>
+      <c r="L78" t="inlineStr"/>
+      <c r="M78" t="inlineStr"/>
+      <c r="N78" t="inlineStr"/>
+      <c r="O78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -3905,6 +4303,7 @@
           <t>B-24 CENTRO RURAL</t>
         </is>
       </c>
+      <c r="D79" t="inlineStr"/>
       <c r="E79" t="inlineStr">
         <is>
           <t>11/09/2026</t>
@@ -3931,6 +4330,11 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="K79" t="inlineStr"/>
+      <c r="L79" t="inlineStr"/>
+      <c r="M79" t="inlineStr"/>
+      <c r="N79" t="inlineStr"/>
+      <c r="O79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -3982,6 +4386,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L80" t="inlineStr"/>
+      <c r="M80" t="inlineStr"/>
+      <c r="N80" t="inlineStr"/>
+      <c r="O80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -4020,11 +4428,17 @@
       <c r="H81" t="n">
         <v>84.09</v>
       </c>
+      <c r="I81" t="inlineStr"/>
+      <c r="J81" t="inlineStr"/>
       <c r="K81" t="inlineStr">
         <is>
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L81" t="inlineStr"/>
+      <c r="M81" t="inlineStr"/>
+      <c r="N81" t="inlineStr"/>
+      <c r="O81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -4040,6 +4454,7 @@
           <t>B-24 CENTRO RURAL</t>
         </is>
       </c>
+      <c r="D82" t="inlineStr"/>
       <c r="E82" t="inlineStr">
         <is>
           <t>11/09/2026</t>
@@ -4066,6 +4481,11 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="K82" t="inlineStr"/>
+      <c r="L82" t="inlineStr"/>
+      <c r="M82" t="inlineStr"/>
+      <c r="N82" t="inlineStr"/>
+      <c r="O82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -4101,6 +4521,14 @@
           <t>17/09/2026</t>
         </is>
       </c>
+      <c r="H83" t="inlineStr"/>
+      <c r="I83" t="inlineStr"/>
+      <c r="J83" t="inlineStr"/>
+      <c r="K83" t="inlineStr"/>
+      <c r="L83" t="inlineStr"/>
+      <c r="M83" t="inlineStr"/>
+      <c r="N83" t="inlineStr"/>
+      <c r="O83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -4152,6 +4580,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L84" t="inlineStr"/>
+      <c r="M84" t="inlineStr"/>
+      <c r="N84" t="inlineStr"/>
+      <c r="O84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -4198,6 +4630,11 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="K85" t="inlineStr"/>
+      <c r="L85" t="inlineStr"/>
+      <c r="M85" t="inlineStr"/>
+      <c r="N85" t="inlineStr"/>
+      <c r="O85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -4249,6 +4686,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L86" t="inlineStr"/>
+      <c r="M86" t="inlineStr"/>
+      <c r="N86" t="inlineStr"/>
+      <c r="O86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -4300,6 +4741,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L87" t="inlineStr"/>
+      <c r="M87" t="inlineStr"/>
+      <c r="N87" t="inlineStr"/>
+      <c r="O87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -4351,6 +4796,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L88" t="inlineStr"/>
+      <c r="M88" t="inlineStr"/>
+      <c r="N88" t="inlineStr"/>
+      <c r="O88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -4366,6 +4815,7 @@
           <t>B-09 FAZ SANTA ROSA AURELIO</t>
         </is>
       </c>
+      <c r="D89" t="inlineStr"/>
       <c r="E89" t="inlineStr">
         <is>
           <t>18/09/2026</t>
@@ -4384,11 +4834,17 @@
       <c r="H89" t="n">
         <v>552.0599999999999</v>
       </c>
+      <c r="I89" t="inlineStr"/>
+      <c r="J89" t="inlineStr"/>
       <c r="K89" t="inlineStr">
         <is>
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L89" t="inlineStr"/>
+      <c r="M89" t="inlineStr"/>
+      <c r="N89" t="inlineStr"/>
+      <c r="O89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -4404,6 +4860,7 @@
           <t>B-24 CENTRO RURAL</t>
         </is>
       </c>
+      <c r="D90" t="inlineStr"/>
       <c r="E90" t="inlineStr">
         <is>
           <t>11/09/2026</t>
@@ -4414,7 +4871,7 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="G90" s="2" t="n">
+      <c r="G90" s="1" t="n">
         <v>46286</v>
       </c>
       <c r="H90" t="n">
@@ -4428,6 +4885,11 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="K90" t="inlineStr"/>
+      <c r="L90" t="inlineStr"/>
+      <c r="M90" t="inlineStr"/>
+      <c r="N90" t="inlineStr"/>
+      <c r="O90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -4458,7 +4920,7 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="G91" s="2" t="n">
+      <c r="G91" s="1" t="n">
         <v>46286</v>
       </c>
       <c r="H91" t="n">
@@ -4477,6 +4939,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L91" t="inlineStr"/>
+      <c r="M91" t="inlineStr"/>
+      <c r="N91" t="inlineStr"/>
+      <c r="O91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -4507,7 +4973,7 @@
           <t>FEITO</t>
         </is>
       </c>
-      <c r="G92" s="2" t="n">
+      <c r="G92" s="1" t="n">
         <v>46286</v>
       </c>
       <c r="H92" t="n">
@@ -4526,6 +4992,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L92" t="inlineStr"/>
+      <c r="M92" t="inlineStr"/>
+      <c r="N92" t="inlineStr"/>
+      <c r="O92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -4541,6 +5011,7 @@
           <t>B-23 FAZ NOSSA SENHORA APARECIDA</t>
         </is>
       </c>
+      <c r="D93" t="inlineStr"/>
       <c r="E93" t="inlineStr">
         <is>
           <t>21/09/2026</t>
@@ -4572,6 +5043,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L93" t="inlineStr"/>
+      <c r="M93" t="inlineStr"/>
+      <c r="N93" t="inlineStr"/>
+      <c r="O93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -4623,6 +5098,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L94" t="inlineStr"/>
+      <c r="M94" t="inlineStr"/>
+      <c r="N94" t="inlineStr"/>
+      <c r="O94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -4638,6 +5117,7 @@
           <t>B-23 FAZ NOSSA SENHORA APARECIDA</t>
         </is>
       </c>
+      <c r="D95" t="inlineStr"/>
       <c r="E95" t="inlineStr">
         <is>
           <t>21/09/2026</t>
@@ -4653,6 +5133,7 @@
           <t>24/07/2026</t>
         </is>
       </c>
+      <c r="H95" t="inlineStr"/>
       <c r="I95" t="n">
         <v>82.73999999999999</v>
       </c>
@@ -4661,6 +5142,11 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="K95" t="inlineStr"/>
+      <c r="L95" t="inlineStr"/>
+      <c r="M95" t="inlineStr"/>
+      <c r="N95" t="inlineStr"/>
+      <c r="O95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -4676,6 +5162,7 @@
           <t>B-016 FAZ RODA VIVA</t>
         </is>
       </c>
+      <c r="D96" t="inlineStr"/>
       <c r="E96" t="inlineStr">
         <is>
           <t>24/09/2026</t>
@@ -4694,11 +5181,17 @@
       <c r="H96" t="n">
         <v>345.05</v>
       </c>
+      <c r="I96" t="inlineStr"/>
+      <c r="J96" t="inlineStr"/>
       <c r="K96" t="inlineStr">
         <is>
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L96" t="inlineStr"/>
+      <c r="M96" t="inlineStr"/>
+      <c r="N96" t="inlineStr"/>
+      <c r="O96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -4745,6 +5238,11 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="K97" t="inlineStr"/>
+      <c r="L97" t="inlineStr"/>
+      <c r="M97" t="inlineStr"/>
+      <c r="N97" t="inlineStr"/>
+      <c r="O97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -4791,6 +5289,11 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="K98" t="inlineStr"/>
+      <c r="L98" t="inlineStr"/>
+      <c r="M98" t="inlineStr"/>
+      <c r="N98" t="inlineStr"/>
+      <c r="O98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -4837,6 +5340,11 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="K99" t="inlineStr"/>
+      <c r="L99" t="inlineStr"/>
+      <c r="M99" t="inlineStr"/>
+      <c r="N99" t="inlineStr"/>
+      <c r="O99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -4883,6 +5391,11 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="K100" t="inlineStr"/>
+      <c r="L100" t="inlineStr"/>
+      <c r="M100" t="inlineStr"/>
+      <c r="N100" t="inlineStr"/>
+      <c r="O100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -4898,6 +5411,7 @@
           <t>B-04 HARAS BILAC</t>
         </is>
       </c>
+      <c r="D101" t="inlineStr"/>
       <c r="E101" t="inlineStr">
         <is>
           <t>23/09/2026</t>
@@ -4929,6 +5443,10 @@
           <t>FEITO</t>
         </is>
       </c>
+      <c r="L101" t="inlineStr"/>
+      <c r="M101" t="inlineStr"/>
+      <c r="N101" t="inlineStr"/>
+      <c r="O101" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -19792,6 +20310,7 @@
       <c r="E391" t="n">
         <v>18.47</v>
       </c>
+      <c r="F391" t="inlineStr"/>
       <c r="G391" t="n">
         <v>0</v>
       </c>
@@ -19825,6 +20344,7 @@
       <c r="E392" t="n">
         <v>10.7</v>
       </c>
+      <c r="F392" t="inlineStr"/>
       <c r="G392" t="n">
         <v>0</v>
       </c>
@@ -19858,6 +20378,7 @@
       <c r="E393" t="n">
         <v>3.89</v>
       </c>
+      <c r="F393" t="inlineStr"/>
       <c r="G393" t="n">
         <v>0</v>
       </c>
@@ -23264,10 +23785,10 @@
         <v>7151.915000000001</v>
       </c>
       <c r="F9" t="n">
-        <v>108.19</v>
+        <v>121.12</v>
       </c>
       <c r="G9" t="n">
-        <v>634.3399999999999</v>
+        <v>647.2699999999999</v>
       </c>
     </row>
     <row r="10">
@@ -23293,10 +23814,10 @@
         <v>9006.105000000001</v>
       </c>
       <c r="F10" t="n">
-        <v>108.19</v>
+        <v>121.12</v>
       </c>
       <c r="G10" t="n">
-        <v>634.3399999999999</v>
+        <v>647.2699999999999</v>
       </c>
     </row>
     <row r="11">
@@ -23484,7 +24005,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:A2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23493,20 +24014,10 @@
           <t>creditos_inforow</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>senha_acesso</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
         <v>11121.66</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Clealco@Geo2026</t>
-        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
revert: restaurar icones oficiais anteriores e aprimorar instalacao do app PWA no celular
</commit_message>
<xml_diff>
--- a/dados.xlsx
+++ b/dados.xlsx
@@ -5534,7 +5534,7 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -5572,7 +5572,7 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -5610,7 +5610,7 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -5648,7 +5648,7 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -5686,7 +5686,7 @@
         </is>
       </c>
       <c r="G6" t="n">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -5724,7 +5724,7 @@
         </is>
       </c>
       <c r="G7" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -5762,7 +5762,7 @@
         </is>
       </c>
       <c r="G8" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -5800,7 +5800,7 @@
         </is>
       </c>
       <c r="G9" t="n">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -5838,7 +5838,7 @@
         </is>
       </c>
       <c r="G10" t="n">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -5876,7 +5876,7 @@
         </is>
       </c>
       <c r="G11" t="n">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -5914,7 +5914,7 @@
         </is>
       </c>
       <c r="G12" t="n">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -5952,7 +5952,7 @@
         </is>
       </c>
       <c r="G13" t="n">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -5990,7 +5990,7 @@
         </is>
       </c>
       <c r="G14" t="n">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
@@ -6028,7 +6028,7 @@
         </is>
       </c>
       <c r="G15" t="n">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -6066,7 +6066,7 @@
         </is>
       </c>
       <c r="G16" t="n">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -6104,7 +6104,7 @@
         </is>
       </c>
       <c r="G17" t="n">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
@@ -6142,7 +6142,7 @@
         </is>
       </c>
       <c r="G18" t="n">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
@@ -6180,7 +6180,7 @@
         </is>
       </c>
       <c r="G19" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -6218,7 +6218,7 @@
         </is>
       </c>
       <c r="G20" t="n">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -6256,7 +6256,7 @@
         </is>
       </c>
       <c r="G21" t="n">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
@@ -6294,7 +6294,7 @@
         </is>
       </c>
       <c r="G22" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
@@ -6332,7 +6332,7 @@
         </is>
       </c>
       <c r="G23" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
@@ -6370,7 +6370,7 @@
         </is>
       </c>
       <c r="G24" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
@@ -6408,7 +6408,7 @@
         </is>
       </c>
       <c r="G25" t="n">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
@@ -6446,7 +6446,7 @@
         </is>
       </c>
       <c r="G26" t="n">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
@@ -6484,7 +6484,7 @@
         </is>
       </c>
       <c r="G27" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
@@ -6522,7 +6522,7 @@
         </is>
       </c>
       <c r="G28" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
@@ -6560,7 +6560,7 @@
         </is>
       </c>
       <c r="G29" t="n">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="H29" t="inlineStr">
         <is>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="G30" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
@@ -6636,7 +6636,7 @@
         </is>
       </c>
       <c r="G31" t="n">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
@@ -6674,7 +6674,7 @@
         </is>
       </c>
       <c r="G32" t="n">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="H32" t="inlineStr">
         <is>
@@ -6712,7 +6712,7 @@
         </is>
       </c>
       <c r="G33" t="n">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H33" t="inlineStr">
         <is>
@@ -6750,7 +6750,7 @@
         </is>
       </c>
       <c r="G34" t="n">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>
@@ -6788,7 +6788,7 @@
         </is>
       </c>
       <c r="G35" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
@@ -6826,7 +6826,7 @@
         </is>
       </c>
       <c r="G36" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
@@ -6864,7 +6864,7 @@
         </is>
       </c>
       <c r="G37" t="n">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
@@ -6902,7 +6902,7 @@
         </is>
       </c>
       <c r="G38" t="n">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="H38" t="inlineStr">
         <is>
@@ -6940,7 +6940,7 @@
         </is>
       </c>
       <c r="G39" t="n">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
@@ -6978,7 +6978,7 @@
         </is>
       </c>
       <c r="G40" t="n">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
@@ -7016,7 +7016,7 @@
         </is>
       </c>
       <c r="G41" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
@@ -7054,7 +7054,7 @@
         </is>
       </c>
       <c r="G42" t="n">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
@@ -7092,7 +7092,7 @@
         </is>
       </c>
       <c r="G43" t="n">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
@@ -7130,7 +7130,7 @@
         </is>
       </c>
       <c r="G44" t="n">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="H44" t="inlineStr">
         <is>
@@ -7168,7 +7168,7 @@
         </is>
       </c>
       <c r="G45" t="n">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>
@@ -7206,7 +7206,7 @@
         </is>
       </c>
       <c r="G46" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H46" t="inlineStr">
         <is>
@@ -7244,7 +7244,7 @@
         </is>
       </c>
       <c r="G47" t="n">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="H47" t="inlineStr">
         <is>
@@ -7282,7 +7282,7 @@
         </is>
       </c>
       <c r="G48" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="H48" t="inlineStr">
         <is>
@@ -7320,7 +7320,7 @@
         </is>
       </c>
       <c r="G49" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H49" t="inlineStr">
         <is>
@@ -7358,7 +7358,7 @@
         </is>
       </c>
       <c r="G50" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H50" t="inlineStr">
         <is>
@@ -7396,7 +7396,7 @@
         </is>
       </c>
       <c r="G51" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H51" t="inlineStr">
         <is>
@@ -7434,7 +7434,7 @@
         </is>
       </c>
       <c r="G52" t="n">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="H52" t="inlineStr">
         <is>
@@ -7472,7 +7472,7 @@
         </is>
       </c>
       <c r="G53" t="n">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H53" t="inlineStr">
         <is>
@@ -7510,7 +7510,7 @@
         </is>
       </c>
       <c r="G54" t="n">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="H54" t="inlineStr">
         <is>
@@ -7548,7 +7548,7 @@
         </is>
       </c>
       <c r="G55" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="H55" t="inlineStr">
         <is>
@@ -7586,7 +7586,7 @@
         </is>
       </c>
       <c r="G56" t="n">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="H56" t="inlineStr">
         <is>
@@ -7624,7 +7624,7 @@
         </is>
       </c>
       <c r="G57" t="n">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="H57" t="inlineStr">
         <is>
@@ -7662,7 +7662,7 @@
         </is>
       </c>
       <c r="G58" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="H58" t="inlineStr">
         <is>
@@ -7700,7 +7700,7 @@
         </is>
       </c>
       <c r="G59" t="n">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="H59" t="inlineStr">
         <is>
@@ -7738,7 +7738,7 @@
         </is>
       </c>
       <c r="G60" t="n">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="H60" t="inlineStr">
         <is>
@@ -7776,7 +7776,7 @@
         </is>
       </c>
       <c r="G61" t="n">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="H61" t="inlineStr">
         <is>
@@ -7814,7 +7814,7 @@
         </is>
       </c>
       <c r="G62" t="n">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="H62" t="inlineStr">
         <is>
@@ -7852,7 +7852,7 @@
         </is>
       </c>
       <c r="G63" t="n">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H63" t="inlineStr">
         <is>
@@ -7890,7 +7890,7 @@
         </is>
       </c>
       <c r="G64" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H64" t="inlineStr">
         <is>
@@ -7928,7 +7928,7 @@
         </is>
       </c>
       <c r="G65" t="n">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="H65" t="inlineStr">
         <is>
@@ -7966,7 +7966,7 @@
         </is>
       </c>
       <c r="G66" t="n">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="H66" t="inlineStr">
         <is>
@@ -8004,7 +8004,7 @@
         </is>
       </c>
       <c r="G67" t="n">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="H67" t="inlineStr">
         <is>
@@ -8042,7 +8042,7 @@
         </is>
       </c>
       <c r="G68" t="n">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="H68" t="inlineStr">
         <is>
@@ -8080,7 +8080,7 @@
         </is>
       </c>
       <c r="G69" t="n">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H69" t="inlineStr">
         <is>
@@ -8118,7 +8118,7 @@
         </is>
       </c>
       <c r="G70" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="H70" t="inlineStr">
         <is>
@@ -8156,7 +8156,7 @@
         </is>
       </c>
       <c r="G71" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H71" t="inlineStr">
         <is>
@@ -8194,7 +8194,7 @@
         </is>
       </c>
       <c r="G72" t="n">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H72" t="inlineStr">
         <is>
@@ -8232,7 +8232,7 @@
         </is>
       </c>
       <c r="G73" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H73" t="inlineStr">
         <is>
@@ -8270,7 +8270,7 @@
         </is>
       </c>
       <c r="G74" t="n">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H74" t="inlineStr">
         <is>
@@ -8308,7 +8308,7 @@
         </is>
       </c>
       <c r="G75" t="n">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="H75" t="inlineStr">
         <is>
@@ -8346,7 +8346,7 @@
         </is>
       </c>
       <c r="G76" t="n">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H76" t="inlineStr">
         <is>
@@ -8384,7 +8384,7 @@
         </is>
       </c>
       <c r="G77" t="n">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="H77" t="inlineStr">
         <is>
@@ -8422,7 +8422,7 @@
         </is>
       </c>
       <c r="G78" t="n">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="H78" t="inlineStr">
         <is>
@@ -8460,7 +8460,7 @@
         </is>
       </c>
       <c r="G79" t="n">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H79" t="inlineStr">
         <is>
@@ -8498,7 +8498,7 @@
         </is>
       </c>
       <c r="G80" t="n">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="H80" t="inlineStr">
         <is>
@@ -8536,7 +8536,7 @@
         </is>
       </c>
       <c r="G81" t="n">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="H81" t="inlineStr">
         <is>
@@ -8574,7 +8574,7 @@
         </is>
       </c>
       <c r="G82" t="n">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="H82" t="inlineStr">
         <is>
@@ -8612,7 +8612,7 @@
         </is>
       </c>
       <c r="G83" t="n">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="H83" t="inlineStr">
         <is>
@@ -8650,7 +8650,7 @@
         </is>
       </c>
       <c r="G84" t="n">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H84" t="inlineStr">
         <is>
@@ -8688,7 +8688,7 @@
         </is>
       </c>
       <c r="G85" t="n">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H85" t="inlineStr">
         <is>
@@ -8726,7 +8726,7 @@
         </is>
       </c>
       <c r="G86" t="n">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H86" t="inlineStr">
         <is>
@@ -8764,7 +8764,7 @@
         </is>
       </c>
       <c r="G87" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="H87" t="inlineStr">
         <is>
@@ -8802,7 +8802,7 @@
         </is>
       </c>
       <c r="G88" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H88" t="inlineStr">
         <is>
@@ -8840,7 +8840,7 @@
         </is>
       </c>
       <c r="G89" t="n">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H89" t="inlineStr">
         <is>
@@ -8878,7 +8878,7 @@
         </is>
       </c>
       <c r="G90" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H90" t="inlineStr">
         <is>
@@ -8916,7 +8916,7 @@
         </is>
       </c>
       <c r="G91" t="n">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="H91" t="inlineStr">
         <is>
@@ -8954,7 +8954,7 @@
         </is>
       </c>
       <c r="G92" t="n">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="H92" t="inlineStr">
         <is>
@@ -8992,7 +8992,7 @@
         </is>
       </c>
       <c r="G93" t="n">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="H93" t="inlineStr">
         <is>
@@ -9030,7 +9030,7 @@
         </is>
       </c>
       <c r="G94" t="n">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="H94" t="inlineStr">
         <is>
@@ -9068,7 +9068,7 @@
         </is>
       </c>
       <c r="G95" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H95" t="inlineStr">
         <is>
@@ -9106,7 +9106,7 @@
         </is>
       </c>
       <c r="G96" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H96" t="inlineStr">
         <is>
@@ -9144,7 +9144,7 @@
         </is>
       </c>
       <c r="G97" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H97" t="inlineStr">
         <is>
@@ -9182,7 +9182,7 @@
         </is>
       </c>
       <c r="G98" t="n">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="H98" t="inlineStr">
         <is>
@@ -9220,7 +9220,7 @@
         </is>
       </c>
       <c r="G99" t="n">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H99" t="inlineStr">
         <is>
@@ -9258,7 +9258,7 @@
         </is>
       </c>
       <c r="G100" t="n">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="H100" t="inlineStr">
         <is>
@@ -9296,7 +9296,7 @@
         </is>
       </c>
       <c r="G101" t="n">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H101" t="inlineStr">
         <is>
@@ -9334,7 +9334,7 @@
         </is>
       </c>
       <c r="G102" t="n">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H102" t="inlineStr">
         <is>
@@ -9372,7 +9372,7 @@
         </is>
       </c>
       <c r="G103" t="n">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H103" t="inlineStr">
         <is>
@@ -9410,7 +9410,7 @@
         </is>
       </c>
       <c r="G104" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="H104" t="inlineStr">
         <is>
@@ -9448,7 +9448,7 @@
         </is>
       </c>
       <c r="G105" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H105" t="inlineStr">
         <is>
@@ -9486,7 +9486,7 @@
         </is>
       </c>
       <c r="G106" t="n">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="H106" t="inlineStr">
         <is>
@@ -9524,7 +9524,7 @@
         </is>
       </c>
       <c r="G107" t="n">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="H107" t="inlineStr">
         <is>
@@ -9562,7 +9562,7 @@
         </is>
       </c>
       <c r="G108" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H108" t="inlineStr">
         <is>
@@ -9600,7 +9600,7 @@
         </is>
       </c>
       <c r="G109" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="H109" t="inlineStr">
         <is>
@@ -9638,7 +9638,7 @@
         </is>
       </c>
       <c r="G110" t="n">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H110" t="inlineStr">
         <is>
@@ -9676,7 +9676,7 @@
         </is>
       </c>
       <c r="G111" t="n">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="H111" t="inlineStr">
         <is>
@@ -9714,7 +9714,7 @@
         </is>
       </c>
       <c r="G112" t="n">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H112" t="inlineStr">
         <is>
@@ -9752,7 +9752,7 @@
         </is>
       </c>
       <c r="G113" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H113" t="inlineStr">
         <is>
@@ -9790,7 +9790,7 @@
         </is>
       </c>
       <c r="G114" t="n">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="H114" t="inlineStr">
         <is>
@@ -9828,7 +9828,7 @@
         </is>
       </c>
       <c r="G115" t="n">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H115" t="inlineStr">
         <is>
@@ -9866,7 +9866,7 @@
         </is>
       </c>
       <c r="G116" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="H116" t="inlineStr">
         <is>
@@ -9904,7 +9904,7 @@
         </is>
       </c>
       <c r="G117" t="n">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="H117" t="inlineStr">
         <is>
@@ -9942,7 +9942,7 @@
         </is>
       </c>
       <c r="G118" t="n">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="H118" t="inlineStr">
         <is>
@@ -9980,7 +9980,7 @@
         </is>
       </c>
       <c r="G119" t="n">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="H119" t="inlineStr">
         <is>
@@ -10018,7 +10018,7 @@
         </is>
       </c>
       <c r="G120" t="n">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H120" t="inlineStr">
         <is>
@@ -10056,7 +10056,7 @@
         </is>
       </c>
       <c r="G121" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H121" t="inlineStr">
         <is>
@@ -10094,7 +10094,7 @@
         </is>
       </c>
       <c r="G122" t="n">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="H122" t="inlineStr">
         <is>
@@ -10132,7 +10132,7 @@
         </is>
       </c>
       <c r="G123" t="n">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H123" t="inlineStr">
         <is>
@@ -10170,7 +10170,7 @@
         </is>
       </c>
       <c r="G124" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H124" t="inlineStr">
         <is>
@@ -10208,7 +10208,7 @@
         </is>
       </c>
       <c r="G125" t="n">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="H125" t="inlineStr">
         <is>
@@ -10246,7 +10246,7 @@
         </is>
       </c>
       <c r="G126" t="n">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="H126" t="inlineStr">
         <is>
@@ -10284,7 +10284,7 @@
         </is>
       </c>
       <c r="G127" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H127" t="inlineStr">
         <is>
@@ -10322,7 +10322,7 @@
         </is>
       </c>
       <c r="G128" t="n">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H128" t="inlineStr">
         <is>
@@ -10360,7 +10360,7 @@
         </is>
       </c>
       <c r="G129" t="n">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H129" t="inlineStr">
         <is>
@@ -10398,7 +10398,7 @@
         </is>
       </c>
       <c r="G130" t="n">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="H130" t="inlineStr">
         <is>
@@ -10436,7 +10436,7 @@
         </is>
       </c>
       <c r="G131" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H131" t="inlineStr">
         <is>
@@ -10474,7 +10474,7 @@
         </is>
       </c>
       <c r="G132" t="n">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="H132" t="inlineStr">
         <is>
@@ -10512,7 +10512,7 @@
         </is>
       </c>
       <c r="G133" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H133" t="inlineStr">
         <is>
@@ -10550,7 +10550,7 @@
         </is>
       </c>
       <c r="G134" t="n">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H134" t="inlineStr">
         <is>
@@ -10588,7 +10588,7 @@
         </is>
       </c>
       <c r="G135" t="n">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="H135" t="inlineStr">
         <is>
@@ -10626,7 +10626,7 @@
         </is>
       </c>
       <c r="G136" t="n">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="H136" t="inlineStr">
         <is>
@@ -10664,7 +10664,7 @@
         </is>
       </c>
       <c r="G137" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H137" t="inlineStr">
         <is>
@@ -10702,7 +10702,7 @@
         </is>
       </c>
       <c r="G138" t="n">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="H138" t="inlineStr">
         <is>
@@ -10740,7 +10740,7 @@
         </is>
       </c>
       <c r="G139" t="n">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="H139" t="inlineStr">
         <is>
@@ -10778,7 +10778,7 @@
         </is>
       </c>
       <c r="G140" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H140" t="inlineStr">
         <is>
@@ -10816,7 +10816,7 @@
         </is>
       </c>
       <c r="G141" t="n">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H141" t="inlineStr">
         <is>
@@ -10854,7 +10854,7 @@
         </is>
       </c>
       <c r="G142" t="n">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H142" t="inlineStr">
         <is>
@@ -10892,7 +10892,7 @@
         </is>
       </c>
       <c r="G143" t="n">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H143" t="inlineStr">
         <is>
@@ -10930,7 +10930,7 @@
         </is>
       </c>
       <c r="G144" t="n">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="H144" t="inlineStr">
         <is>
@@ -10968,7 +10968,7 @@
         </is>
       </c>
       <c r="G145" t="n">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="H145" t="inlineStr">
         <is>
@@ -11006,7 +11006,7 @@
         </is>
       </c>
       <c r="G146" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="H146" t="inlineStr">
         <is>
@@ -11044,7 +11044,7 @@
         </is>
       </c>
       <c r="G147" t="n">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="H147" t="inlineStr">
         <is>
@@ -11082,7 +11082,7 @@
         </is>
       </c>
       <c r="G148" t="n">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="H148" t="inlineStr">
         <is>
@@ -11120,7 +11120,7 @@
         </is>
       </c>
       <c r="G149" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="H149" t="inlineStr">
         <is>
@@ -11158,7 +11158,7 @@
         </is>
       </c>
       <c r="G150" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H150" t="inlineStr">
         <is>
@@ -11196,7 +11196,7 @@
         </is>
       </c>
       <c r="G151" t="n">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="H151" t="inlineStr">
         <is>
@@ -11234,7 +11234,7 @@
         </is>
       </c>
       <c r="G152" t="n">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="H152" t="inlineStr">
         <is>
@@ -11272,7 +11272,7 @@
         </is>
       </c>
       <c r="G153" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H153" t="inlineStr">
         <is>
@@ -11310,7 +11310,7 @@
         </is>
       </c>
       <c r="G154" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H154" t="inlineStr">
         <is>
@@ -11348,7 +11348,7 @@
         </is>
       </c>
       <c r="G155" t="n">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="H155" t="inlineStr">
         <is>
@@ -11386,7 +11386,7 @@
         </is>
       </c>
       <c r="G156" t="n">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="H156" t="inlineStr">
         <is>
@@ -11424,7 +11424,7 @@
         </is>
       </c>
       <c r="G157" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H157" t="inlineStr">
         <is>
@@ -11462,7 +11462,7 @@
         </is>
       </c>
       <c r="G158" t="n">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H158" t="inlineStr">
         <is>
@@ -11500,7 +11500,7 @@
         </is>
       </c>
       <c r="G159" t="n">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H159" t="inlineStr">
         <is>
@@ -11538,7 +11538,7 @@
         </is>
       </c>
       <c r="G160" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H160" t="inlineStr">
         <is>
@@ -11576,7 +11576,7 @@
         </is>
       </c>
       <c r="G161" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H161" t="inlineStr">
         <is>
@@ -11614,7 +11614,7 @@
         </is>
       </c>
       <c r="G162" t="n">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H162" t="inlineStr">
         <is>
@@ -11652,7 +11652,7 @@
         </is>
       </c>
       <c r="G163" t="n">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="H163" t="inlineStr">
         <is>
@@ -11690,7 +11690,7 @@
         </is>
       </c>
       <c r="G164" t="n">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H164" t="inlineStr">
         <is>
@@ -11728,7 +11728,7 @@
         </is>
       </c>
       <c r="G165" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H165" t="inlineStr">
         <is>
@@ -11766,7 +11766,7 @@
         </is>
       </c>
       <c r="G166" t="n">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="H166" t="inlineStr">
         <is>
@@ -11804,7 +11804,7 @@
         </is>
       </c>
       <c r="G167" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H167" t="inlineStr">
         <is>
@@ -11842,7 +11842,7 @@
         </is>
       </c>
       <c r="G168" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H168" t="inlineStr">
         <is>
@@ -11880,7 +11880,7 @@
         </is>
       </c>
       <c r="G169" t="n">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H169" t="inlineStr">
         <is>
@@ -11918,7 +11918,7 @@
         </is>
       </c>
       <c r="G170" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H170" t="inlineStr">
         <is>
@@ -11956,7 +11956,7 @@
         </is>
       </c>
       <c r="G171" t="n">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="H171" t="inlineStr">
         <is>
@@ -11994,7 +11994,7 @@
         </is>
       </c>
       <c r="G172" t="n">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="H172" t="inlineStr">
         <is>
@@ -12032,7 +12032,7 @@
         </is>
       </c>
       <c r="G173" t="n">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="H173" t="inlineStr">
         <is>
@@ -12070,7 +12070,7 @@
         </is>
       </c>
       <c r="G174" t="n">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="H174" t="inlineStr">
         <is>
@@ -12108,7 +12108,7 @@
         </is>
       </c>
       <c r="G175" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H175" t="inlineStr">
         <is>
@@ -12146,7 +12146,7 @@
         </is>
       </c>
       <c r="G176" t="n">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="H176" t="inlineStr">
         <is>
@@ -12184,7 +12184,7 @@
         </is>
       </c>
       <c r="G177" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H177" t="inlineStr">
         <is>
@@ -12222,7 +12222,7 @@
         </is>
       </c>
       <c r="G178" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H178" t="inlineStr">
         <is>
@@ -12260,7 +12260,7 @@
         </is>
       </c>
       <c r="G179" t="n">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H179" t="inlineStr">
         <is>
@@ -12298,7 +12298,7 @@
         </is>
       </c>
       <c r="G180" t="n">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="H180" t="inlineStr">
         <is>
@@ -12336,7 +12336,7 @@
         </is>
       </c>
       <c r="G181" t="n">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="H181" t="inlineStr">
         <is>
@@ -12374,7 +12374,7 @@
         </is>
       </c>
       <c r="G182" t="n">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="H182" t="inlineStr">
         <is>
@@ -12412,7 +12412,7 @@
         </is>
       </c>
       <c r="G183" t="n">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="H183" t="inlineStr">
         <is>
@@ -12450,7 +12450,7 @@
         </is>
       </c>
       <c r="G184" t="n">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H184" t="inlineStr">
         <is>
@@ -12488,7 +12488,7 @@
         </is>
       </c>
       <c r="G185" t="n">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H185" t="inlineStr">
         <is>
@@ -12526,7 +12526,7 @@
         </is>
       </c>
       <c r="G186" t="n">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H186" t="inlineStr">
         <is>
@@ -12564,7 +12564,7 @@
         </is>
       </c>
       <c r="G187" t="n">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="H187" t="inlineStr">
         <is>
@@ -12602,7 +12602,7 @@
         </is>
       </c>
       <c r="G188" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H188" t="inlineStr">
         <is>
@@ -12640,7 +12640,7 @@
         </is>
       </c>
       <c r="G189" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H189" t="inlineStr">
         <is>
@@ -12678,7 +12678,7 @@
         </is>
       </c>
       <c r="G190" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H190" t="inlineStr">
         <is>
@@ -12716,7 +12716,7 @@
         </is>
       </c>
       <c r="G191" t="n">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H191" t="inlineStr">
         <is>
@@ -12754,7 +12754,7 @@
         </is>
       </c>
       <c r="G192" t="n">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="H192" t="inlineStr">
         <is>
@@ -12792,7 +12792,7 @@
         </is>
       </c>
       <c r="G193" t="n">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H193" t="inlineStr">
         <is>
@@ -12830,7 +12830,7 @@
         </is>
       </c>
       <c r="G194" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H194" t="inlineStr">
         <is>
@@ -12868,7 +12868,7 @@
         </is>
       </c>
       <c r="G195" t="n">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="H195" t="inlineStr">
         <is>
@@ -12906,7 +12906,7 @@
         </is>
       </c>
       <c r="G196" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H196" t="inlineStr">
         <is>
@@ -12944,7 +12944,7 @@
         </is>
       </c>
       <c r="G197" t="n">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="H197" t="inlineStr">
         <is>
@@ -12982,7 +12982,7 @@
         </is>
       </c>
       <c r="G198" t="n">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H198" t="inlineStr">
         <is>
@@ -13020,7 +13020,7 @@
         </is>
       </c>
       <c r="G199" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="H199" t="inlineStr">
         <is>
@@ -13058,7 +13058,7 @@
         </is>
       </c>
       <c r="G200" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H200" t="inlineStr">
         <is>
@@ -13096,7 +13096,7 @@
         </is>
       </c>
       <c r="G201" t="n">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H201" t="inlineStr">
         <is>
@@ -13134,7 +13134,7 @@
         </is>
       </c>
       <c r="G202" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H202" t="inlineStr">
         <is>
@@ -13172,7 +13172,7 @@
         </is>
       </c>
       <c r="G203" t="n">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="H203" t="inlineStr">
         <is>
@@ -13210,7 +13210,7 @@
         </is>
       </c>
       <c r="G204" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H204" t="inlineStr">
         <is>
@@ -13248,7 +13248,7 @@
         </is>
       </c>
       <c r="G205" t="n">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="H205" t="inlineStr">
         <is>
@@ -13286,7 +13286,7 @@
         </is>
       </c>
       <c r="G206" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="H206" t="inlineStr">
         <is>
@@ -13324,7 +13324,7 @@
         </is>
       </c>
       <c r="G207" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H207" t="inlineStr">
         <is>
@@ -13362,7 +13362,7 @@
         </is>
       </c>
       <c r="G208" t="n">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="H208" t="inlineStr">
         <is>
@@ -13400,7 +13400,7 @@
         </is>
       </c>
       <c r="G209" t="n">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="H209" t="inlineStr">
         <is>
@@ -13438,7 +13438,7 @@
         </is>
       </c>
       <c r="G210" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H210" t="inlineStr">
         <is>
@@ -13476,7 +13476,7 @@
         </is>
       </c>
       <c r="G211" t="n">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="H211" t="inlineStr">
         <is>
@@ -13514,7 +13514,7 @@
         </is>
       </c>
       <c r="G212" t="n">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="H212" t="inlineStr">
         <is>
@@ -13552,7 +13552,7 @@
         </is>
       </c>
       <c r="G213" t="n">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="H213" t="inlineStr">
         <is>
@@ -13590,7 +13590,7 @@
         </is>
       </c>
       <c r="G214" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H214" t="inlineStr">
         <is>
@@ -13628,7 +13628,7 @@
         </is>
       </c>
       <c r="G215" t="n">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H215" t="inlineStr">
         <is>
@@ -13666,7 +13666,7 @@
         </is>
       </c>
       <c r="G216" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H216" t="inlineStr">
         <is>
@@ -13704,7 +13704,7 @@
         </is>
       </c>
       <c r="G217" t="n">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="H217" t="inlineStr">
         <is>
@@ -13742,7 +13742,7 @@
         </is>
       </c>
       <c r="G218" t="n">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H218" t="inlineStr">
         <is>
@@ -13780,7 +13780,7 @@
         </is>
       </c>
       <c r="G219" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="H219" t="inlineStr">
         <is>
@@ -13818,7 +13818,7 @@
         </is>
       </c>
       <c r="G220" t="n">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H220" t="inlineStr">
         <is>
@@ -13856,7 +13856,7 @@
         </is>
       </c>
       <c r="G221" t="n">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="H221" t="inlineStr">
         <is>
@@ -13894,7 +13894,7 @@
         </is>
       </c>
       <c r="G222" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H222" t="inlineStr">
         <is>
@@ -13932,7 +13932,7 @@
         </is>
       </c>
       <c r="G223" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H223" t="inlineStr">
         <is>
@@ -13970,7 +13970,7 @@
         </is>
       </c>
       <c r="G224" t="n">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="H224" t="inlineStr">
         <is>
@@ -14008,7 +14008,7 @@
         </is>
       </c>
       <c r="G225" t="n">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="H225" t="inlineStr">
         <is>
@@ -14046,7 +14046,7 @@
         </is>
       </c>
       <c r="G226" t="n">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H226" t="inlineStr">
         <is>
@@ -14084,7 +14084,7 @@
         </is>
       </c>
       <c r="G227" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H227" t="inlineStr">
         <is>
@@ -14122,7 +14122,7 @@
         </is>
       </c>
       <c r="G228" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H228" t="inlineStr">
         <is>
@@ -14160,7 +14160,7 @@
         </is>
       </c>
       <c r="G229" t="n">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H229" t="inlineStr">
         <is>
@@ -14198,7 +14198,7 @@
         </is>
       </c>
       <c r="G230" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="H230" t="inlineStr">
         <is>
@@ -14236,7 +14236,7 @@
         </is>
       </c>
       <c r="G231" t="n">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H231" t="inlineStr">
         <is>
@@ -14274,7 +14274,7 @@
         </is>
       </c>
       <c r="G232" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="H232" t="inlineStr">
         <is>
@@ -14312,7 +14312,7 @@
         </is>
       </c>
       <c r="G233" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H233" t="inlineStr">
         <is>
@@ -14350,7 +14350,7 @@
         </is>
       </c>
       <c r="G234" t="n">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="H234" t="inlineStr">
         <is>
@@ -14388,7 +14388,7 @@
         </is>
       </c>
       <c r="G235" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H235" t="inlineStr">
         <is>
@@ -14426,7 +14426,7 @@
         </is>
       </c>
       <c r="G236" t="n">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="H236" t="inlineStr">
         <is>
@@ -14464,7 +14464,7 @@
         </is>
       </c>
       <c r="G237" t="n">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="H237" t="inlineStr">
         <is>
@@ -14502,7 +14502,7 @@
         </is>
       </c>
       <c r="G238" t="n">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="H238" t="inlineStr">
         <is>
@@ -14540,7 +14540,7 @@
         </is>
       </c>
       <c r="G239" t="n">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H239" t="inlineStr">
         <is>
@@ -14578,7 +14578,7 @@
         </is>
       </c>
       <c r="G240" t="n">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H240" t="inlineStr">
         <is>
@@ -14616,7 +14616,7 @@
         </is>
       </c>
       <c r="G241" t="n">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H241" t="inlineStr">
         <is>
@@ -14654,7 +14654,7 @@
         </is>
       </c>
       <c r="G242" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H242" t="inlineStr">
         <is>
@@ -14692,7 +14692,7 @@
         </is>
       </c>
       <c r="G243" t="n">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="H243" t="inlineStr">
         <is>
@@ -14730,7 +14730,7 @@
         </is>
       </c>
       <c r="G244" t="n">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="H244" t="inlineStr">
         <is>
@@ -14768,7 +14768,7 @@
         </is>
       </c>
       <c r="G245" t="n">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H245" t="inlineStr">
         <is>
@@ -14806,7 +14806,7 @@
         </is>
       </c>
       <c r="G246" t="n">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="H246" t="inlineStr">
         <is>
@@ -14844,7 +14844,7 @@
         </is>
       </c>
       <c r="G247" t="n">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="H247" t="inlineStr">
         <is>
@@ -14882,7 +14882,7 @@
         </is>
       </c>
       <c r="G248" t="n">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="H248" t="inlineStr">
         <is>
@@ -14920,7 +14920,7 @@
         </is>
       </c>
       <c r="G249" t="n">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="H249" t="inlineStr">
         <is>
@@ -14958,7 +14958,7 @@
         </is>
       </c>
       <c r="G250" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="H250" t="inlineStr">
         <is>
@@ -14996,7 +14996,7 @@
         </is>
       </c>
       <c r="G251" t="n">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="H251" t="inlineStr">
         <is>
@@ -15034,7 +15034,7 @@
         </is>
       </c>
       <c r="G252" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="H252" t="inlineStr">
         <is>
@@ -15072,7 +15072,7 @@
         </is>
       </c>
       <c r="G253" t="n">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="H253" t="inlineStr">
         <is>
@@ -15110,7 +15110,7 @@
         </is>
       </c>
       <c r="G254" t="n">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="H254" t="inlineStr">
         <is>
@@ -15148,7 +15148,7 @@
         </is>
       </c>
       <c r="G255" t="n">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="H255" t="inlineStr">
         <is>
@@ -15186,7 +15186,7 @@
         </is>
       </c>
       <c r="G256" t="n">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H256" t="inlineStr">
         <is>
@@ -15224,7 +15224,7 @@
         </is>
       </c>
       <c r="G257" t="n">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="H257" t="inlineStr">
         <is>
@@ -15262,7 +15262,7 @@
         </is>
       </c>
       <c r="G258" t="n">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H258" t="inlineStr">
         <is>
@@ -15300,7 +15300,7 @@
         </is>
       </c>
       <c r="G259" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H259" t="inlineStr">
         <is>
@@ -15338,7 +15338,7 @@
         </is>
       </c>
       <c r="G260" t="n">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="H260" t="inlineStr">
         <is>
@@ -15376,7 +15376,7 @@
         </is>
       </c>
       <c r="G261" t="n">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H261" t="inlineStr">
         <is>
@@ -15414,7 +15414,7 @@
         </is>
       </c>
       <c r="G262" t="n">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="H262" t="inlineStr">
         <is>
@@ -15452,7 +15452,7 @@
         </is>
       </c>
       <c r="G263" t="n">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="H263" t="inlineStr">
         <is>
@@ -15490,7 +15490,7 @@
         </is>
       </c>
       <c r="G264" t="n">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="H264" t="inlineStr">
         <is>
@@ -15528,7 +15528,7 @@
         </is>
       </c>
       <c r="G265" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H265" t="inlineStr">
         <is>
@@ -15566,7 +15566,7 @@
         </is>
       </c>
       <c r="G266" t="n">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H266" t="inlineStr">
         <is>
@@ -15604,7 +15604,7 @@
         </is>
       </c>
       <c r="G267" t="n">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="H267" t="inlineStr">
         <is>
@@ -15642,7 +15642,7 @@
         </is>
       </c>
       <c r="G268" t="n">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="H268" t="inlineStr">
         <is>
@@ -15680,7 +15680,7 @@
         </is>
       </c>
       <c r="G269" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H269" t="inlineStr">
         <is>
@@ -15718,7 +15718,7 @@
         </is>
       </c>
       <c r="G270" t="n">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H270" t="inlineStr">
         <is>
@@ -15756,7 +15756,7 @@
         </is>
       </c>
       <c r="G271" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H271" t="inlineStr">
         <is>
@@ -15794,7 +15794,7 @@
         </is>
       </c>
       <c r="G272" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="H272" t="inlineStr">
         <is>
@@ -15832,7 +15832,7 @@
         </is>
       </c>
       <c r="G273" t="n">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="H273" t="inlineStr">
         <is>
@@ -15870,7 +15870,7 @@
         </is>
       </c>
       <c r="G274" t="n">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="H274" t="inlineStr">
         <is>
@@ -15908,7 +15908,7 @@
         </is>
       </c>
       <c r="G275" t="n">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="H275" t="inlineStr">
         <is>
@@ -15946,7 +15946,7 @@
         </is>
       </c>
       <c r="G276" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="H276" t="inlineStr">
         <is>
@@ -15984,7 +15984,7 @@
         </is>
       </c>
       <c r="G277" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H277" t="inlineStr">
         <is>
@@ -16022,7 +16022,7 @@
         </is>
       </c>
       <c r="G278" t="n">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="H278" t="inlineStr">
         <is>
@@ -16060,7 +16060,7 @@
         </is>
       </c>
       <c r="G279" t="n">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H279" t="inlineStr">
         <is>
@@ -16098,7 +16098,7 @@
         </is>
       </c>
       <c r="G280" t="n">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="H280" t="inlineStr">
         <is>
@@ -16136,7 +16136,7 @@
         </is>
       </c>
       <c r="G281" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H281" t="inlineStr">
         <is>
@@ -16174,7 +16174,7 @@
         </is>
       </c>
       <c r="G282" t="n">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="H282" t="inlineStr">
         <is>
@@ -16212,7 +16212,7 @@
         </is>
       </c>
       <c r="G283" t="n">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H283" t="inlineStr">
         <is>
@@ -16250,7 +16250,7 @@
         </is>
       </c>
       <c r="G284" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H284" t="inlineStr">
         <is>
@@ -16288,7 +16288,7 @@
         </is>
       </c>
       <c r="G285" t="n">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="H285" t="inlineStr">
         <is>
@@ -16326,7 +16326,7 @@
         </is>
       </c>
       <c r="G286" t="n">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="H286" t="inlineStr">
         <is>
@@ -16364,7 +16364,7 @@
         </is>
       </c>
       <c r="G287" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H287" t="inlineStr">
         <is>
@@ -16402,7 +16402,7 @@
         </is>
       </c>
       <c r="G288" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="H288" t="inlineStr">
         <is>
@@ -16440,7 +16440,7 @@
         </is>
       </c>
       <c r="G289" t="n">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H289" t="inlineStr">
         <is>
@@ -16478,7 +16478,7 @@
         </is>
       </c>
       <c r="G290" t="n">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H290" t="inlineStr">
         <is>
@@ -16516,7 +16516,7 @@
         </is>
       </c>
       <c r="G291" t="n">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="H291" t="inlineStr">
         <is>
@@ -16554,7 +16554,7 @@
         </is>
       </c>
       <c r="G292" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="H292" t="inlineStr">
         <is>
@@ -16592,7 +16592,7 @@
         </is>
       </c>
       <c r="G293" t="n">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="H293" t="inlineStr">
         <is>
@@ -16630,7 +16630,7 @@
         </is>
       </c>
       <c r="G294" t="n">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="H294" t="inlineStr">
         <is>
@@ -16668,7 +16668,7 @@
         </is>
       </c>
       <c r="G295" t="n">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="H295" t="inlineStr">
         <is>
@@ -16706,7 +16706,7 @@
         </is>
       </c>
       <c r="G296" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H296" t="inlineStr">
         <is>
@@ -16744,7 +16744,7 @@
         </is>
       </c>
       <c r="G297" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H297" t="inlineStr">
         <is>
@@ -16782,7 +16782,7 @@
         </is>
       </c>
       <c r="G298" t="n">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="H298" t="inlineStr">
         <is>
@@ -16820,7 +16820,7 @@
         </is>
       </c>
       <c r="G299" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="H299" t="inlineStr">
         <is>
@@ -16858,7 +16858,7 @@
         </is>
       </c>
       <c r="G300" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="H300" t="inlineStr">
         <is>
@@ -16896,7 +16896,7 @@
         </is>
       </c>
       <c r="G301" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="H301" t="inlineStr">
         <is>
@@ -16934,7 +16934,7 @@
         </is>
       </c>
       <c r="G302" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="H302" t="inlineStr">
         <is>
@@ -16972,7 +16972,7 @@
         </is>
       </c>
       <c r="G303" t="n">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="H303" t="inlineStr">
         <is>
@@ -17010,7 +17010,7 @@
         </is>
       </c>
       <c r="G304" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H304" t="inlineStr">
         <is>
@@ -17048,7 +17048,7 @@
         </is>
       </c>
       <c r="G305" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H305" t="inlineStr">
         <is>
@@ -17086,7 +17086,7 @@
         </is>
       </c>
       <c r="G306" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H306" t="inlineStr">
         <is>
@@ -17124,7 +17124,7 @@
         </is>
       </c>
       <c r="G307" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H307" t="inlineStr">
         <is>
@@ -17162,7 +17162,7 @@
         </is>
       </c>
       <c r="G308" t="n">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="H308" t="inlineStr">
         <is>
@@ -17200,7 +17200,7 @@
         </is>
       </c>
       <c r="G309" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H309" t="inlineStr">
         <is>
@@ -17238,7 +17238,7 @@
         </is>
       </c>
       <c r="G310" t="n">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="H310" t="inlineStr">
         <is>
@@ -17276,7 +17276,7 @@
         </is>
       </c>
       <c r="G311" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="H311" t="inlineStr">
         <is>
@@ -17314,7 +17314,7 @@
         </is>
       </c>
       <c r="G312" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H312" t="inlineStr">
         <is>
@@ -17352,7 +17352,7 @@
         </is>
       </c>
       <c r="G313" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="H313" t="inlineStr">
         <is>
@@ -17390,7 +17390,7 @@
         </is>
       </c>
       <c r="G314" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H314" t="inlineStr">
         <is>
@@ -17428,7 +17428,7 @@
         </is>
       </c>
       <c r="G315" t="n">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H315" t="inlineStr">
         <is>
@@ -17466,7 +17466,7 @@
         </is>
       </c>
       <c r="G316" t="n">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="H316" t="inlineStr">
         <is>
@@ -17504,7 +17504,7 @@
         </is>
       </c>
       <c r="G317" t="n">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="H317" t="inlineStr">
         <is>
@@ -17542,7 +17542,7 @@
         </is>
       </c>
       <c r="G318" t="n">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="H318" t="inlineStr">
         <is>
@@ -17580,7 +17580,7 @@
         </is>
       </c>
       <c r="G319" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="H319" t="inlineStr">
         <is>
@@ -17618,7 +17618,7 @@
         </is>
       </c>
       <c r="G320" t="n">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="H320" t="inlineStr">
         <is>
@@ -17656,7 +17656,7 @@
         </is>
       </c>
       <c r="G321" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H321" t="inlineStr">
         <is>
@@ -17694,7 +17694,7 @@
         </is>
       </c>
       <c r="G322" t="n">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="H322" t="inlineStr">
         <is>
@@ -17732,7 +17732,7 @@
         </is>
       </c>
       <c r="G323" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H323" t="inlineStr">
         <is>
@@ -17770,7 +17770,7 @@
         </is>
       </c>
       <c r="G324" t="n">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="H324" t="inlineStr">
         <is>
@@ -17808,7 +17808,7 @@
         </is>
       </c>
       <c r="G325" t="n">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H325" t="inlineStr">
         <is>
@@ -17846,7 +17846,7 @@
         </is>
       </c>
       <c r="G326" t="n">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H326" t="inlineStr">
         <is>
@@ -17884,7 +17884,7 @@
         </is>
       </c>
       <c r="G327" t="n">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="H327" t="inlineStr">
         <is>
@@ -17922,7 +17922,7 @@
         </is>
       </c>
       <c r="G328" t="n">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="H328" t="inlineStr">
         <is>
@@ -17960,7 +17960,7 @@
         </is>
       </c>
       <c r="G329" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H329" t="inlineStr">
         <is>
@@ -17998,7 +17998,7 @@
         </is>
       </c>
       <c r="G330" t="n">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H330" t="inlineStr">
         <is>
@@ -18036,7 +18036,7 @@
         </is>
       </c>
       <c r="G331" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H331" t="inlineStr">
         <is>
@@ -18074,7 +18074,7 @@
         </is>
       </c>
       <c r="G332" t="n">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="H332" t="inlineStr">
         <is>
@@ -18112,7 +18112,7 @@
         </is>
       </c>
       <c r="G333" t="n">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="H333" t="inlineStr">
         <is>
@@ -18150,7 +18150,7 @@
         </is>
       </c>
       <c r="G334" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H334" t="inlineStr">
         <is>
@@ -18188,7 +18188,7 @@
         </is>
       </c>
       <c r="G335" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H335" t="inlineStr">
         <is>
@@ -18226,7 +18226,7 @@
         </is>
       </c>
       <c r="G336" t="n">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="H336" t="inlineStr">
         <is>
@@ -18264,7 +18264,7 @@
         </is>
       </c>
       <c r="G337" t="n">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="H337" t="inlineStr">
         <is>
@@ -18302,7 +18302,7 @@
         </is>
       </c>
       <c r="G338" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H338" t="inlineStr">
         <is>
@@ -18340,7 +18340,7 @@
         </is>
       </c>
       <c r="G339" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H339" t="inlineStr">
         <is>
@@ -18378,7 +18378,7 @@
         </is>
       </c>
       <c r="G340" t="n">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="H340" t="inlineStr">
         <is>
@@ -18416,7 +18416,7 @@
         </is>
       </c>
       <c r="G341" t="n">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="H341" t="inlineStr">
         <is>
@@ -18454,7 +18454,7 @@
         </is>
       </c>
       <c r="G342" t="n">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="H342" t="inlineStr">
         <is>
@@ -18492,7 +18492,7 @@
         </is>
       </c>
       <c r="G343" t="n">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H343" t="inlineStr">
         <is>
@@ -18530,7 +18530,7 @@
         </is>
       </c>
       <c r="G344" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H344" t="inlineStr">
         <is>
@@ -18568,7 +18568,7 @@
         </is>
       </c>
       <c r="G345" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H345" t="inlineStr">
         <is>
@@ -18606,7 +18606,7 @@
         </is>
       </c>
       <c r="G346" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H346" t="inlineStr">
         <is>
@@ -18644,7 +18644,7 @@
         </is>
       </c>
       <c r="G347" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H347" t="inlineStr">
         <is>
@@ -18682,7 +18682,7 @@
         </is>
       </c>
       <c r="G348" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H348" t="inlineStr">
         <is>
@@ -18720,7 +18720,7 @@
         </is>
       </c>
       <c r="G349" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H349" t="inlineStr">
         <is>
@@ -18758,7 +18758,7 @@
         </is>
       </c>
       <c r="G350" t="n">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="H350" t="inlineStr">
         <is>
@@ -18796,7 +18796,7 @@
         </is>
       </c>
       <c r="G351" t="n">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="H351" t="inlineStr">
         <is>
@@ -18834,7 +18834,7 @@
         </is>
       </c>
       <c r="G352" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H352" t="inlineStr">
         <is>
@@ -18872,7 +18872,7 @@
         </is>
       </c>
       <c r="G353" t="n">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="H353" t="inlineStr">
         <is>
@@ -18910,7 +18910,7 @@
         </is>
       </c>
       <c r="G354" t="n">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="H354" t="inlineStr">
         <is>
@@ -18948,7 +18948,7 @@
         </is>
       </c>
       <c r="G355" t="n">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="H355" t="inlineStr">
         <is>
@@ -18986,7 +18986,7 @@
         </is>
       </c>
       <c r="G356" t="n">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H356" t="inlineStr">
         <is>
@@ -19024,7 +19024,7 @@
         </is>
       </c>
       <c r="G357" t="n">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H357" t="inlineStr">
         <is>
@@ -19062,7 +19062,7 @@
         </is>
       </c>
       <c r="G358" t="n">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H358" t="inlineStr">
         <is>
@@ -19100,7 +19100,7 @@
         </is>
       </c>
       <c r="G359" t="n">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H359" t="inlineStr">
         <is>
@@ -19138,7 +19138,7 @@
         </is>
       </c>
       <c r="G360" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="H360" t="inlineStr">
         <is>
@@ -19176,7 +19176,7 @@
         </is>
       </c>
       <c r="G361" t="n">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="H361" t="inlineStr">
         <is>
@@ -19214,7 +19214,7 @@
         </is>
       </c>
       <c r="G362" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H362" t="inlineStr">
         <is>
@@ -19252,7 +19252,7 @@
         </is>
       </c>
       <c r="G363" t="n">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="H363" t="inlineStr">
         <is>
@@ -19290,7 +19290,7 @@
         </is>
       </c>
       <c r="G364" t="n">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H364" t="inlineStr">
         <is>
@@ -19328,7 +19328,7 @@
         </is>
       </c>
       <c r="G365" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="H365" t="inlineStr">
         <is>
@@ -19366,7 +19366,7 @@
         </is>
       </c>
       <c r="G366" t="n">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="H366" t="inlineStr">
         <is>
@@ -19404,7 +19404,7 @@
         </is>
       </c>
       <c r="G367" t="n">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="H367" t="inlineStr">
         <is>
@@ -19442,7 +19442,7 @@
         </is>
       </c>
       <c r="G368" t="n">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="H368" t="inlineStr">
         <is>
@@ -19480,7 +19480,7 @@
         </is>
       </c>
       <c r="G369" t="n">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="H369" t="inlineStr">
         <is>
@@ -19518,7 +19518,7 @@
         </is>
       </c>
       <c r="G370" t="n">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H370" t="inlineStr">
         <is>
@@ -19556,7 +19556,7 @@
         </is>
       </c>
       <c r="G371" t="n">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="H371" t="inlineStr">
         <is>
@@ -19594,7 +19594,7 @@
         </is>
       </c>
       <c r="G372" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H372" t="inlineStr">
         <is>
@@ -19632,7 +19632,7 @@
         </is>
       </c>
       <c r="G373" t="n">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H373" t="inlineStr">
         <is>
@@ -19670,7 +19670,7 @@
         </is>
       </c>
       <c r="G374" t="n">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="H374" t="inlineStr">
         <is>
@@ -19708,7 +19708,7 @@
         </is>
       </c>
       <c r="G375" t="n">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H375" t="inlineStr">
         <is>
@@ -19746,7 +19746,7 @@
         </is>
       </c>
       <c r="G376" t="n">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H376" t="inlineStr">
         <is>
@@ -19784,7 +19784,7 @@
         </is>
       </c>
       <c r="G377" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H377" t="inlineStr">
         <is>
@@ -19822,7 +19822,7 @@
         </is>
       </c>
       <c r="G378" t="n">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="H378" t="inlineStr">
         <is>
@@ -19860,7 +19860,7 @@
         </is>
       </c>
       <c r="G379" t="n">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="H379" t="inlineStr">
         <is>
@@ -19898,7 +19898,7 @@
         </is>
       </c>
       <c r="G380" t="n">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="H380" t="inlineStr">
         <is>
@@ -19936,7 +19936,7 @@
         </is>
       </c>
       <c r="G381" t="n">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="H381" t="inlineStr">
         <is>
@@ -19974,7 +19974,7 @@
         </is>
       </c>
       <c r="G382" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H382" t="inlineStr">
         <is>
@@ -20012,7 +20012,7 @@
         </is>
       </c>
       <c r="G383" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H383" t="inlineStr">
         <is>
@@ -20050,7 +20050,7 @@
         </is>
       </c>
       <c r="G384" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H384" t="inlineStr">
         <is>
@@ -20088,7 +20088,7 @@
         </is>
       </c>
       <c r="G385" t="n">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="H385" t="inlineStr">
         <is>
@@ -20126,7 +20126,7 @@
         </is>
       </c>
       <c r="G386" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H386" t="inlineStr">
         <is>
@@ -20164,7 +20164,7 @@
         </is>
       </c>
       <c r="G387" t="n">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="H387" t="inlineStr">
         <is>
@@ -20202,7 +20202,7 @@
         </is>
       </c>
       <c r="G388" t="n">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="H388" t="inlineStr">
         <is>
@@ -20240,7 +20240,7 @@
         </is>
       </c>
       <c r="G389" t="n">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="H389" t="inlineStr">
         <is>
@@ -20278,7 +20278,7 @@
         </is>
       </c>
       <c r="G390" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H390" t="inlineStr">
         <is>

</xml_diff>